<commit_message>
data: lottery skills decided
lottery skills decided (J30, F22): bad outcomes softened, good ones
raised, Heaven or Hell made worth it
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L462"/>
+  <dimension ref="A1:L473"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26341,6 +26341,622 @@
         </is>
       </c>
     </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Technique 114 Roulette Circus Effect</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>effect 128 (HP recovery of a random enemy)</t>
+        </is>
+      </c>
+      <c r="E463" t="n">
+        <v>1</v>
+      </c>
+      <c r="F463" t="n">
+        <v>1</v>
+      </c>
+      <c r="G463" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>J30, F22</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>Less luck: a bad draw no longer sinks the fight: it healed an enemy fully. The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+        </is>
+      </c>
+      <c r="K463" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L463" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>L002</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Technique 115 Roulette Circus Effect</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>effect 435 (damage = level x value)</t>
+        </is>
+      </c>
+      <c r="E464" t="n">
+        <v>1</v>
+      </c>
+      <c r="F464" t="n">
+        <v>10</v>
+      </c>
+      <c r="G464" t="n">
+        <v>15</v>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>J30, F22</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>A good draw pays for the TP of the skill. The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+        </is>
+      </c>
+      <c r="K464" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L464" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>L003</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Technique 126 Magic Box Effect</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>effect 119 (instant death of the user)</t>
+        </is>
+      </c>
+      <c r="E465" t="n">
+        <v>1</v>
+      </c>
+      <c r="F465" t="n">
+        <v>10</v>
+      </c>
+      <c r="G465" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>J30, F22</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>Less luck: a bad draw no longer sinks the fight: it was certain. The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+        </is>
+      </c>
+      <c r="K465" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L465" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>L004</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Technique 122 Magic Box Effect</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>effect 26 (power of the hit on the user)</t>
+        </is>
+      </c>
+      <c r="E466" t="n">
+        <v>1</v>
+      </c>
+      <c r="F466" t="n">
+        <v>1</v>
+      </c>
+      <c r="G466" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>J30, F22</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>Less luck: a bad draw no longer sinks the fight: a fright instead of a double hit. The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+        </is>
+      </c>
+      <c r="K466" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L466" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>L005</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Technique 118 Magic Box Effect</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>effect 26 (power on all enemies)</t>
+        </is>
+      </c>
+      <c r="E467" t="n">
+        <v>1</v>
+      </c>
+      <c r="F467" t="n">
+        <v>1</v>
+      </c>
+      <c r="G467" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>J30, F22</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>A good draw pays for the TP of the skill. The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+        </is>
+      </c>
+      <c r="K467" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L467" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>L006</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Technique 131 Showtime Effect</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>effect 118 (stun of the whole party)</t>
+        </is>
+      </c>
+      <c r="E468" t="n">
+        <v>1</v>
+      </c>
+      <c r="F468" t="n">
+        <v>10</v>
+      </c>
+      <c r="G468" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>J30, F22</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>Less luck: a bad draw no longer sinks the fight: it was certain. The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+        </is>
+      </c>
+      <c r="K468" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>L007</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Technique 139 Showtime Effect</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>effect 26 (power of the seven hits)</t>
+        </is>
+      </c>
+      <c r="E469" t="n">
+        <v>1</v>
+      </c>
+      <c r="F469" t="n">
+        <v>1</v>
+      </c>
+      <c r="G469" t="n">
+        <v>2</v>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>J30, F22</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>A good draw pays for the TP of the skill and makes up for the rest of the table (the user, 2026-10-09). The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+        </is>
+      </c>
+      <c r="K469" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>L008</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Technique 141 Heaven or Hell Effect</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>effect 138 (damage, share of the target max HP)</t>
+        </is>
+      </c>
+      <c r="E470" t="n">
+        <v>1</v>
+      </c>
+      <c r="F470" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G470" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>J30, F22</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>Heaven or Hell was never worth it (the user, 2026-10-09). The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+        </is>
+      </c>
+      <c r="K470" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>L009</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Technique 141 Heaven or Hell Effect</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>effect 296 (damage cap)</t>
+        </is>
+      </c>
+      <c r="E471" t="n">
+        <v>1</v>
+      </c>
+      <c r="F471" t="n">
+        <v>222</v>
+      </c>
+      <c r="G471" t="n">
+        <v>2220</v>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>J30, F22</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>The cap kept the damage at 222 against bosses of tens of thousands of HP. The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+        </is>
+      </c>
+      <c r="K471" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>L010</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Technique 142 Heaven or Hell Effect</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>effect 132 (heal of the target, share of its max HP)</t>
+        </is>
+      </c>
+      <c r="E472" t="n">
+        <v>1</v>
+      </c>
+      <c r="F472" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G472" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>J30, F22</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>Less luck: a bad draw no longer sinks the fight. The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+        </is>
+      </c>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>L011</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Technique 142 Heaven or Hell Effect</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>effect 295 (heal cap)</t>
+        </is>
+      </c>
+      <c r="E473" t="n">
+        <v>1</v>
+      </c>
+      <c r="F473" t="n">
+        <v>555</v>
+      </c>
+      <c r="G473" t="n">
+        <v>222</v>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>J30, F22</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>Less luck: a bad draw no longer sinks the fight. The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+        </is>
+      </c>
+      <c r="K473" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: trickster, Papillon and Joker decided
trickster, Papillon and Joker decided (F75, F19, F74, J32): Graceful
Rose, Checkmate, Trump Card, Limit Field
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L473"/>
+  <dimension ref="A1:L494"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26957,6 +26957,1182 @@
         </is>
       </c>
     </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Technique 89 Graceful Rose</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E474" t="n">
+        <v>1</v>
+      </c>
+      <c r="F474" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G474" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>F75</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>The single-target fan strike of the Papillon (her only tool against a lone boss was the area attack Rose Queen). The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K474" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Technique 89 Graceful Rose</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E475" t="n">
+        <v>1</v>
+      </c>
+      <c r="F475" t="n">
+        <v>5</v>
+      </c>
+      <c r="G475" t="n">
+        <v>12</v>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>F75</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>The single-target fan strike of the Papillon (her only tool against a lone boss was the area attack Rose Queen). The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K475" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E476" t="n">
+        <v>1</v>
+      </c>
+      <c r="F476" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G476" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>U02 (the Spieler line)</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K476" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E477" t="n">
+        <v>2</v>
+      </c>
+      <c r="F477" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="G477" t="n">
+        <v>0.638</v>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>U02 (the Spieler line)</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K477" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>S005</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E478" t="n">
+        <v>3</v>
+      </c>
+      <c r="F478" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G478" t="n">
+        <v>0.716</v>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>U02 (the Spieler line)</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K478" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>S006</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E479" t="n">
+        <v>4</v>
+      </c>
+      <c r="F479" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G479" t="n">
+        <v>0.794</v>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>U02 (the Spieler line)</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K479" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>S007</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E480" t="n">
+        <v>5</v>
+      </c>
+      <c r="F480" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G480" t="n">
+        <v>0.846</v>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>U02 (the Spieler line)</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K480" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>S008</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E481" t="n">
+        <v>6</v>
+      </c>
+      <c r="F481" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G481" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>U02 (the Spieler line)</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K481" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L481" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>S009</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E482" t="n">
+        <v>7</v>
+      </c>
+      <c r="F482" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G482" t="n">
+        <v>1.054</v>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>U02 (the Spieler line)</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>S010</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E483" t="n">
+        <v>8</v>
+      </c>
+      <c r="F483" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G483" t="n">
+        <v>1.184</v>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>U02 (the Spieler line)</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K483" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>S011</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E484" t="n">
+        <v>9</v>
+      </c>
+      <c r="F484" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G484" t="n">
+        <v>1.314</v>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>U02 (the Spieler line)</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>S012</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E485" t="n">
+        <v>10</v>
+      </c>
+      <c r="F485" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G485" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>U02 (the Spieler line)</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K485" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>S013</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Technique 92 Trump Card</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>effect 48 (ATK gained, DEF x value)</t>
+        </is>
+      </c>
+      <c r="E486" t="n">
+        <v>1</v>
+      </c>
+      <c r="F486" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G486" t="n">
+        <v>1</v>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>Trump Card worth it before its top level; the top is unchanged; the DEF of -10,000 (code) is the Joker's identity. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K486" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>S014</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Technique 92 Trump Card</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>effect 48 (ATK gained, DEF x value)</t>
+        </is>
+      </c>
+      <c r="E487" t="n">
+        <v>2</v>
+      </c>
+      <c r="F487" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G487" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>Trump Card worth it before its top level; the top is unchanged; the DEF of -10,000 (code) is the Joker's identity. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K487" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L487" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>S015</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Technique 92 Trump Card</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>effect 48 (ATK gained, DEF x value)</t>
+        </is>
+      </c>
+      <c r="E488" t="n">
+        <v>3</v>
+      </c>
+      <c r="F488" t="n">
+        <v>1</v>
+      </c>
+      <c r="G488" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>Trump Card worth it before its top level; the top is unchanged; the DEF of -10,000 (code) is the Joker's identity. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K488" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L488" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>S016</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Technique 92 Trump Card</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>effect 48 (ATK gained, DEF x value)</t>
+        </is>
+      </c>
+      <c r="E489" t="n">
+        <v>4</v>
+      </c>
+      <c r="F489" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G489" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>Trump Card worth it before its top level; the top is unchanged; the DEF of -10,000 (code) is the Joker's identity. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K489" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>S017</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Magic 228 Limit Field</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E490" t="n">
+        <v>1</v>
+      </c>
+      <c r="F490" t="n">
+        <v>28</v>
+      </c>
+      <c r="G490" t="n">
+        <v>16</v>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>F74</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>Limit Field lowers damage on both sides (the value cannot make it one-sided): a cheaper niche tool. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K490" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L490" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>S018</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Magic 228 Limit Field</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E491" t="n">
+        <v>2</v>
+      </c>
+      <c r="F491" t="n">
+        <v>31</v>
+      </c>
+      <c r="G491" t="n">
+        <v>18</v>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>F74</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>Limit Field lowers damage on both sides (the value cannot make it one-sided): a cheaper niche tool. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K491" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>S019</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Magic 228 Limit Field</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E492" t="n">
+        <v>3</v>
+      </c>
+      <c r="F492" t="n">
+        <v>34</v>
+      </c>
+      <c r="G492" t="n">
+        <v>19</v>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>F74</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>Limit Field lowers damage on both sides (the value cannot make it one-sided): a cheaper niche tool. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K492" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>S020</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Magic 228 Limit Field</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E493" t="n">
+        <v>4</v>
+      </c>
+      <c r="F493" t="n">
+        <v>37</v>
+      </c>
+      <c r="G493" t="n">
+        <v>21</v>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>F74</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>Limit Field lowers damage on both sides (the value cannot make it one-sided): a cheaper niche tool. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K493" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>S021</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Magic 228 Limit Field</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E494" t="n">
+        <v>5</v>
+      </c>
+      <c r="F494" t="n">
+        <v>40</v>
+      </c>
+      <c r="G494" t="n">
+        <v>22</v>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>F74</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>Limit Field lowers damage on both sides (the value cannot make it one-sided): a cheaper niche tool. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+        </is>
+      </c>
+      <c r="K494" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: T02 decided: guns open to four bow skills
T02 decided: guns open to four bow skills, whips, multi-attack passives,
a small cut to two-handed pieces

Whole boss fights show one hand and a shield winning more late (P24 82%
against 57%): F08 becomes partly true.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L494"/>
+  <dimension ref="A1:L533"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28133,6 +28133,2179 @@
         </is>
       </c>
     </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>W001</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>27 Claymore</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>ATK (base)</t>
+        </is>
+      </c>
+      <c r="F495" t="n">
+        <v>37</v>
+      </c>
+      <c r="G495" t="n">
+        <v>33</v>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>J07, F08</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>A small cut to two-handed pieces (the user, 2026-10-09): base ATK -10%, the upgrade rate kept, so the middle of the game moves (one-handed from 68 - 69% to 71 - 72% of the axe) and the end hardly does, where one hand and a shield already win more boss fights (P24: 82% against 57%)</t>
+        </is>
+      </c>
+      <c r="K495" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>W002</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>131 Heavy Axe</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>ATK (base)</t>
+        </is>
+      </c>
+      <c r="F496" t="n">
+        <v>43</v>
+      </c>
+      <c r="G496" t="n">
+        <v>38</v>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>J07, F08</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>A small cut to two-handed pieces (the user, 2026-10-09): base ATK -10%, the upgrade rate kept, so the middle of the game moves (one-handed from 68 - 69% to 71 - 72% of the axe) and the end hardly does, where one hand and a shield already win more boss fights (P24: 82% against 57%)</t>
+        </is>
+      </c>
+      <c r="K496" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>W003</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>183 Heavy Lance</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>ATK (base)</t>
+        </is>
+      </c>
+      <c r="F497" t="n">
+        <v>39</v>
+      </c>
+      <c r="G497" t="n">
+        <v>35</v>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>J07, F08</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>A small cut to two-handed pieces (the user, 2026-10-09): base ATK -10%, the upgrade rate kept, so the middle of the game moves (one-handed from 68 - 69% to 71 - 72% of the axe) and the end hardly does, where one hand and a shield already win more boss fights (P24: 82% against 57%)</t>
+        </is>
+      </c>
+      <c r="K497" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>W004</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>382 Tachi</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>ATK (base)</t>
+        </is>
+      </c>
+      <c r="F498" t="n">
+        <v>45</v>
+      </c>
+      <c r="G498" t="n">
+        <v>40</v>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>J07, F08</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>A small cut to two-handed pieces (the user, 2026-10-09): base ATK -10%, the upgrade rate kept, so the middle of the game moves (one-handed from 68 - 69% to 71 - 72% of the axe) and the end hardly does, where one hand and a shield already win more boss fights (P24: 82% against 57%)</t>
+        </is>
+      </c>
+      <c r="K498" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>W005</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>434 Whip</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>upgrade rate</t>
+        </is>
+      </c>
+      <c r="F499" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="G499" t="n">
+        <v>2</v>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>Whips: the Mistress from 40% to 82% of the Dark Lord at C34 and from 10% to 30% at P24, with Whip Mastery x2; more makes her pass the Dark Lord in the middle of the game</t>
+        </is>
+      </c>
+      <c r="K499" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>W006</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Passive 249 Whip Mastery</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>effect 243</t>
+        </is>
+      </c>
+      <c r="E500" t="n">
+        <v>1</v>
+      </c>
+      <c r="F500" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G500" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>Whip Mastery multiplies the whip, so it weighs most late, where the whip lagged most</t>
+        </is>
+      </c>
+      <c r="K500" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>W007</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Passive 249 Whip Mastery</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>effect 243</t>
+        </is>
+      </c>
+      <c r="E501" t="n">
+        <v>2</v>
+      </c>
+      <c r="F501" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G501" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>Whip Mastery multiplies the whip, so it weighs most late, where the whip lagged most</t>
+        </is>
+      </c>
+      <c r="K501" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>W008</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Passive 249 Whip Mastery</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>effect 243</t>
+        </is>
+      </c>
+      <c r="E502" t="n">
+        <v>3</v>
+      </c>
+      <c r="F502" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G502" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>Whip Mastery multiplies the whip, so it weighs most late, where the whip lagged most</t>
+        </is>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>W009</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Passive 249 Whip Mastery</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>effect 243</t>
+        </is>
+      </c>
+      <c r="E503" t="n">
+        <v>4</v>
+      </c>
+      <c r="F503" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="G503" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>Whip Mastery multiplies the whip, so it weighs most late, where the whip lagged most</t>
+        </is>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>W010</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Passive 249 Whip Mastery</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>effect 243</t>
+        </is>
+      </c>
+      <c r="E504" t="n">
+        <v>5</v>
+      </c>
+      <c r="F504" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G504" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>Whip Mastery multiplies the whip, so it weighs most late, where the whip lagged most</t>
+        </is>
+      </c>
+      <c r="K504" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>W011</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Passive 249 Whip Mastery</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>effect 243</t>
+        </is>
+      </c>
+      <c r="E505" t="n">
+        <v>6</v>
+      </c>
+      <c r="F505" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G505" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J505" t="inlineStr">
+        <is>
+          <t>Whip Mastery multiplies the whip, so it weighs most late, where the whip lagged most</t>
+        </is>
+      </c>
+      <c r="K505" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>W012</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Passive 249 Whip Mastery</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>effect 243</t>
+        </is>
+      </c>
+      <c r="E506" t="n">
+        <v>7</v>
+      </c>
+      <c r="F506" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G506" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J506" t="inlineStr">
+        <is>
+          <t>Whip Mastery multiplies the whip, so it weighs most late, where the whip lagged most</t>
+        </is>
+      </c>
+      <c r="K506" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>W013</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Passive 249 Whip Mastery</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>effect 243</t>
+        </is>
+      </c>
+      <c r="E507" t="n">
+        <v>8</v>
+      </c>
+      <c r="F507" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G507" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J507" t="inlineStr">
+        <is>
+          <t>Whip Mastery multiplies the whip, so it weighs most late, where the whip lagged most</t>
+        </is>
+      </c>
+      <c r="K507" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>W014</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Passive 249 Whip Mastery</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>effect 243</t>
+        </is>
+      </c>
+      <c r="E508" t="n">
+        <v>9</v>
+      </c>
+      <c r="F508" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G508" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J508" t="inlineStr">
+        <is>
+          <t>Whip Mastery multiplies the whip, so it weighs most late, where the whip lagged most</t>
+        </is>
+      </c>
+      <c r="K508" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L508" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>W015</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Passive 249 Whip Mastery</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>effect 243</t>
+        </is>
+      </c>
+      <c r="E509" t="n">
+        <v>10</v>
+      </c>
+      <c r="F509" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G509" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J509" t="inlineStr">
+        <is>
+          <t>Whip Mastery multiplies the whip, so it weighs most late, where the whip lagged most</t>
+        </is>
+      </c>
+      <c r="K509" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L509" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>W016</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Passive 261 Double Attack</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E510" t="n">
+        <v>1</v>
+      </c>
+      <c r="F510" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="G510" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J510" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K510" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L510" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>W017</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Passive 261 Double Attack</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E511" t="n">
+        <v>2</v>
+      </c>
+      <c r="F511" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G511" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J511" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K511" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L511" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>W018</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Passive 261 Double Attack</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E512" t="n">
+        <v>3</v>
+      </c>
+      <c r="F512" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G512" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J512" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K512" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L512" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>W019</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Passive 261 Double Attack</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E513" t="n">
+        <v>4</v>
+      </c>
+      <c r="F513" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G513" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J513" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K513" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L513" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>W020</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Passive 261 Double Attack</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E514" t="n">
+        <v>5</v>
+      </c>
+      <c r="F514" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G514" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J514" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K514" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L514" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>W021</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Passive 262 Triple Attack</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>effect 252</t>
+        </is>
+      </c>
+      <c r="E515" t="n">
+        <v>1</v>
+      </c>
+      <c r="F515" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G515" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J515" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K515" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L515" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>W022</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Passive 262 Triple Attack</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>effect 252</t>
+        </is>
+      </c>
+      <c r="E516" t="n">
+        <v>2</v>
+      </c>
+      <c r="F516" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G516" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J516" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K516" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L516" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>W023</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Passive 262 Triple Attack</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>effect 252</t>
+        </is>
+      </c>
+      <c r="E517" t="n">
+        <v>3</v>
+      </c>
+      <c r="F517" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="G517" t="n">
+        <v>0.138</v>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J517" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K517" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L517" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>W024</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Passive 262 Triple Attack</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>effect 252</t>
+        </is>
+      </c>
+      <c r="E518" t="n">
+        <v>4</v>
+      </c>
+      <c r="F518" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G518" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J518" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K518" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L518" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>W025</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Passive 262 Triple Attack</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>effect 252</t>
+        </is>
+      </c>
+      <c r="E519" t="n">
+        <v>5</v>
+      </c>
+      <c r="F519" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="G519" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J519" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K519" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L519" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>W026</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Passive 302 Barrage</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E520" t="n">
+        <v>1</v>
+      </c>
+      <c r="F520" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G520" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J520" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K520" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L520" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>W027</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Passive 302 Barrage</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E521" t="n">
+        <v>2</v>
+      </c>
+      <c r="F521" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G521" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J521" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K521" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L521" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>W028</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Passive 302 Barrage</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E522" t="n">
+        <v>3</v>
+      </c>
+      <c r="F522" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G522" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J522" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K522" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L522" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>W029</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Passive 302 Barrage</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E523" t="n">
+        <v>4</v>
+      </c>
+      <c r="F523" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G523" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J523" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K523" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L523" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>W030</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Passive 302 Barrage</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E524" t="n">
+        <v>5</v>
+      </c>
+      <c r="F524" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G524" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J524" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K524" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L524" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>W031</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Passive 302 Barrage</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E525" t="n">
+        <v>6</v>
+      </c>
+      <c r="F525" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G525" t="n">
+        <v>0.312</v>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J525" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K525" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L525" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>W032</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Passive 302 Barrage</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E526" t="n">
+        <v>7</v>
+      </c>
+      <c r="F526" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="G526" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J526" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K526" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L526" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>W033</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Passive 302 Barrage</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E527" t="n">
+        <v>8</v>
+      </c>
+      <c r="F527" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G527" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J527" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K527" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L527" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>W034</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Passive 302 Barrage</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E528" t="n">
+        <v>9</v>
+      </c>
+      <c r="F528" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G528" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H528" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I528" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J528" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K528" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L528" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>W035</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Passive 302 Barrage</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>effect 251</t>
+        </is>
+      </c>
+      <c r="E529" t="n">
+        <v>10</v>
+      </c>
+      <c r="F529" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G529" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H529" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="J529" t="inlineStr">
+        <is>
+          <t>A little more for the characters who hit many times (+25%)</t>
+        </is>
+      </c>
+      <c r="K529" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L529" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>W036</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Technique 43 Spiral Arrow</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>weapon codes</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>8, 15</t>
+        </is>
+      </c>
+      <c r="H530" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I530" t="inlineStr">
+        <is>
+          <t>J06, F10</t>
+        </is>
+      </c>
+      <c r="J530" t="inlineStr">
+        <is>
+          <t>Guns may use four more bow skills (structural: a weapon mask the game already uses for Chain Spike, Guided Shot and Poison Shot)</t>
+        </is>
+      </c>
+      <c r="K530" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L530" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>W037</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Technique 50 Divine Cannon</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>weapon codes</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>8, 15</t>
+        </is>
+      </c>
+      <c r="H531" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>J06, F10</t>
+        </is>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>Guns may use four more bow skills (structural: a weapon mask the game already uses for Chain Spike, Guided Shot and Poison Shot)</t>
+        </is>
+      </c>
+      <c r="K531" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L531" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>W038</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Passive 270 Warning Shot</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>weapon codes</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>8, 15</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>J06, F10</t>
+        </is>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>Guns may use four more bow skills (structural: a weapon mask the game already uses for Chain Spike, Guided Shot and Poison Shot)</t>
+        </is>
+      </c>
+      <c r="K532" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L532" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>W039</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Passive 271 Support Shot</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>weapon codes</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>8, 15</t>
+        </is>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>J06, F10</t>
+        </is>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>Guns may use four more bow skills (structural: a weapon mask the game already uses for Chain Spike, Guided Shot and Poison Shot)</t>
+        </is>
+      </c>
+      <c r="K533" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L533" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: T04 decided: faster chant of top spells, magic defence x1.5
T04 decided: faster chant of top spells, magic defence x1.5; J02 partly
true (superboss wall) sent to T08
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L533"/>
+  <dimension ref="A1:L618"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30306,6 +30306,4766 @@
         </is>
       </c>
     </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>M001</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Magic 146 Crimson Flare</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E534" t="n">
+        <v>1</v>
+      </c>
+      <c r="F534" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G534" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I534" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J534" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K534" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L534" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>M002</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Magic 146 Crimson Flare</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E535" t="n">
+        <v>2</v>
+      </c>
+      <c r="F535" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G535" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I535" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J535" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K535" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L535" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>M003</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Magic 146 Crimson Flare</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E536" t="n">
+        <v>3</v>
+      </c>
+      <c r="F536" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G536" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I536" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J536" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K536" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L536" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>M004</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Magic 146 Crimson Flare</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E537" t="n">
+        <v>4</v>
+      </c>
+      <c r="F537" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G537" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J537" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K537" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L537" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>M005</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Magic 146 Crimson Flare</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E538" t="n">
+        <v>5</v>
+      </c>
+      <c r="F538" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G538" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J538" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K538" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L538" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>M006</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Magic 150 Cocytus</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E539" t="n">
+        <v>1</v>
+      </c>
+      <c r="F539" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G539" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K539" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L539" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>M007</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Magic 150 Cocytus</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E540" t="n">
+        <v>2</v>
+      </c>
+      <c r="F540" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G540" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K540" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L540" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>M008</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Magic 150 Cocytus</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E541" t="n">
+        <v>3</v>
+      </c>
+      <c r="F541" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G541" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K541" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L541" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>M009</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Magic 150 Cocytus</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E542" t="n">
+        <v>4</v>
+      </c>
+      <c r="F542" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G542" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K542" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L542" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>M010</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Magic 150 Cocytus</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E543" t="n">
+        <v>5</v>
+      </c>
+      <c r="F543" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G543" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I543" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J543" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K543" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L543" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>M011</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Magic 154 Muon Plasma</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E544" t="n">
+        <v>1</v>
+      </c>
+      <c r="F544" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G544" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J544" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K544" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L544" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>M012</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Magic 154 Muon Plasma</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E545" t="n">
+        <v>2</v>
+      </c>
+      <c r="F545" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G545" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J545" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K545" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L545" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>M013</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Magic 154 Muon Plasma</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E546" t="n">
+        <v>3</v>
+      </c>
+      <c r="F546" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G546" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I546" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J546" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K546" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L546" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>M014</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Magic 154 Muon Plasma</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E547" t="n">
+        <v>4</v>
+      </c>
+      <c r="F547" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G547" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K547" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L547" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>M015</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Magic 154 Muon Plasma</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E548" t="n">
+        <v>5</v>
+      </c>
+      <c r="F548" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G548" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K548" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L548" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>M016</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Magic 158 Tempest</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E549" t="n">
+        <v>1</v>
+      </c>
+      <c r="F549" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G549" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H549" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K549" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L549" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>M017</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Magic 158 Tempest</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E550" t="n">
+        <v>2</v>
+      </c>
+      <c r="F550" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G550" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K550" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L550" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>M018</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Magic 158 Tempest</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E551" t="n">
+        <v>3</v>
+      </c>
+      <c r="F551" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G551" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H551" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J551" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K551" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L551" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>M019</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Magic 158 Tempest</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E552" t="n">
+        <v>4</v>
+      </c>
+      <c r="F552" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G552" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J552" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K552" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L552" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>M020</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Magic 158 Tempest</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E553" t="n">
+        <v>5</v>
+      </c>
+      <c r="F553" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G553" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J553" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K553" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L553" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>M021</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Magic 162 Gaia Crush</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E554" t="n">
+        <v>1</v>
+      </c>
+      <c r="F554" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G554" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K554" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L554" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>M022</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Magic 162 Gaia Crush</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E555" t="n">
+        <v>2</v>
+      </c>
+      <c r="F555" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G555" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K555" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L555" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>M023</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Magic 162 Gaia Crush</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E556" t="n">
+        <v>3</v>
+      </c>
+      <c r="F556" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G556" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K556" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L556" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>M024</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Magic 162 Gaia Crush</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E557" t="n">
+        <v>4</v>
+      </c>
+      <c r="F557" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G557" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K557" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L557" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>M025</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Magic 162 Gaia Crush</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E558" t="n">
+        <v>5</v>
+      </c>
+      <c r="F558" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G558" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>J33, J14</t>
+        </is>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>The top single spell chants faster (0.85 at every level, it was 0.75 - 0.70): less time exposed to interruption, its power per time closer to its power per TP</t>
+        </is>
+      </c>
+      <c r="K558" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L558" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>M026</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Magic 145 Inferno</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E559" t="n">
+        <v>2</v>
+      </c>
+      <c r="F559" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G559" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K559" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L559" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>M027</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Magic 145 Inferno</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E560" t="n">
+        <v>3</v>
+      </c>
+      <c r="F560" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G560" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K560" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L560" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>M028</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Magic 145 Inferno</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E561" t="n">
+        <v>4</v>
+      </c>
+      <c r="F561" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G561" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K561" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L561" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>M029</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Magic 145 Inferno</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E562" t="n">
+        <v>5</v>
+      </c>
+      <c r="F562" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G562" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K562" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L562" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>M030</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Magic 145 Inferno</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E563" t="n">
+        <v>6</v>
+      </c>
+      <c r="F563" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G563" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K563" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L563" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>M031</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Magic 145 Inferno</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E564" t="n">
+        <v>7</v>
+      </c>
+      <c r="F564" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G564" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K564" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L564" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>M032</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Magic 145 Inferno</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E565" t="n">
+        <v>8</v>
+      </c>
+      <c r="F565" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G565" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K565" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L565" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>M033</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Magic 145 Inferno</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E566" t="n">
+        <v>9</v>
+      </c>
+      <c r="F566" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G566" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K566" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L566" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>M034</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Magic 145 Inferno</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E567" t="n">
+        <v>10</v>
+      </c>
+      <c r="F567" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G567" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K567" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L567" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>M035</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Magic 149 Diamond Dust</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E568" t="n">
+        <v>2</v>
+      </c>
+      <c r="F568" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G568" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K568" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L568" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>M036</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Magic 149 Diamond Dust</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E569" t="n">
+        <v>3</v>
+      </c>
+      <c r="F569" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G569" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K569" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L569" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>M037</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Magic 149 Diamond Dust</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E570" t="n">
+        <v>4</v>
+      </c>
+      <c r="F570" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G570" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J570" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K570" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L570" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>M038</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Magic 149 Diamond Dust</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E571" t="n">
+        <v>5</v>
+      </c>
+      <c r="F571" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G571" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J571" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K571" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L571" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>M039</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Magic 149 Diamond Dust</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E572" t="n">
+        <v>6</v>
+      </c>
+      <c r="F572" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G572" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J572" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K572" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L572" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>M040</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Magic 149 Diamond Dust</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E573" t="n">
+        <v>7</v>
+      </c>
+      <c r="F573" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G573" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K573" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L573" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>M041</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Magic 149 Diamond Dust</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E574" t="n">
+        <v>8</v>
+      </c>
+      <c r="F574" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G574" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J574" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K574" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L574" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>M042</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Magic 149 Diamond Dust</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E575" t="n">
+        <v>9</v>
+      </c>
+      <c r="F575" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G575" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J575" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K575" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L575" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>M043</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Magic 149 Diamond Dust</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E576" t="n">
+        <v>10</v>
+      </c>
+      <c r="F576" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G576" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J576" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K576" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L576" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>M044</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Magic 153 Lightning</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E577" t="n">
+        <v>2</v>
+      </c>
+      <c r="F577" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G577" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J577" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K577" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L577" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>M045</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Magic 153 Lightning</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E578" t="n">
+        <v>3</v>
+      </c>
+      <c r="F578" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G578" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K578" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L578" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>M046</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Magic 153 Lightning</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E579" t="n">
+        <v>4</v>
+      </c>
+      <c r="F579" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G579" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K579" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L579" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>M047</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Magic 153 Lightning</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E580" t="n">
+        <v>5</v>
+      </c>
+      <c r="F580" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G580" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J580" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K580" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L580" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>M048</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Magic 153 Lightning</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E581" t="n">
+        <v>6</v>
+      </c>
+      <c r="F581" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G581" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K581" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L581" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>M049</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Magic 153 Lightning</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E582" t="n">
+        <v>7</v>
+      </c>
+      <c r="F582" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G582" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K582" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L582" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>M050</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Magic 153 Lightning</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E583" t="n">
+        <v>8</v>
+      </c>
+      <c r="F583" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G583" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K583" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L583" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>M051</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Magic 153 Lightning</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E584" t="n">
+        <v>9</v>
+      </c>
+      <c r="F584" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G584" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K584" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L584" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>M052</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Magic 153 Lightning</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E585" t="n">
+        <v>10</v>
+      </c>
+      <c r="F585" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G585" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K585" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L585" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>M053</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Magic 157 Tornado</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E586" t="n">
+        <v>2</v>
+      </c>
+      <c r="F586" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G586" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J586" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K586" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L586" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>M054</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Magic 157 Tornado</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E587" t="n">
+        <v>3</v>
+      </c>
+      <c r="F587" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G587" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K587" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L587" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>M055</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Magic 157 Tornado</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E588" t="n">
+        <v>4</v>
+      </c>
+      <c r="F588" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G588" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K588" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L588" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>M056</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Magic 157 Tornado</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E589" t="n">
+        <v>5</v>
+      </c>
+      <c r="F589" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G589" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K589" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L589" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>M057</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Magic 157 Tornado</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E590" t="n">
+        <v>6</v>
+      </c>
+      <c r="F590" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G590" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K590" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L590" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>M058</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Magic 157 Tornado</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E591" t="n">
+        <v>7</v>
+      </c>
+      <c r="F591" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G591" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K591" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L591" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>M059</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Magic 157 Tornado</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E592" t="n">
+        <v>8</v>
+      </c>
+      <c r="F592" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G592" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J592" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K592" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L592" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>M060</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Magic 157 Tornado</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E593" t="n">
+        <v>9</v>
+      </c>
+      <c r="F593" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G593" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J593" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K593" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L593" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>M061</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Magic 157 Tornado</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E594" t="n">
+        <v>10</v>
+      </c>
+      <c r="F594" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G594" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K594" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L594" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>M062</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Magic 161 Meteor</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E595" t="n">
+        <v>2</v>
+      </c>
+      <c r="F595" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G595" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K595" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L595" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>M063</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Magic 161 Meteor</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E596" t="n">
+        <v>3</v>
+      </c>
+      <c r="F596" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G596" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K596" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L596" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>M064</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Magic 161 Meteor</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E597" t="n">
+        <v>4</v>
+      </c>
+      <c r="F597" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G597" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K597" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L597" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>M065</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Magic 161 Meteor</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E598" t="n">
+        <v>5</v>
+      </c>
+      <c r="F598" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G598" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K598" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L598" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>M066</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Magic 161 Meteor</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E599" t="n">
+        <v>6</v>
+      </c>
+      <c r="F599" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G599" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K599" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L599" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>M067</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Magic 161 Meteor</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E600" t="n">
+        <v>7</v>
+      </c>
+      <c r="F600" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G600" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K600" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L600" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>M068</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Magic 161 Meteor</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E601" t="n">
+        <v>8</v>
+      </c>
+      <c r="F601" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G601" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K601" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L601" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>M069</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Magic 161 Meteor</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E602" t="n">
+        <v>9</v>
+      </c>
+      <c r="F602" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G602" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H602" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K602" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L602" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>M070</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Magic 161 Meteor</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E603" t="n">
+        <v>10</v>
+      </c>
+      <c r="F603" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G603" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H603" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>J33</t>
+        </is>
+      </c>
+      <c r="J603" t="inlineStr">
+        <is>
+          <t>The area spell no longer chants slower as it rises (0.70 at every level, it fell to 0.60)</t>
+        </is>
+      </c>
+      <c r="K603" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L603" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>M071</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Magic 195 Sun Veil</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E604" t="n">
+        <v>1</v>
+      </c>
+      <c r="F604" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G604" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H604" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J604" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K604" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L604" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>M072</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Magic 195 Sun Veil</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E605" t="n">
+        <v>2</v>
+      </c>
+      <c r="F605" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G605" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H605" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K605" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L605" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>M073</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Magic 195 Sun Veil</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E606" t="n">
+        <v>3</v>
+      </c>
+      <c r="F606" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G606" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="H606" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K606" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L606" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>M074</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Magic 195 Sun Veil</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E607" t="n">
+        <v>4</v>
+      </c>
+      <c r="F607" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G607" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="H607" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K607" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L607" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>M075</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Magic 195 Sun Veil</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E608" t="n">
+        <v>5</v>
+      </c>
+      <c r="F608" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G608" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="H608" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K608" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L608" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>M076</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Magic 220 Water Scroll</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E609" t="n">
+        <v>1</v>
+      </c>
+      <c r="F609" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="G609" t="n">
+        <v>-0.105</v>
+      </c>
+      <c r="H609" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K609" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L609" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>M077</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Magic 220 Water Scroll</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E610" t="n">
+        <v>2</v>
+      </c>
+      <c r="F610" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="G610" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="H610" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J610" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K610" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L610" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>M078</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Magic 220 Water Scroll</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E611" t="n">
+        <v>3</v>
+      </c>
+      <c r="F611" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="G611" t="n">
+        <v>-0.195</v>
+      </c>
+      <c r="H611" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J611" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K611" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L611" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>M079</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Magic 220 Water Scroll</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E612" t="n">
+        <v>4</v>
+      </c>
+      <c r="F612" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="G612" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K612" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L612" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>M080</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Magic 220 Water Scroll</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E613" t="n">
+        <v>5</v>
+      </c>
+      <c r="F613" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="G613" t="n">
+        <v>-0.27</v>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K613" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L613" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>M081</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Magic 231 Carrot and Stick</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E614" t="n">
+        <v>1</v>
+      </c>
+      <c r="F614" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="G614" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K614" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L614" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>M082</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Magic 231 Carrot and Stick</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E615" t="n">
+        <v>2</v>
+      </c>
+      <c r="F615" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="G615" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K615" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L615" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>M083</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Magic 231 Carrot and Stick</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E616" t="n">
+        <v>3</v>
+      </c>
+      <c r="F616" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="G616" t="n">
+        <v>-0.195</v>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K616" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L616" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>M084</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Magic 231 Carrot and Stick</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E617" t="n">
+        <v>4</v>
+      </c>
+      <c r="F617" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="G617" t="n">
+        <v>-0.21</v>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K617" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L617" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>M085</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Magic 231 Carrot and Stick</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>effect 163 (magic defence modifier)</t>
+        </is>
+      </c>
+      <c r="E618" t="n">
+        <v>5</v>
+      </c>
+      <c r="F618" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="G618" t="n">
+        <v>-0.225</v>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>Magic defence buffs and debuffs x1.5: +27% at the top of Sun Veil cuts a spell by 12% (it was 8%; INT 300, power 900, RES 300)</t>
+        </is>
+      </c>
+      <c r="K618" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L618" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: spieler moderated (Graceful Rose +80%
spieler moderated (Graceful Rose +80%, Checkmate x1.15) so it does not
become mandatory; the slot wins on par with the other lines
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -26985,7 +26985,7 @@
         <v>0.2</v>
       </c>
       <c r="G474" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="H474" t="inlineStr">
         <is>
@@ -26999,7 +26999,7 @@
       </c>
       <c r="J474" t="inlineStr">
         <is>
-          <t>The single-target fan strike of the Papillon (her only tool against a lone boss was the area attack Rose Queen). The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>The single-target fan strike of the Papillon (her only tool against a lone boss was the area attack Rose Queen). Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K474" t="inlineStr">
@@ -27055,7 +27055,7 @@
       </c>
       <c r="J475" t="inlineStr">
         <is>
-          <t>The single-target fan strike of the Papillon (her only tool against a lone boss was the area attack Rose Queen). The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>The single-target fan strike of the Papillon (her only tool against a lone boss was the area attack Rose Queen). Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K475" t="inlineStr">
@@ -27097,7 +27097,7 @@
         <v>0.2</v>
       </c>
       <c r="G476" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.38</v>
       </c>
       <c r="H476" t="inlineStr">
         <is>
@@ -27111,7 +27111,7 @@
       </c>
       <c r="J476" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K476" t="inlineStr">
@@ -27153,7 +27153,7 @@
         <v>0.26</v>
       </c>
       <c r="G477" t="n">
-        <v>0.638</v>
+        <v>0.449</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
@@ -27167,7 +27167,7 @@
       </c>
       <c r="J477" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K477" t="inlineStr">
@@ -27209,7 +27209,7 @@
         <v>0.32</v>
       </c>
       <c r="G478" t="n">
-        <v>0.716</v>
+        <v>0.518</v>
       </c>
       <c r="H478" t="inlineStr">
         <is>
@@ -27223,7 +27223,7 @@
       </c>
       <c r="J478" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K478" t="inlineStr">
@@ -27265,7 +27265,7 @@
         <v>0.38</v>
       </c>
       <c r="G479" t="n">
-        <v>0.794</v>
+        <v>0.587</v>
       </c>
       <c r="H479" t="inlineStr">
         <is>
@@ -27279,7 +27279,7 @@
       </c>
       <c r="J479" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K479" t="inlineStr">
@@ -27321,7 +27321,7 @@
         <v>0.42</v>
       </c>
       <c r="G480" t="n">
-        <v>0.846</v>
+        <v>0.633</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
@@ -27335,7 +27335,7 @@
       </c>
       <c r="J480" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K480" t="inlineStr">
@@ -27377,7 +27377,7 @@
         <v>0.5</v>
       </c>
       <c r="G481" t="n">
-        <v>0.95</v>
+        <v>0.725</v>
       </c>
       <c r="H481" t="inlineStr">
         <is>
@@ -27391,7 +27391,7 @@
       </c>
       <c r="J481" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K481" t="inlineStr">
@@ -27433,7 +27433,7 @@
         <v>0.58</v>
       </c>
       <c r="G482" t="n">
-        <v>1.054</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
@@ -27447,7 +27447,7 @@
       </c>
       <c r="J482" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K482" t="inlineStr">
@@ -27489,7 +27489,7 @@
         <v>0.68</v>
       </c>
       <c r="G483" t="n">
-        <v>1.184</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
@@ -27503,7 +27503,7 @@
       </c>
       <c r="J483" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K483" t="inlineStr">
@@ -27545,7 +27545,7 @@
         <v>0.78</v>
       </c>
       <c r="G484" t="n">
-        <v>1.314</v>
+        <v>1.047</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
@@ -27559,7 +27559,7 @@
       </c>
       <c r="J484" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K484" t="inlineStr">
@@ -27601,7 +27601,7 @@
         <v>0.9</v>
       </c>
       <c r="G485" t="n">
-        <v>1.47</v>
+        <v>1.185</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
@@ -27615,7 +27615,7 @@
       </c>
       <c r="J485" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. The first Papillon slot goes from 70% to 94% of the Fighter/Scout band (C13 74%, C18 111%, C25 113%, C34 70%, C38 101%; sim/measures.py slot_share, 20 battles)</t>
+          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
         </is>
       </c>
       <c r="K485" t="inlineStr">

</xml_diff>

<commit_message>
data: kunoichi decided (K001 - K025)
kunoichi decided (K001 - K025): Shadow Clone and Ninja Piledriver -25%
TP, Ninja Piledriver x2.5 power; F04, J27, F88 verdicts
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1004"/>
+  <dimension ref="A1:L1029"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56311,6 +56311,1406 @@
         </is>
       </c>
     </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>K001</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Magic 216 Shadow Clone</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1005" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1005" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1005" t="n">
+        <v>17</v>
+      </c>
+      <c r="H1005" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1005" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1005" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1005" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1005" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>K002</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Magic 216 Shadow Clone</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1006" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1006" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1006" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1006" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1006" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1006" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1006" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1006" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>K003</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Magic 216 Shadow Clone</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1007" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1007" t="n">
+        <v>32</v>
+      </c>
+      <c r="G1007" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1007" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1007" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1007" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1007" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1007" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>K004</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>Magic 216 Shadow Clone</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1008" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1008" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1008" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1008" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1008" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1008" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1008" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1008" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>K005</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>Magic 216 Shadow Clone</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1009" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1009" t="n">
+        <v>45</v>
+      </c>
+      <c r="G1009" t="n">
+        <v>33</v>
+      </c>
+      <c r="H1009" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1009" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1009" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1009" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1009" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>K006</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1010" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1010" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1010" t="n">
+        <v>9</v>
+      </c>
+      <c r="H1010" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1010" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1010" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1010" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1010" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>K007</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1011" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1011" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1011" t="n">
+        <v>11</v>
+      </c>
+      <c r="H1011" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1011" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1011" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1011" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1011" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>K008</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1012" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1012" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1012" t="n">
+        <v>13</v>
+      </c>
+      <c r="H1012" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1012" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1012" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1012" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1012" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>K009</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1013" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1013" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1013" t="n">
+        <v>15</v>
+      </c>
+      <c r="H1013" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1013" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1013" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1013" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1013" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>K010</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1014" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1014" t="n">
+        <v>24</v>
+      </c>
+      <c r="G1014" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1014" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1014" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1014" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1014" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1014" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>K011</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1015" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1015" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1015" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1015" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1015" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1015" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1015" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1015" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>K012</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1016" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1016" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1016" t="n">
+        <v>22</v>
+      </c>
+      <c r="H1016" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1016" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1016" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1016" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1016" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>K013</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1017" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1017" t="n">
+        <v>32</v>
+      </c>
+      <c r="G1017" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1017" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1017" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1017" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1017" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1017" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>K014</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1018" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1018" t="n">
+        <v>34</v>
+      </c>
+      <c r="G1018" t="n">
+        <v>25</v>
+      </c>
+      <c r="H1018" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1018" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1018" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1018" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1018" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>K015</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1019" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1019" t="n">
+        <v>36</v>
+      </c>
+      <c r="G1019" t="n">
+        <v>27</v>
+      </c>
+      <c r="H1019" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1019" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1019" t="inlineStr">
+        <is>
+          <t>The Kunoichi wins as often as the Papillon in her slot but takes much longer (C40 40 s against 29, P24 21 s against 13): Shadow Clone and Ninja Piledriver drain her TP and she ends on plain hits. A quarter off both (the cap of the user on TP cuts); the JP guide notes Shadow Clone cost more than in the prequel (atwiki dt2-2 page 142)</t>
+        </is>
+      </c>
+      <c r="K1019" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1019" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>K016</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1020" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1020" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G1020" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H1020" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1020" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1020" t="inlineStr">
+        <is>
+          <t>Her own strike, Ninja Piledriver, x2.5 power at every level: with the TP cut she matches the Papillon in time at C34 and C40 (31 / 28 s against 31 / 29) and is 23% slower at P24 while winning more (100% against 80%); her share of damage (20 - 39%) stays below the Papillon (29 - 44%), so she does not become mandatory. Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1020" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1020" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>K017</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1021" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1021" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="G1021" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H1021" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1021" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1021" t="inlineStr">
+        <is>
+          <t>Her own strike, Ninja Piledriver, x2.5 power at every level: with the TP cut she matches the Papillon in time at C34 and C40 (31 / 28 s against 31 / 29) and is 23% slower at P24 while winning more (100% against 80%); her share of damage (20 - 39%) stays below the Papillon (29 - 44%), so she does not become mandatory. Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1021" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1021" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>K018</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1022" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1022" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G1022" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H1022" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1022" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1022" t="inlineStr">
+        <is>
+          <t>Her own strike, Ninja Piledriver, x2.5 power at every level: with the TP cut she matches the Papillon in time at C34 and C40 (31 / 28 s against 31 / 29) and is 23% slower at P24 while winning more (100% against 80%); her share of damage (20 - 39%) stays below the Papillon (29 - 44%), so she does not become mandatory. Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1022" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1022" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>K019</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1023" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1023" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="G1023" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="H1023" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1023" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1023" t="inlineStr">
+        <is>
+          <t>Her own strike, Ninja Piledriver, x2.5 power at every level: with the TP cut she matches the Papillon in time at C34 and C40 (31 / 28 s against 31 / 29) and is 23% slower at P24 while winning more (100% against 80%); her share of damage (20 - 39%) stays below the Papillon (29 - 44%), so she does not become mandatory. Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1023" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1023" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>K020</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1024" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1024" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="G1024" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="H1024" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1024" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1024" t="inlineStr">
+        <is>
+          <t>Her own strike, Ninja Piledriver, x2.5 power at every level: with the TP cut she matches the Papillon in time at C34 and C40 (31 / 28 s against 31 / 29) and is 23% slower at P24 while winning more (100% against 80%); her share of damage (20 - 39%) stays below the Papillon (29 - 44%), so she does not become mandatory. Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1024" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1024" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>K021</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1025" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1025" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="G1025" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="H1025" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1025" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1025" t="inlineStr">
+        <is>
+          <t>Her own strike, Ninja Piledriver, x2.5 power at every level: with the TP cut she matches the Papillon in time at C34 and C40 (31 / 28 s against 31 / 29) and is 23% slower at P24 while winning more (100% against 80%); her share of damage (20 - 39%) stays below the Papillon (29 - 44%), so she does not become mandatory. Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1025" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1025" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>K022</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1026" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1026" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G1026" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="H1026" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1026" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1026" t="inlineStr">
+        <is>
+          <t>Her own strike, Ninja Piledriver, x2.5 power at every level: with the TP cut she matches the Papillon in time at C34 and C40 (31 / 28 s against 31 / 29) and is 23% slower at P24 while winning more (100% against 80%); her share of damage (20 - 39%) stays below the Papillon (29 - 44%), so she does not become mandatory. Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1026" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1026" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>K023</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1027" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1027" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G1027" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H1027" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1027" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1027" t="inlineStr">
+        <is>
+          <t>Her own strike, Ninja Piledriver, x2.5 power at every level: with the TP cut she matches the Papillon in time at C34 and C40 (31 / 28 s against 31 / 29) and is 23% slower at P24 while winning more (100% against 80%); her share of damage (20 - 39%) stays below the Papillon (29 - 44%), so she does not become mandatory. Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1027" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1027" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>K024</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1028" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1028" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G1028" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1028" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1028" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1028" t="inlineStr">
+        <is>
+          <t>Her own strike, Ninja Piledriver, x2.5 power at every level: with the TP cut she matches the Papillon in time at C34 and C40 (31 / 28 s against 31 / 29) and is 23% slower at P24 while winning more (100% against 80%); her share of damage (20 - 39%) stays below the Papillon (29 - 44%), so she does not become mandatory. Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1028" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1028" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>K025</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>Technique 52 Ninja Piledriver</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1029" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1029" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G1029" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="H1029" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1029" t="inlineStr">
+        <is>
+          <t>F04, J27, F88</t>
+        </is>
+      </c>
+      <c r="J1029" t="inlineStr">
+        <is>
+          <t>Her own strike, Ninja Piledriver, x2.5 power at every level: with the TP cut she matches the Papillon in time at C34 and C40 (31 / 28 s against 31 / 29) and is 23% slower at P24 while winning more (100% against 80%); her share of damage (20 - 39%) stays below the Papillon (29 - 44%), so she does not become mandatory. Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1029" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1029" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: magical Princess decided
magical Princess decided (Q001 - Q015): Magical Change -25% TP, Magical
Spark x1.7 power; F05, J25 verdicts
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1029"/>
+  <dimension ref="A1:L1044"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57711,6 +57711,846 @@
         </is>
       </c>
     </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>Q001</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>Technique 59 Magical Change</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1030" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1030" t="n">
+        <v>52</v>
+      </c>
+      <c r="G1030" t="n">
+        <v>39</v>
+      </c>
+      <c r="H1030" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1030" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1030" t="inlineStr">
+        <is>
+          <t>The Magical Princess wins as often as the Papillon in her slot but her fights last 10 - 34% longer: Magical Change (92 TP at the top level, renewed every few turns) drains her TP. A quarter off (the cap of the user on TP cuts)</t>
+        </is>
+      </c>
+      <c r="K1030" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1030" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>Q002</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>Technique 59 Magical Change</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1031" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1031" t="n">
+        <v>60</v>
+      </c>
+      <c r="G1031" t="n">
+        <v>45</v>
+      </c>
+      <c r="H1031" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1031" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1031" t="inlineStr">
+        <is>
+          <t>The Magical Princess wins as often as the Papillon in her slot but her fights last 10 - 34% longer: Magical Change (92 TP at the top level, renewed every few turns) drains her TP. A quarter off (the cap of the user on TP cuts)</t>
+        </is>
+      </c>
+      <c r="K1031" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1031" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>Q003</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Technique 59 Magical Change</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1032" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1032" t="n">
+        <v>70</v>
+      </c>
+      <c r="G1032" t="n">
+        <v>52</v>
+      </c>
+      <c r="H1032" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1032" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1032" t="inlineStr">
+        <is>
+          <t>The Magical Princess wins as often as the Papillon in her slot but her fights last 10 - 34% longer: Magical Change (92 TP at the top level, renewed every few turns) drains her TP. A quarter off (the cap of the user on TP cuts)</t>
+        </is>
+      </c>
+      <c r="K1032" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1032" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>Q004</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>Technique 59 Magical Change</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1033" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1033" t="n">
+        <v>80</v>
+      </c>
+      <c r="G1033" t="n">
+        <v>60</v>
+      </c>
+      <c r="H1033" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1033" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1033" t="inlineStr">
+        <is>
+          <t>The Magical Princess wins as often as the Papillon in her slot but her fights last 10 - 34% longer: Magical Change (92 TP at the top level, renewed every few turns) drains her TP. A quarter off (the cap of the user on TP cuts)</t>
+        </is>
+      </c>
+      <c r="K1033" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1033" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>Q005</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>Technique 59 Magical Change</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1034" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1034" t="n">
+        <v>92</v>
+      </c>
+      <c r="G1034" t="n">
+        <v>69</v>
+      </c>
+      <c r="H1034" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1034" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1034" t="inlineStr">
+        <is>
+          <t>The Magical Princess wins as often as the Papillon in her slot but her fights last 10 - 34% longer: Magical Change (92 TP at the top level, renewed every few turns) drains her TP. A quarter off (the cap of the user on TP cuts)</t>
+        </is>
+      </c>
+      <c r="K1034" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1034" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>Q006</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>Technique 60 Magical Spark</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1035" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1035" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G1035" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="H1035" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1035" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1035" t="inlineStr">
+        <is>
+          <t>Magical Spark, her main strike, x1.7 power at every level: with the TP cut she is within 6 - 15% of the time of the Papillon (C34, C40, P24) with the same share of damage (27 / 44 / 38% against 29 / 44 / 42%), so she does not become mandatory. Magical Change stays her transformation (atwiki dt2-2 page 137). Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1035" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1035" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>Q007</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>Technique 60 Magical Spark</t>
+        </is>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1036" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1036" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G1036" t="n">
+        <v>0.714</v>
+      </c>
+      <c r="H1036" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1036" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1036" t="inlineStr">
+        <is>
+          <t>Magical Spark, her main strike, x1.7 power at every level: with the TP cut she is within 6 - 15% of the time of the Papillon (C34, C40, P24) with the same share of damage (27 / 44 / 38% against 29 / 44 / 42%), so she does not become mandatory. Magical Change stays her transformation (atwiki dt2-2 page 137). Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1036" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1036" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>Q008</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>Technique 60 Magical Spark</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1037" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1037" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="G1037" t="n">
+        <v>0.8159999999999999</v>
+      </c>
+      <c r="H1037" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1037" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1037" t="inlineStr">
+        <is>
+          <t>Magical Spark, her main strike, x1.7 power at every level: with the TP cut she is within 6 - 15% of the time of the Papillon (C34, C40, P24) with the same share of damage (27 / 44 / 38% against 29 / 44 / 42%), so she does not become mandatory. Magical Change stays her transformation (atwiki dt2-2 page 137). Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1037" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1037" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>Q009</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>Technique 60 Magical Spark</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1038" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1038" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G1038" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="H1038" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1038" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1038" t="inlineStr">
+        <is>
+          <t>Magical Spark, her main strike, x1.7 power at every level: with the TP cut she is within 6 - 15% of the time of the Papillon (C34, C40, P24) with the same share of damage (27 / 44 / 38% against 29 / 44 / 42%), so she does not become mandatory. Magical Change stays her transformation (atwiki dt2-2 page 137). Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1038" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1038" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>Q010</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>Technique 60 Magical Spark</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1039" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1039" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G1039" t="n">
+        <v>1.054</v>
+      </c>
+      <c r="H1039" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1039" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1039" t="inlineStr">
+        <is>
+          <t>Magical Spark, her main strike, x1.7 power at every level: with the TP cut she is within 6 - 15% of the time of the Papillon (C34, C40, P24) with the same share of damage (27 / 44 / 38% against 29 / 44 / 42%), so she does not become mandatory. Magical Change stays her transformation (atwiki dt2-2 page 137). Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1039" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1039" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>Q011</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>Technique 60 Magical Spark</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1040" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1040" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G1040" t="n">
+        <v>1.224</v>
+      </c>
+      <c r="H1040" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1040" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1040" t="inlineStr">
+        <is>
+          <t>Magical Spark, her main strike, x1.7 power at every level: with the TP cut she is within 6 - 15% of the time of the Papillon (C34, C40, P24) with the same share of damage (27 / 44 / 38% against 29 / 44 / 42%), so she does not become mandatory. Magical Change stays her transformation (atwiki dt2-2 page 137). Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1040" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1040" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>Q012</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>Technique 60 Magical Spark</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1041" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1041" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G1041" t="n">
+        <v>1.394</v>
+      </c>
+      <c r="H1041" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1041" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1041" t="inlineStr">
+        <is>
+          <t>Magical Spark, her main strike, x1.7 power at every level: with the TP cut she is within 6 - 15% of the time of the Papillon (C34, C40, P24) with the same share of damage (27 / 44 / 38% against 29 / 44 / 42%), so she does not become mandatory. Magical Change stays her transformation (atwiki dt2-2 page 137). Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1041" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1041" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>Q013</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>Technique 60 Magical Spark</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1042" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1042" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G1042" t="n">
+        <v>1.581</v>
+      </c>
+      <c r="H1042" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1042" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1042" t="inlineStr">
+        <is>
+          <t>Magical Spark, her main strike, x1.7 power at every level: with the TP cut she is within 6 - 15% of the time of the Papillon (C34, C40, P24) with the same share of damage (27 / 44 / 38% against 29 / 44 / 42%), so she does not become mandatory. Magical Change stays her transformation (atwiki dt2-2 page 137). Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1042" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1042" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>Q014</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>Technique 60 Magical Spark</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1043" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1043" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G1043" t="n">
+        <v>1.768</v>
+      </c>
+      <c r="H1043" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1043" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1043" t="inlineStr">
+        <is>
+          <t>Magical Spark, her main strike, x1.7 power at every level: with the TP cut she is within 6 - 15% of the time of the Papillon (C34, C40, P24) with the same share of damage (27 / 44 / 38% against 29 / 44 / 42%), so she does not become mandatory. Magical Change stays her transformation (atwiki dt2-2 page 137). Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1043" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1043" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>Q015</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>Technique 60 Magical Spark</t>
+        </is>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1044" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1044" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="G1044" t="n">
+        <v>1.972</v>
+      </c>
+      <c r="H1044" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1044" t="inlineStr">
+        <is>
+          <t>F05, J25</t>
+        </is>
+      </c>
+      <c r="J1044" t="inlineStr">
+        <is>
+          <t>Magical Spark, her main strike, x1.7 power at every level: with the TP cut she is within 6 - 15% of the time of the Papillon (C34, C40, P24) with the same share of damage (27 / 44 / 38% against 29 / 44 / 42%), so she does not become mandatory. Magical Change stays her transformation (atwiki dt2-2 page 137). Measured: measures.slot_share, 15 battles, on the variant</t>
+        </is>
+      </c>
+      <c r="K1044" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1044" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: T05 by stage: Assassin stings x2.5 decided
T05 by stage: Assassin stings x2.5 decided; Trickster, Treasure Hunter,
Mistress and Sage proposals ; weapon by class in Roles (Kunoichi, Joker)

69 of 76 role and stage rows within the band with every proposal (66
before)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1044"/>
+  <dimension ref="A1:L1119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58551,6 +58551,4206 @@
         </is>
       </c>
     </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>T001</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>Technique 38 Sleep Sting</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1045" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1045" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G1045" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H1045" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1045" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1045" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1045" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1045" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>T002</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>Technique 38 Sleep Sting</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1046" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1046" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G1046" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H1046" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1046" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1046" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1046" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1046" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>T003</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>Technique 38 Sleep Sting</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1047" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1047" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G1047" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H1047" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1047" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1047" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1047" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1047" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>T004</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>Technique 38 Sleep Sting</t>
+        </is>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1048" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1048" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G1048" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H1048" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1048" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1048" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1048" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1048" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>T005</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>Technique 38 Sleep Sting</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1049" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1049" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G1049" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H1049" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1049" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1049" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1049" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1049" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>T006</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>Technique 38 Sleep Sting</t>
+        </is>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1050" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1050" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G1050" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H1050" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1050" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1050" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1050" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1050" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>T007</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>Technique 38 Sleep Sting</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1051" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1051" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G1051" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1051" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1051" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1051" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1051" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1051" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>T008</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>Technique 38 Sleep Sting</t>
+        </is>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1052" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1052" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G1052" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H1052" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1052" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1052" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1052" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1052" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>T009</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>Technique 38 Sleep Sting</t>
+        </is>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1053" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1053" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G1053" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H1053" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1053" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1053" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1053" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1053" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>T010</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>Technique 38 Sleep Sting</t>
+        </is>
+      </c>
+      <c r="D1054" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1054" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1054" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G1054" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H1054" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1054" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1054" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1054" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1054" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>T011</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>Technique 40 Stun Sting</t>
+        </is>
+      </c>
+      <c r="D1055" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1055" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1055" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G1055" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H1055" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1055" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1055" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1055" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1055" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>T012</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Technique 40 Stun Sting</t>
+        </is>
+      </c>
+      <c r="D1056" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1056" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1056" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G1056" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H1056" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1056" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1056" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1056" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1056" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>T013</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>Technique 40 Stun Sting</t>
+        </is>
+      </c>
+      <c r="D1057" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1057" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1057" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G1057" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H1057" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1057" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1057" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1057" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1057" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>T014</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>Technique 40 Stun Sting</t>
+        </is>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1058" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1058" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G1058" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H1058" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1058" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1058" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1058" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1058" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>T015</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>Technique 40 Stun Sting</t>
+        </is>
+      </c>
+      <c r="D1059" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1059" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1059" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G1059" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H1059" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1059" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1059" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1059" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1059" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>T016</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>Technique 40 Stun Sting</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1060" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1060" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G1060" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H1060" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1060" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1060" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1060" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1060" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>T017</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>Technique 40 Stun Sting</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1061" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1061" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G1061" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H1061" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1061" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1061" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1061" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1061" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>T018</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>Technique 40 Stun Sting</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1062" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1062" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G1062" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1062" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1062" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1062" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1062" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1062" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>T019</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>Technique 40 Stun Sting</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1063" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1063" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G1063" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H1063" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1063" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1063" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1063" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1063" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>T020</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>Technique 40 Stun Sting</t>
+        </is>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1064" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1064" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G1064" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H1064" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1064" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1064" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1064" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1064" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>T021</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>Technique 39 Silence Sting</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1065" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1065" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G1065" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H1065" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1065" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1065" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1065" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1065" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>T022</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>Technique 39 Silence Sting</t>
+        </is>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1066" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1066" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G1066" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H1066" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1066" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1066" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1066" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1066" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>T023</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>Technique 39 Silence Sting</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1067" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1067" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G1067" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H1067" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1067" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1067" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1067" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1067" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>T024</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Technique 39 Silence Sting</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1068" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1068" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G1068" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H1068" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1068" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1068" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1068" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1068" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>T025</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>Technique 39 Silence Sting</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1069" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1069" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G1069" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H1069" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1069" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1069" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1069" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1069" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>T026</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>Technique 39 Silence Sting</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1070" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1070" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G1070" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H1070" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1070" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1070" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1070" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1070" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>T027</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>Technique 39 Silence Sting</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1071" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1071" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G1071" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1071" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1071" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1071" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1071" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1071" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>T028</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>Technique 39 Silence Sting</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1072" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1072" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G1072" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H1072" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1072" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1072" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1072" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1072" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>T029</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>Technique 39 Silence Sting</t>
+        </is>
+      </c>
+      <c r="D1073" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1073" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1073" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G1073" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H1073" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1073" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1073" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1073" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1073" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>T030</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>Technique 39 Silence Sting</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1074" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1074" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G1074" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H1074" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1074" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1074" t="inlineStr">
+        <is>
+          <t>The stings, the own strikes of the Assassin, x2.5 power at every level: their power (0.12 - 0.56) was about half of the strikes of the other intermediate classes (Frost Slash 0.30 - 1.28, Gust Thrust 0.35 - 1.45). Measured at C10, C13, C18 (tools/class_stages.py, the Kunoichi build): fights 26% longer than the median attacker, 12% after; still below the other strikes at the top levels, the ailment chance kept</t>
+        </is>
+      </c>
+      <c r="K1074" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1074" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>T031</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1075" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1075" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="G1075" t="n">
+        <v>0.608</v>
+      </c>
+      <c r="H1075" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1075" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="J1075" t="inlineStr">
+        <is>
+          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+        </is>
+      </c>
+      <c r="K1075" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1075" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>T032</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1076" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1076" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="G1076" t="n">
+        <v>0.718</v>
+      </c>
+      <c r="H1076" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1076" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="J1076" t="inlineStr">
+        <is>
+          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+        </is>
+      </c>
+      <c r="K1076" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1076" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>T033</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1077" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1077" t="n">
+        <v>0.518</v>
+      </c>
+      <c r="G1077" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="H1077" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1077" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="J1077" t="inlineStr">
+        <is>
+          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+        </is>
+      </c>
+      <c r="K1077" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1077" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>T034</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D1078" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1078" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1078" t="n">
+        <v>0.587</v>
+      </c>
+      <c r="G1078" t="n">
+        <v>0.9389999999999999</v>
+      </c>
+      <c r="H1078" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1078" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="J1078" t="inlineStr">
+        <is>
+          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+        </is>
+      </c>
+      <c r="K1078" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1078" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>T035</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D1079" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1079" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1079" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="G1079" t="n">
+        <v>1.013</v>
+      </c>
+      <c r="H1079" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1079" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="J1079" t="inlineStr">
+        <is>
+          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+        </is>
+      </c>
+      <c r="K1079" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1079" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>T036</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D1080" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1080" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1080" t="n">
+        <v>0.725</v>
+      </c>
+      <c r="G1080" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="H1080" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1080" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="J1080" t="inlineStr">
+        <is>
+          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+        </is>
+      </c>
+      <c r="K1080" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1080" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>T037</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1081" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1081" t="n">
+        <v>0.8169999999999999</v>
+      </c>
+      <c r="G1081" t="n">
+        <v>1.307</v>
+      </c>
+      <c r="H1081" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1081" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="J1081" t="inlineStr">
+        <is>
+          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+        </is>
+      </c>
+      <c r="K1081" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1081" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>T038</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1082" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1082" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="G1082" t="n">
+        <v>1.491</v>
+      </c>
+      <c r="H1082" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1082" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="J1082" t="inlineStr">
+        <is>
+          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+        </is>
+      </c>
+      <c r="K1082" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1082" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>T039</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1083" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1083" t="n">
+        <v>1.047</v>
+      </c>
+      <c r="G1083" t="n">
+        <v>1.675</v>
+      </c>
+      <c r="H1083" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1083" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="J1083" t="inlineStr">
+        <is>
+          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+        </is>
+      </c>
+      <c r="K1083" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1083" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>T040</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Technique 82 Checkmate</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1084" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1084" t="n">
+        <v>1.185</v>
+      </c>
+      <c r="G1084" t="n">
+        <v>1.896</v>
+      </c>
+      <c r="H1084" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1084" t="inlineStr">
+        <is>
+          <t>F17</t>
+        </is>
+      </c>
+      <c r="J1084" t="inlineStr">
+        <is>
+          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+        </is>
+      </c>
+      <c r="K1084" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1084" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>T041</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>Technique 32 Pursuit Stab</t>
+        </is>
+      </c>
+      <c r="D1085" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1085" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1085" t="n">
+        <v>24</v>
+      </c>
+      <c r="G1085" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1085" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1085" t="inlineStr">
+        <is>
+          <t>J26</t>
+        </is>
+      </c>
+      <c r="J1085" t="inlineStr">
+        <is>
+          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+        </is>
+      </c>
+      <c r="K1085" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1085" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>T042</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Technique 32 Pursuit Stab</t>
+        </is>
+      </c>
+      <c r="D1086" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1086" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1086" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1086" t="n">
+        <v>21</v>
+      </c>
+      <c r="H1086" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1086" t="inlineStr">
+        <is>
+          <t>J26</t>
+        </is>
+      </c>
+      <c r="J1086" t="inlineStr">
+        <is>
+          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+        </is>
+      </c>
+      <c r="K1086" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1086" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>T043</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>Technique 32 Pursuit Stab</t>
+        </is>
+      </c>
+      <c r="D1087" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1087" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1087" t="n">
+        <v>32</v>
+      </c>
+      <c r="G1087" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1087" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1087" t="inlineStr">
+        <is>
+          <t>J26</t>
+        </is>
+      </c>
+      <c r="J1087" t="inlineStr">
+        <is>
+          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+        </is>
+      </c>
+      <c r="K1087" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1087" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>T044</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>Technique 32 Pursuit Stab</t>
+        </is>
+      </c>
+      <c r="D1088" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1088" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1088" t="n">
+        <v>35</v>
+      </c>
+      <c r="G1088" t="n">
+        <v>26</v>
+      </c>
+      <c r="H1088" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1088" t="inlineStr">
+        <is>
+          <t>J26</t>
+        </is>
+      </c>
+      <c r="J1088" t="inlineStr">
+        <is>
+          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+        </is>
+      </c>
+      <c r="K1088" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1088" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>T045</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>Technique 32 Pursuit Stab</t>
+        </is>
+      </c>
+      <c r="D1089" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1089" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1089" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1089" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1089" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1089" t="inlineStr">
+        <is>
+          <t>J26</t>
+        </is>
+      </c>
+      <c r="J1089" t="inlineStr">
+        <is>
+          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+        </is>
+      </c>
+      <c r="K1089" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1089" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>T046</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>Technique 32 Pursuit Stab</t>
+        </is>
+      </c>
+      <c r="D1090" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1090" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1090" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G1090" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H1090" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1090" t="inlineStr">
+        <is>
+          <t>J26</t>
+        </is>
+      </c>
+      <c r="J1090" t="inlineStr">
+        <is>
+          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+        </is>
+      </c>
+      <c r="K1090" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1090" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>T047</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>Technique 32 Pursuit Stab</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1091" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1091" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G1091" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="H1091" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1091" t="inlineStr">
+        <is>
+          <t>J26</t>
+        </is>
+      </c>
+      <c r="J1091" t="inlineStr">
+        <is>
+          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+        </is>
+      </c>
+      <c r="K1091" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1091" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>T048</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Technique 32 Pursuit Stab</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1092" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1092" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G1092" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="H1092" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1092" t="inlineStr">
+        <is>
+          <t>J26</t>
+        </is>
+      </c>
+      <c r="J1092" t="inlineStr">
+        <is>
+          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+        </is>
+      </c>
+      <c r="K1092" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1092" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>T049</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Technique 32 Pursuit Stab</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1093" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1093" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G1093" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="H1093" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1093" t="inlineStr">
+        <is>
+          <t>J26</t>
+        </is>
+      </c>
+      <c r="J1093" t="inlineStr">
+        <is>
+          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+        </is>
+      </c>
+      <c r="K1093" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1093" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>T050</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Technique 32 Pursuit Stab</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1094" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1094" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="G1094" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="H1094" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1094" t="inlineStr">
+        <is>
+          <t>J26</t>
+        </is>
+      </c>
+      <c r="J1094" t="inlineStr">
+        <is>
+          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+        </is>
+      </c>
+      <c r="K1094" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1094" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>T051</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Technique 77 Enticing Love</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1095" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1095" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1095" t="n">
+        <v>22</v>
+      </c>
+      <c r="H1095" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1095" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1095" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1095" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1095" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>T052</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Technique 77 Enticing Love</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1096" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1096" t="n">
+        <v>34</v>
+      </c>
+      <c r="G1096" t="n">
+        <v>25</v>
+      </c>
+      <c r="H1096" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1096" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1096" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1096" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1096" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>T053</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Technique 77 Enticing Love</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1097" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1097" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1097" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1097" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1097" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1097" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1097" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1097" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>T054</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Technique 77 Enticing Love</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1098" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1098" t="n">
+        <v>42</v>
+      </c>
+      <c r="G1098" t="n">
+        <v>31</v>
+      </c>
+      <c r="H1098" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1098" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1098" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1098" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1098" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>T055</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Technique 77 Enticing Love</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1099" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1099" t="n">
+        <v>46</v>
+      </c>
+      <c r="G1099" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1099" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1099" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1099" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1099" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1099" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>T056</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Technique 76 Hard Whipping</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1100" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1100" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G1100" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H1100" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1100" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1100" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1100" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1100" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>T057</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>Technique 76 Hard Whipping</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1101" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1101" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G1101" t="n">
+        <v>0.384</v>
+      </c>
+      <c r="H1101" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1101" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1101" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1101" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1101" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>T058</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Technique 76 Hard Whipping</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1102" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1102" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G1102" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="H1102" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1102" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1102" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1102" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1102" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>T059</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>Technique 76 Hard Whipping</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1103" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1103" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G1103" t="n">
+        <v>0.512</v>
+      </c>
+      <c r="H1103" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1103" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1103" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1103" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1103" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>T060</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>Technique 76 Hard Whipping</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1104" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1104" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G1104" t="n">
+        <v>0.576</v>
+      </c>
+      <c r="H1104" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1104" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1104" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1104" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1104" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>T061</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>Technique 76 Hard Whipping</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1105" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1105" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G1105" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="H1105" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1105" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1105" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1105" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1105" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>T062</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>Technique 76 Hard Whipping</t>
+        </is>
+      </c>
+      <c r="D1106" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1106" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1106" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G1106" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="H1106" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1106" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1106" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1106" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1106" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>T063</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>Technique 76 Hard Whipping</t>
+        </is>
+      </c>
+      <c r="D1107" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1107" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1107" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G1107" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H1107" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1107" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1107" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1107" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1107" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>T064</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>Technique 76 Hard Whipping</t>
+        </is>
+      </c>
+      <c r="D1108" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1108" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1108" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G1108" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H1108" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1108" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1108" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1108" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1108" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>T065</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>Technique 76 Hard Whipping</t>
+        </is>
+      </c>
+      <c r="D1109" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1109" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1109" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G1109" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="H1109" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1109" t="inlineStr">
+        <is>
+          <t>F03, J29, F88</t>
+        </is>
+      </c>
+      <c r="J1109" t="inlineStr">
+        <is>
+          <t>Mistress (advanced): fights 16 - 18% longer than the median attacker at C22, C29, C34, C40 (her TP spent on Enticing Love). Enticing Love -25% TP and Hard Whipping, her single whip strike, x1.6 power: 1.07 after. Hard Whipping alone leaves 1.16. At the late checkpoints she is already within the band (1.01)</t>
+        </is>
+      </c>
+      <c r="K1109" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1109" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>T066</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>Magic 226 Circle Brave</t>
+        </is>
+      </c>
+      <c r="D1110" t="inlineStr">
+        <is>
+          <t>effect 161 (party ATK)</t>
+        </is>
+      </c>
+      <c r="E1110" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1110" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G1110" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="H1110" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1110" t="inlineStr">
+        <is>
+          <t>J23</t>
+        </is>
+      </c>
+      <c r="J1110" t="inlineStr">
+        <is>
+          <t>Sage (advanced): the weakest support in the same place of the party (wins in the contested fights C29, C40: 30 / 62% against 55 - 92% for the Bishop and the Etoile). Her party buffs Circle Brave and Circle Protect x1.6 (0.08 - 0.16 to 0.13 - 0.26, the range of the single-target Brave and Protect of the Valkyrie line): C40 62 to 85%, fights 1.39 to 1.27 of the median. Prism Dawn x1.6 changes nothing (she seldom attacks). C29 is the heal wall of Calliope, which needs damage, not buffs</t>
+        </is>
+      </c>
+      <c r="K1110" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1110" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>T067</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>Magic 226 Circle Brave</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr">
+        <is>
+          <t>effect 161 (party ATK)</t>
+        </is>
+      </c>
+      <c r="E1111" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1111" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G1111" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H1111" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1111" t="inlineStr">
+        <is>
+          <t>J23</t>
+        </is>
+      </c>
+      <c r="J1111" t="inlineStr">
+        <is>
+          <t>Sage (advanced): the weakest support in the same place of the party (wins in the contested fights C29, C40: 30 / 62% against 55 - 92% for the Bishop and the Etoile). Her party buffs Circle Brave and Circle Protect x1.6 (0.08 - 0.16 to 0.13 - 0.26, the range of the single-target Brave and Protect of the Valkyrie line): C40 62 to 85%, fights 1.39 to 1.27 of the median. Prism Dawn x1.6 changes nothing (she seldom attacks). C29 is the heal wall of Calliope, which needs damage, not buffs</t>
+        </is>
+      </c>
+      <c r="K1111" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1111" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>T068</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>Magic 226 Circle Brave</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>effect 161 (party ATK)</t>
+        </is>
+      </c>
+      <c r="E1112" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1112" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G1112" t="n">
+        <v>0.192</v>
+      </c>
+      <c r="H1112" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1112" t="inlineStr">
+        <is>
+          <t>J23</t>
+        </is>
+      </c>
+      <c r="J1112" t="inlineStr">
+        <is>
+          <t>Sage (advanced): the weakest support in the same place of the party (wins in the contested fights C29, C40: 30 / 62% against 55 - 92% for the Bishop and the Etoile). Her party buffs Circle Brave and Circle Protect x1.6 (0.08 - 0.16 to 0.13 - 0.26, the range of the single-target Brave and Protect of the Valkyrie line): C40 62 to 85%, fights 1.39 to 1.27 of the median. Prism Dawn x1.6 changes nothing (she seldom attacks). C29 is the heal wall of Calliope, which needs damage, not buffs</t>
+        </is>
+      </c>
+      <c r="K1112" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1112" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>T069</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Magic 226 Circle Brave</t>
+        </is>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>effect 161 (party ATK)</t>
+        </is>
+      </c>
+      <c r="E1113" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1113" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G1113" t="n">
+        <v>0.224</v>
+      </c>
+      <c r="H1113" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1113" t="inlineStr">
+        <is>
+          <t>J23</t>
+        </is>
+      </c>
+      <c r="J1113" t="inlineStr">
+        <is>
+          <t>Sage (advanced): the weakest support in the same place of the party (wins in the contested fights C29, C40: 30 / 62% against 55 - 92% for the Bishop and the Etoile). Her party buffs Circle Brave and Circle Protect x1.6 (0.08 - 0.16 to 0.13 - 0.26, the range of the single-target Brave and Protect of the Valkyrie line): C40 62 to 85%, fights 1.39 to 1.27 of the median. Prism Dawn x1.6 changes nothing (she seldom attacks). C29 is the heal wall of Calliope, which needs damage, not buffs</t>
+        </is>
+      </c>
+      <c r="K1113" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1113" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>T070</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>Magic 226 Circle Brave</t>
+        </is>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>effect 161 (party ATK)</t>
+        </is>
+      </c>
+      <c r="E1114" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1114" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G1114" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="H1114" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1114" t="inlineStr">
+        <is>
+          <t>J23</t>
+        </is>
+      </c>
+      <c r="J1114" t="inlineStr">
+        <is>
+          <t>Sage (advanced): the weakest support in the same place of the party (wins in the contested fights C29, C40: 30 / 62% against 55 - 92% for the Bishop and the Etoile). Her party buffs Circle Brave and Circle Protect x1.6 (0.08 - 0.16 to 0.13 - 0.26, the range of the single-target Brave and Protect of the Valkyrie line): C40 62 to 85%, fights 1.39 to 1.27 of the median. Prism Dawn x1.6 changes nothing (she seldom attacks). C29 is the heal wall of Calliope, which needs damage, not buffs</t>
+        </is>
+      </c>
+      <c r="K1114" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1114" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>T071</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>Magic 227 Circle Protect</t>
+        </is>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>effect 162 (party DEF)</t>
+        </is>
+      </c>
+      <c r="E1115" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1115" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G1115" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="H1115" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1115" t="inlineStr">
+        <is>
+          <t>J23</t>
+        </is>
+      </c>
+      <c r="J1115" t="inlineStr">
+        <is>
+          <t>Sage (advanced): the weakest support in the same place of the party (wins in the contested fights C29, C40: 30 / 62% against 55 - 92% for the Bishop and the Etoile). Her party buffs Circle Brave and Circle Protect x1.6 (0.08 - 0.16 to 0.13 - 0.26, the range of the single-target Brave and Protect of the Valkyrie line): C40 62 to 85%, fights 1.39 to 1.27 of the median. Prism Dawn x1.6 changes nothing (she seldom attacks). C29 is the heal wall of Calliope, which needs damage, not buffs</t>
+        </is>
+      </c>
+      <c r="K1115" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1115" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>T072</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Magic 227 Circle Protect</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>effect 162 (party DEF)</t>
+        </is>
+      </c>
+      <c r="E1116" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1116" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G1116" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H1116" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1116" t="inlineStr">
+        <is>
+          <t>J23</t>
+        </is>
+      </c>
+      <c r="J1116" t="inlineStr">
+        <is>
+          <t>Sage (advanced): the weakest support in the same place of the party (wins in the contested fights C29, C40: 30 / 62% against 55 - 92% for the Bishop and the Etoile). Her party buffs Circle Brave and Circle Protect x1.6 (0.08 - 0.16 to 0.13 - 0.26, the range of the single-target Brave and Protect of the Valkyrie line): C40 62 to 85%, fights 1.39 to 1.27 of the median. Prism Dawn x1.6 changes nothing (she seldom attacks). C29 is the heal wall of Calliope, which needs damage, not buffs</t>
+        </is>
+      </c>
+      <c r="K1116" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1116" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>T073</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Magic 227 Circle Protect</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>effect 162 (party DEF)</t>
+        </is>
+      </c>
+      <c r="E1117" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1117" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G1117" t="n">
+        <v>0.192</v>
+      </c>
+      <c r="H1117" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1117" t="inlineStr">
+        <is>
+          <t>J23</t>
+        </is>
+      </c>
+      <c r="J1117" t="inlineStr">
+        <is>
+          <t>Sage (advanced): the weakest support in the same place of the party (wins in the contested fights C29, C40: 30 / 62% against 55 - 92% for the Bishop and the Etoile). Her party buffs Circle Brave and Circle Protect x1.6 (0.08 - 0.16 to 0.13 - 0.26, the range of the single-target Brave and Protect of the Valkyrie line): C40 62 to 85%, fights 1.39 to 1.27 of the median. Prism Dawn x1.6 changes nothing (she seldom attacks). C29 is the heal wall of Calliope, which needs damage, not buffs</t>
+        </is>
+      </c>
+      <c r="K1117" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1117" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>T074</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Magic 227 Circle Protect</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>effect 162 (party DEF)</t>
+        </is>
+      </c>
+      <c r="E1118" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1118" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G1118" t="n">
+        <v>0.224</v>
+      </c>
+      <c r="H1118" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1118" t="inlineStr">
+        <is>
+          <t>J23</t>
+        </is>
+      </c>
+      <c r="J1118" t="inlineStr">
+        <is>
+          <t>Sage (advanced): the weakest support in the same place of the party (wins in the contested fights C29, C40: 30 / 62% against 55 - 92% for the Bishop and the Etoile). Her party buffs Circle Brave and Circle Protect x1.6 (0.08 - 0.16 to 0.13 - 0.26, the range of the single-target Brave and Protect of the Valkyrie line): C40 62 to 85%, fights 1.39 to 1.27 of the median. Prism Dawn x1.6 changes nothing (she seldom attacks). C29 is the heal wall of Calliope, which needs damage, not buffs</t>
+        </is>
+      </c>
+      <c r="K1118" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1118" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>T075</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>Magic 227 Circle Protect</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>effect 162 (party DEF)</t>
+        </is>
+      </c>
+      <c r="E1119" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1119" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G1119" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="H1119" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1119" t="inlineStr">
+        <is>
+          <t>J23</t>
+        </is>
+      </c>
+      <c r="J1119" t="inlineStr">
+        <is>
+          <t>Sage (advanced): the weakest support in the same place of the party (wins in the contested fights C29, C40: 30 / 62% against 55 - 92% for the Bishop and the Etoile). Her party buffs Circle Brave and Circle Protect x1.6 (0.08 - 0.16 to 0.13 - 0.26, the range of the single-target Brave and Protect of the Valkyrie line): C40 62 to 85%, fights 1.39 to 1.27 of the median. Prism Dawn x1.6 changes nothing (she seldom attacks). C29 is the heal wall of Calliope, which needs damage, not buffs</t>
+        </is>
+      </c>
+      <c r="K1119" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1119" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: T05 proposals accepted
T05 proposals accepted (Trickster, Treasure Hunter, Mistress, Sage);
verdicts F17, J30, J26, F03, J29, F88, J23
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -60283,7 +60283,7 @@
       </c>
       <c r="L1075" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60339,7 +60339,7 @@
       </c>
       <c r="L1076" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60395,7 +60395,7 @@
       </c>
       <c r="L1077" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60451,7 +60451,7 @@
       </c>
       <c r="L1078" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60507,7 +60507,7 @@
       </c>
       <c r="L1079" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60563,7 +60563,7 @@
       </c>
       <c r="L1080" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60619,7 +60619,7 @@
       </c>
       <c r="L1081" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60675,7 +60675,7 @@
       </c>
       <c r="L1082" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60731,7 +60731,7 @@
       </c>
       <c r="L1083" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60787,7 +60787,7 @@
       </c>
       <c r="L1084" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60843,7 +60843,7 @@
       </c>
       <c r="L1085" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60899,7 +60899,7 @@
       </c>
       <c r="L1086" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -60955,7 +60955,7 @@
       </c>
       <c r="L1087" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61011,7 +61011,7 @@
       </c>
       <c r="L1088" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61067,7 +61067,7 @@
       </c>
       <c r="L1089" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61123,7 +61123,7 @@
       </c>
       <c r="L1090" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61179,7 +61179,7 @@
       </c>
       <c r="L1091" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61235,7 +61235,7 @@
       </c>
       <c r="L1092" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61291,7 +61291,7 @@
       </c>
       <c r="L1093" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61347,7 +61347,7 @@
       </c>
       <c r="L1094" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61403,7 +61403,7 @@
       </c>
       <c r="L1095" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61459,7 +61459,7 @@
       </c>
       <c r="L1096" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61515,7 +61515,7 @@
       </c>
       <c r="L1097" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61571,7 +61571,7 @@
       </c>
       <c r="L1098" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61627,7 +61627,7 @@
       </c>
       <c r="L1099" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61683,7 +61683,7 @@
       </c>
       <c r="L1100" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61739,7 +61739,7 @@
       </c>
       <c r="L1101" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61795,7 +61795,7 @@
       </c>
       <c r="L1102" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61851,7 +61851,7 @@
       </c>
       <c r="L1103" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61907,7 +61907,7 @@
       </c>
       <c r="L1104" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -61963,7 +61963,7 @@
       </c>
       <c r="L1105" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62019,7 +62019,7 @@
       </c>
       <c r="L1106" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62075,7 +62075,7 @@
       </c>
       <c r="L1107" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62131,7 +62131,7 @@
       </c>
       <c r="L1108" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62187,7 +62187,7 @@
       </c>
       <c r="L1109" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62243,7 +62243,7 @@
       </c>
       <c r="L1110" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62299,7 +62299,7 @@
       </c>
       <c r="L1111" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62355,7 +62355,7 @@
       </c>
       <c r="L1112" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62411,7 +62411,7 @@
       </c>
       <c r="L1113" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62467,7 +62467,7 @@
       </c>
       <c r="L1114" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62523,7 +62523,7 @@
       </c>
       <c r="L1115" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62579,7 +62579,7 @@
       </c>
       <c r="L1116" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62635,7 +62635,7 @@
       </c>
       <c r="L1117" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62691,7 +62691,7 @@
       </c>
       <c r="L1118" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -62747,7 +62747,7 @@
       </c>
       <c r="L1119" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: T06 skills: tools/skill_worth.py
T06 skills: tools/skill_worth.py (attacking skills against the best of
their class) and skill_value.py (with and without); X001 - X060 decided
(scrolls, drains, Soul Absorb, Life Bringer), X061 - X088 proposed
(Brave, Protect, Illusion, Shadow Clone chant, Shadow Sew, Blood Rage);
verdicts of 63 T06 rows
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1119"/>
+  <dimension ref="A1:L1207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62751,6 +62751,4934 @@
         </is>
       </c>
     </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>X001</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>Magic 219 Fire Scroll</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1120" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1120" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G1120" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H1120" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1120" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1120" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1120" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1120" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>X002</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Magic 219 Fire Scroll</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1121" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1121" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G1121" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="H1121" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1121" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1121" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1121" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1121" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>X003</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Magic 219 Fire Scroll</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1122" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1122" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G1122" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H1122" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1122" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1122" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1122" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1122" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>X004</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Magic 219 Fire Scroll</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1123" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1123" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G1123" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="H1123" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1123" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1123" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1123" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1123" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>X005</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Magic 219 Fire Scroll</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1124" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1124" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G1124" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H1124" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1124" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1124" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1124" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1124" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>X006</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>Magic 220 Water Scroll</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1125" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1125" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G1125" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H1125" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1125" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1125" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1125" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1125" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>X007</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>Magic 220 Water Scroll</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1126" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1126" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G1126" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="H1126" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1126" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1126" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1126" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1126" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>X008</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>Magic 220 Water Scroll</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1127" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1127" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G1127" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H1127" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1127" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1127" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1127" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1127" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>X009</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Magic 220 Water Scroll</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1128" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1128" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G1128" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="H1128" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1128" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1128" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1128" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1128" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>X010</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>Magic 220 Water Scroll</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1129" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1129" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G1129" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H1129" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1129" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1129" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1129" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1129" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>X011</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Magic 222 Wind Scroll</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1130" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1130" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G1130" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H1130" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1130" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1130" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1130" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1130" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>X012</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Magic 222 Wind Scroll</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1131" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1131" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G1131" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="H1131" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1131" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1131" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1131" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1131" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>X013</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Magic 222 Wind Scroll</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1132" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1132" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G1132" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H1132" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1132" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1132" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1132" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1132" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>X014</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>Magic 222 Wind Scroll</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1133" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1133" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G1133" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="H1133" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1133" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1133" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1133" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1133" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>X015</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>Magic 222 Wind Scroll</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1134" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1134" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G1134" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H1134" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1134" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1134" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1134" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1134" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>X016</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Magic 223 Earth Scroll</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1135" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1135" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G1135" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H1135" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1135" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1135" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1135" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1135" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>X017</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>Magic 223 Earth Scroll</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1136" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1136" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G1136" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="H1136" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1136" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1136" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1136" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1136" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>X018</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>Magic 223 Earth Scroll</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1137" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1137" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G1137" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H1137" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1137" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1137" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1137" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1137" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>X019</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Magic 223 Earth Scroll</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1138" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1138" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G1138" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="H1138" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1138" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1138" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1138" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1138" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>X020</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Magic 223 Earth Scroll</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1139" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1139" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G1139" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H1139" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1139" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1139" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1139" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1139" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>X021</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>Magic 221 Lightning Scroll</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1140" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1140" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G1140" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H1140" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1140" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1140" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1140" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1140" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>X022</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Magic 221 Lightning Scroll</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1141" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1141" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G1141" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="H1141" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1141" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1141" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1141" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1141" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>X023</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Magic 221 Lightning Scroll</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1142" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1142" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G1142" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H1142" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1142" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1142" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1142" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1142" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>X024</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Magic 221 Lightning Scroll</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1143" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1143" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G1143" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="H1143" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1143" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1143" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1143" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1143" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>X025</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Magic 221 Lightning Scroll</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>effect 138</t>
+        </is>
+      </c>
+      <c r="E1144" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1144" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G1144" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H1144" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1144" t="inlineStr">
+        <is>
+          <t>F62, J27</t>
+        </is>
+      </c>
+      <c r="J1144" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): the scrolls dealt 44 - 51% of Ninja Piledriver; their share of the target max HP x1.5 brings them to 66 - 77% (x2 made Fire Scroll pass Ninja Piledriver; the cap x2 changed nothing). Their debuff, the reason to cast them, is kept</t>
+        </is>
+      </c>
+      <c r="K1144" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1144" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>X026</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Magic 164 Soul Absorb</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>effect 1</t>
+        </is>
+      </c>
+      <c r="E1145" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1145" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1145" t="n">
+        <v>55</v>
+      </c>
+      <c r="H1145" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1145" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1145" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of Blood Absorb, the other drain of the Witch; magic power x2.5 brings it to 68%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1145" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1145" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>X027</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Magic 164 Soul Absorb</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>effect 1</t>
+        </is>
+      </c>
+      <c r="E1146" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1146" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1146" t="n">
+        <v>75</v>
+      </c>
+      <c r="H1146" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1146" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1146" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of Blood Absorb, the other drain of the Witch; magic power x2.5 brings it to 68%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1146" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1146" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>X028</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Magic 164 Soul Absorb</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>effect 1</t>
+        </is>
+      </c>
+      <c r="E1147" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1147" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1147" t="n">
+        <v>95</v>
+      </c>
+      <c r="H1147" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1147" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1147" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of Blood Absorb, the other drain of the Witch; magic power x2.5 brings it to 68%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1147" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1147" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>X029</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Magic 164 Soul Absorb</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>effect 1</t>
+        </is>
+      </c>
+      <c r="E1148" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1148" t="n">
+        <v>46</v>
+      </c>
+      <c r="G1148" t="n">
+        <v>115</v>
+      </c>
+      <c r="H1148" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1148" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1148" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of Blood Absorb, the other drain of the Witch; magic power x2.5 brings it to 68%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1148" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1148" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>X030</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>Magic 164 Soul Absorb</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>effect 1</t>
+        </is>
+      </c>
+      <c r="E1149" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1149" t="n">
+        <v>54</v>
+      </c>
+      <c r="G1149" t="n">
+        <v>135</v>
+      </c>
+      <c r="H1149" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1149" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1149" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of Blood Absorb, the other drain of the Witch; magic power x2.5 brings it to 68%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1149" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1149" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>X031</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>Magic 164 Soul Absorb</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>effect 1</t>
+        </is>
+      </c>
+      <c r="E1150" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1150" t="n">
+        <v>60</v>
+      </c>
+      <c r="G1150" t="n">
+        <v>150</v>
+      </c>
+      <c r="H1150" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1150" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1150" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of Blood Absorb, the other drain of the Witch; magic power x2.5 brings it to 68%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1150" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1150" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>X032</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>Magic 164 Soul Absorb</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>effect 1</t>
+        </is>
+      </c>
+      <c r="E1151" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1151" t="n">
+        <v>66</v>
+      </c>
+      <c r="G1151" t="n">
+        <v>165</v>
+      </c>
+      <c r="H1151" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1151" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1151" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of Blood Absorb, the other drain of the Witch; magic power x2.5 brings it to 68%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1151" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1151" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>X033</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>Magic 164 Soul Absorb</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>effect 1</t>
+        </is>
+      </c>
+      <c r="E1152" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1152" t="n">
+        <v>72</v>
+      </c>
+      <c r="G1152" t="n">
+        <v>180</v>
+      </c>
+      <c r="H1152" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1152" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1152" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of Blood Absorb, the other drain of the Witch; magic power x2.5 brings it to 68%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1152" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1152" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>X034</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>Magic 164 Soul Absorb</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>effect 1</t>
+        </is>
+      </c>
+      <c r="E1153" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1153" t="n">
+        <v>78</v>
+      </c>
+      <c r="G1153" t="n">
+        <v>195</v>
+      </c>
+      <c r="H1153" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1153" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1153" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of Blood Absorb, the other drain of the Witch; magic power x2.5 brings it to 68%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1153" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1153" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>X035</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>Magic 164 Soul Absorb</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>effect 1</t>
+        </is>
+      </c>
+      <c r="E1154" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1154" t="n">
+        <v>82</v>
+      </c>
+      <c r="G1154" t="n">
+        <v>205</v>
+      </c>
+      <c r="H1154" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1154" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1154" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of Blood Absorb, the other drain of the Witch; magic power x2.5 brings it to 68%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1154" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1154" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>X036</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>Technique 14 Blood Drain</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1155" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1155" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="G1155" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="H1155" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1155" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="J1155" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56% of the best strike of the Dark Lord; +0.6 power at every level (it was -0.26 to +0.10) brings it to 69%, the HP drain kept</t>
+        </is>
+      </c>
+      <c r="K1155" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1155" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>X037</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>Technique 14 Blood Drain</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1156" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1156" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="G1156" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="H1156" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1156" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="J1156" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56% of the best strike of the Dark Lord; +0.6 power at every level (it was -0.26 to +0.10) brings it to 69%, the HP drain kept</t>
+        </is>
+      </c>
+      <c r="K1156" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1156" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>X038</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>Technique 14 Blood Drain</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1157" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1157" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="G1157" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="H1157" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1157" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="J1157" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56% of the best strike of the Dark Lord; +0.6 power at every level (it was -0.26 to +0.10) brings it to 69%, the HP drain kept</t>
+        </is>
+      </c>
+      <c r="K1157" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1157" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>X039</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>Technique 14 Blood Drain</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1158" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1158" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="G1158" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="H1158" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1158" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="J1158" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56% of the best strike of the Dark Lord; +0.6 power at every level (it was -0.26 to +0.10) brings it to 69%, the HP drain kept</t>
+        </is>
+      </c>
+      <c r="K1158" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1158" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>X040</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>Technique 14 Blood Drain</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1159" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1159" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="G1159" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H1159" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1159" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="J1159" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56% of the best strike of the Dark Lord; +0.6 power at every level (it was -0.26 to +0.10) brings it to 69%, the HP drain kept</t>
+        </is>
+      </c>
+      <c r="K1159" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1159" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>X041</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Technique 14 Blood Drain</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1160" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1160" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="G1160" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="H1160" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1160" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="J1160" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56% of the best strike of the Dark Lord; +0.6 power at every level (it was -0.26 to +0.10) brings it to 69%, the HP drain kept</t>
+        </is>
+      </c>
+      <c r="K1160" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1160" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>X042</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>Technique 14 Blood Drain</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1161" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1161" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="G1161" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="H1161" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1161" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="J1161" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56% of the best strike of the Dark Lord; +0.6 power at every level (it was -0.26 to +0.10) brings it to 69%, the HP drain kept</t>
+        </is>
+      </c>
+      <c r="K1161" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1161" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>X043</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>Technique 14 Blood Drain</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1162" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1162" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G1162" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="H1162" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1162" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="J1162" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56% of the best strike of the Dark Lord; +0.6 power at every level (it was -0.26 to +0.10) brings it to 69%, the HP drain kept</t>
+        </is>
+      </c>
+      <c r="K1162" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1162" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>X044</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>Technique 14 Blood Drain</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1163" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1163" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G1163" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="H1163" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1163" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="J1163" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56% of the best strike of the Dark Lord; +0.6 power at every level (it was -0.26 to +0.10) brings it to 69%, the HP drain kept</t>
+        </is>
+      </c>
+      <c r="K1163" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1163" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>X045</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Technique 14 Blood Drain</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1164" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1164" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G1164" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H1164" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1164" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="J1164" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56% of the best strike of the Dark Lord; +0.6 power at every level (it was -0.26 to +0.10) brings it to 69%, the HP drain kept</t>
+        </is>
+      </c>
+      <c r="K1164" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1164" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>X046</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>Technique 15 Soul Drain</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1165" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1165" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="G1165" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H1165" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1165" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1165" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56%; +0.6 power at every level (it was -0.35 to 0) brings it to 65%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1165" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1165" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>X047</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>Technique 15 Soul Drain</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1166" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1166" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="G1166" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H1166" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1166" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1166" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56%; +0.6 power at every level (it was -0.35 to 0) brings it to 65%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1166" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1166" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>X048</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>Technique 15 Soul Drain</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1167" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1167" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="G1167" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H1167" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1167" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1167" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56%; +0.6 power at every level (it was -0.35 to 0) brings it to 65%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1167" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1167" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>X049</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>Technique 15 Soul Drain</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1168" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1168" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G1168" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H1168" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1168" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1168" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56%; +0.6 power at every level (it was -0.35 to 0) brings it to 65%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1168" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1168" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>X050</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>Technique 15 Soul Drain</t>
+        </is>
+      </c>
+      <c r="D1169" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1169" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1169" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="G1169" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="H1169" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1169" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1169" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56%; +0.6 power at every level (it was -0.35 to 0) brings it to 65%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1169" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1169" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>X051</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>Technique 15 Soul Drain</t>
+        </is>
+      </c>
+      <c r="D1170" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1170" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1170" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="G1170" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="H1170" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1170" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1170" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56%; +0.6 power at every level (it was -0.35 to 0) brings it to 65%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1170" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1170" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>X052</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>Technique 15 Soul Drain</t>
+        </is>
+      </c>
+      <c r="D1171" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1171" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1171" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="G1171" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="H1171" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1171" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1171" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56%; +0.6 power at every level (it was -0.35 to 0) brings it to 65%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1171" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1171" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>X053</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>Technique 15 Soul Drain</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1172" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1172" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="G1172" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="H1172" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1172" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1172" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56%; +0.6 power at every level (it was -0.35 to 0) brings it to 65%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1172" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1172" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>X054</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>Technique 15 Soul Drain</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1173" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1173" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="G1173" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="H1173" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1173" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1173" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56%; +0.6 power at every level (it was -0.35 to 0) brings it to 65%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1173" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1173" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>X055</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>Technique 15 Soul Drain</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1174" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1174" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1174" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H1174" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1174" t="inlineStr">
+        <is>
+          <t>F32</t>
+        </is>
+      </c>
+      <c r="J1174" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 56%; +0.6 power at every level (it was -0.35 to 0) brings it to 65%, the TP drain kept</t>
+        </is>
+      </c>
+      <c r="K1174" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1174" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>X056</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>Technique 91 Life Bringer</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1175" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1175" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="G1175" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="H1175" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1175" t="inlineStr">
+        <is>
+          <t>F72, F33</t>
+        </is>
+      </c>
+      <c r="J1175" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of the best strike of the Joker; +0.7 power at every level (it was -0.12 to +0.10) brings it to 76%, the max HP cut kept</t>
+        </is>
+      </c>
+      <c r="K1175" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1175" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>X057</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>Technique 91 Life Bringer</t>
+        </is>
+      </c>
+      <c r="D1176" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1176" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1176" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="G1176" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="H1176" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1176" t="inlineStr">
+        <is>
+          <t>F72, F33</t>
+        </is>
+      </c>
+      <c r="J1176" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of the best strike of the Joker; +0.7 power at every level (it was -0.12 to +0.10) brings it to 76%, the max HP cut kept</t>
+        </is>
+      </c>
+      <c r="K1176" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1176" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>X058</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>Technique 91 Life Bringer</t>
+        </is>
+      </c>
+      <c r="D1177" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1177" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1177" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="G1177" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="H1177" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1177" t="inlineStr">
+        <is>
+          <t>F72, F33</t>
+        </is>
+      </c>
+      <c r="J1177" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of the best strike of the Joker; +0.7 power at every level (it was -0.12 to +0.10) brings it to 76%, the max HP cut kept</t>
+        </is>
+      </c>
+      <c r="K1177" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1177" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>X059</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>Technique 91 Life Bringer</t>
+        </is>
+      </c>
+      <c r="D1178" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1178" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1178" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G1178" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="H1178" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1178" t="inlineStr">
+        <is>
+          <t>F72, F33</t>
+        </is>
+      </c>
+      <c r="J1178" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of the best strike of the Joker; +0.7 power at every level (it was -0.12 to +0.10) brings it to 76%, the max HP cut kept</t>
+        </is>
+      </c>
+      <c r="K1178" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1178" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>X060</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>Technique 91 Life Bringer</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr">
+        <is>
+          <t>effect 26</t>
+        </is>
+      </c>
+      <c r="E1179" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1179" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G1179" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H1179" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1179" t="inlineStr">
+        <is>
+          <t>F72, F33</t>
+        </is>
+      </c>
+      <c r="J1179" t="inlineStr">
+        <is>
+          <t>T06, tools/skill_worth.py (each attacking skill against the best option of the same member, top level, boss and random battles of the stages): 41% of the best strike of the Joker; +0.7 power at every level (it was -0.12 to +0.10) brings it to 76%, the max HP cut kept</t>
+        </is>
+      </c>
+      <c r="K1179" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1179" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>X061</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>Magic 193 Brave</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr">
+        <is>
+          <t>effect 161 (ATK)</t>
+        </is>
+      </c>
+      <c r="E1180" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1180" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G1180" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H1180" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1180" t="inlineStr">
+        <is>
+          <t>F35</t>
+        </is>
+      </c>
+      <c r="J1180" t="inlineStr">
+        <is>
+          <t>A single-target buff weaker than the party ones it does not stack with (War Cry 0.18, Circle Brave 0.256 on the whole party): x2 (0.20 - 0.44) makes it the buff of the main attacker, as the guide uses it (Brave on Yae)</t>
+        </is>
+      </c>
+      <c r="K1180" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1180" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>X062</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>Magic 193 Brave</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr">
+        <is>
+          <t>effect 161 (ATK)</t>
+        </is>
+      </c>
+      <c r="E1181" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1181" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="G1181" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="H1181" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1181" t="inlineStr">
+        <is>
+          <t>F35</t>
+        </is>
+      </c>
+      <c r="J1181" t="inlineStr">
+        <is>
+          <t>A single-target buff weaker than the party ones it does not stack with (War Cry 0.18, Circle Brave 0.256 on the whole party): x2 (0.20 - 0.44) makes it the buff of the main attacker, as the guide uses it (Brave on Yae)</t>
+        </is>
+      </c>
+      <c r="K1181" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1181" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>X063</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>Magic 193 Brave</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr">
+        <is>
+          <t>effect 161 (ATK)</t>
+        </is>
+      </c>
+      <c r="E1182" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1182" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G1182" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H1182" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1182" t="inlineStr">
+        <is>
+          <t>F35</t>
+        </is>
+      </c>
+      <c r="J1182" t="inlineStr">
+        <is>
+          <t>A single-target buff weaker than the party ones it does not stack with (War Cry 0.18, Circle Brave 0.256 on the whole party): x2 (0.20 - 0.44) makes it the buff of the main attacker, as the guide uses it (Brave on Yae)</t>
+        </is>
+      </c>
+      <c r="K1182" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1182" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>X064</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>Magic 193 Brave</t>
+        </is>
+      </c>
+      <c r="D1183" t="inlineStr">
+        <is>
+          <t>effect 161 (ATK)</t>
+        </is>
+      </c>
+      <c r="E1183" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1183" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="G1183" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="H1183" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1183" t="inlineStr">
+        <is>
+          <t>F35</t>
+        </is>
+      </c>
+      <c r="J1183" t="inlineStr">
+        <is>
+          <t>A single-target buff weaker than the party ones it does not stack with (War Cry 0.18, Circle Brave 0.256 on the whole party): x2 (0.20 - 0.44) makes it the buff of the main attacker, as the guide uses it (Brave on Yae)</t>
+        </is>
+      </c>
+      <c r="K1183" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1183" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>X065</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>Magic 193 Brave</t>
+        </is>
+      </c>
+      <c r="D1184" t="inlineStr">
+        <is>
+          <t>effect 161 (ATK)</t>
+        </is>
+      </c>
+      <c r="E1184" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1184" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G1184" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="H1184" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1184" t="inlineStr">
+        <is>
+          <t>F35</t>
+        </is>
+      </c>
+      <c r="J1184" t="inlineStr">
+        <is>
+          <t>A single-target buff weaker than the party ones it does not stack with (War Cry 0.18, Circle Brave 0.256 on the whole party): x2 (0.20 - 0.44) makes it the buff of the main attacker, as the guide uses it (Brave on Yae)</t>
+        </is>
+      </c>
+      <c r="K1184" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1184" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>X066</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>Magic 194 Protect</t>
+        </is>
+      </c>
+      <c r="D1185" t="inlineStr">
+        <is>
+          <t>effect 162 (DEF)</t>
+        </is>
+      </c>
+      <c r="E1185" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1185" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G1185" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H1185" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1185" t="inlineStr">
+        <is>
+          <t>F35</t>
+        </is>
+      </c>
+      <c r="J1185" t="inlineStr">
+        <is>
+          <t>The same for the single-target Protect beside Circle Protect (0.256 on the party): x2 (0.20 - 0.50), the buff of the tank</t>
+        </is>
+      </c>
+      <c r="K1185" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1185" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>X067</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>Magic 194 Protect</t>
+        </is>
+      </c>
+      <c r="D1186" t="inlineStr">
+        <is>
+          <t>effect 162 (DEF)</t>
+        </is>
+      </c>
+      <c r="E1186" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1186" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G1186" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="H1186" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1186" t="inlineStr">
+        <is>
+          <t>F35</t>
+        </is>
+      </c>
+      <c r="J1186" t="inlineStr">
+        <is>
+          <t>The same for the single-target Protect beside Circle Protect (0.256 on the party): x2 (0.20 - 0.50), the buff of the tank</t>
+        </is>
+      </c>
+      <c r="K1186" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1186" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>X068</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>Magic 194 Protect</t>
+        </is>
+      </c>
+      <c r="D1187" t="inlineStr">
+        <is>
+          <t>effect 162 (DEF)</t>
+        </is>
+      </c>
+      <c r="E1187" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1187" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G1187" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="H1187" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1187" t="inlineStr">
+        <is>
+          <t>F35</t>
+        </is>
+      </c>
+      <c r="J1187" t="inlineStr">
+        <is>
+          <t>The same for the single-target Protect beside Circle Protect (0.256 on the party): x2 (0.20 - 0.50), the buff of the tank</t>
+        </is>
+      </c>
+      <c r="K1187" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1187" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>X069</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>Magic 194 Protect</t>
+        </is>
+      </c>
+      <c r="D1188" t="inlineStr">
+        <is>
+          <t>effect 162 (DEF)</t>
+        </is>
+      </c>
+      <c r="E1188" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1188" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G1188" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="H1188" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1188" t="inlineStr">
+        <is>
+          <t>F35</t>
+        </is>
+      </c>
+      <c r="J1188" t="inlineStr">
+        <is>
+          <t>The same for the single-target Protect beside Circle Protect (0.256 on the party): x2 (0.20 - 0.50), the buff of the tank</t>
+        </is>
+      </c>
+      <c r="K1188" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1188" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>X070</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>Magic 194 Protect</t>
+        </is>
+      </c>
+      <c r="D1189" t="inlineStr">
+        <is>
+          <t>effect 162 (DEF)</t>
+        </is>
+      </c>
+      <c r="E1189" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1189" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G1189" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H1189" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1189" t="inlineStr">
+        <is>
+          <t>F35</t>
+        </is>
+      </c>
+      <c r="J1189" t="inlineStr">
+        <is>
+          <t>The same for the single-target Protect beside Circle Protect (0.256 on the party): x2 (0.20 - 0.50), the buff of the tank</t>
+        </is>
+      </c>
+      <c r="K1189" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1189" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>X071</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>Magic 200 Illusion</t>
+        </is>
+      </c>
+      <c r="D1190" t="inlineStr">
+        <is>
+          <t>effect 102 (hits nullified)</t>
+        </is>
+      </c>
+      <c r="E1190" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1190" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1190" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1190" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1190" t="inlineStr">
+        <is>
+          <t>F44</t>
+        </is>
+      </c>
+      <c r="J1190" t="inlineStr">
+        <is>
+          <t>Two hits nullified for 30 - 46 TP against five for Shadow Clone (17 - 33 TP): 3, 4, 5 by level</t>
+        </is>
+      </c>
+      <c r="K1190" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1190" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>X072</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>Magic 200 Illusion</t>
+        </is>
+      </c>
+      <c r="D1191" t="inlineStr">
+        <is>
+          <t>effect 102 (hits nullified)</t>
+        </is>
+      </c>
+      <c r="E1191" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1191" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1191" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1191" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1191" t="inlineStr">
+        <is>
+          <t>F44</t>
+        </is>
+      </c>
+      <c r="J1191" t="inlineStr">
+        <is>
+          <t>Two hits nullified for 30 - 46 TP against five for Shadow Clone (17 - 33 TP): 3, 4, 5 by level</t>
+        </is>
+      </c>
+      <c r="K1191" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1191" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>X073</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>Magic 200 Illusion</t>
+        </is>
+      </c>
+      <c r="D1192" t="inlineStr">
+        <is>
+          <t>effect 102 (hits nullified)</t>
+        </is>
+      </c>
+      <c r="E1192" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1192" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1192" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1192" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1192" t="inlineStr">
+        <is>
+          <t>F44</t>
+        </is>
+      </c>
+      <c r="J1192" t="inlineStr">
+        <is>
+          <t>Two hits nullified for 30 - 46 TP against five for Shadow Clone (17 - 33 TP): 3, 4, 5 by level</t>
+        </is>
+      </c>
+      <c r="K1192" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1192" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>X074</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Magic 216 Shadow Clone</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E1193" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1193" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G1193" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H1193" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1193" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+      <c r="J1193" t="inlineStr">
+        <is>
+          <t>Its chant got slower with each level (0.75 to 0.53; atwiki dt2-2 page 142 notes it): 0.75 at every level</t>
+        </is>
+      </c>
+      <c r="K1193" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1193" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>X075</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>Magic 216 Shadow Clone</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E1194" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1194" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G1194" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H1194" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1194" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+      <c r="J1194" t="inlineStr">
+        <is>
+          <t>Its chant got slower with each level (0.75 to 0.53; atwiki dt2-2 page 142 notes it): 0.75 at every level</t>
+        </is>
+      </c>
+      <c r="K1194" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1194" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>X076</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>Magic 216 Shadow Clone</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E1195" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1195" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G1195" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H1195" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1195" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+      <c r="J1195" t="inlineStr">
+        <is>
+          <t>Its chant got slower with each level (0.75 to 0.53; atwiki dt2-2 page 142 notes it): 0.75 at every level</t>
+        </is>
+      </c>
+      <c r="K1195" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1195" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>X077</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>Magic 216 Shadow Clone</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E1196" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1196" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G1196" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H1196" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1196" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+      <c r="J1196" t="inlineStr">
+        <is>
+          <t>Its chant got slower with each level (0.75 to 0.53; atwiki dt2-2 page 142 notes it): 0.75 at every level</t>
+        </is>
+      </c>
+      <c r="K1196" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1196" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>X078</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>Magic 216 Shadow Clone</t>
+        </is>
+      </c>
+      <c r="D1197" t="inlineStr">
+        <is>
+          <t>chant speed factor</t>
+        </is>
+      </c>
+      <c r="E1197" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1197" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="G1197" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H1197" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1197" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+      <c r="J1197" t="inlineStr">
+        <is>
+          <t>Its chant got slower with each level (0.75 to 0.53; atwiki dt2-2 page 142 notes it): 0.75 at every level</t>
+        </is>
+      </c>
+      <c r="K1197" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1197" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>X079</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>Magic 217 Shadow Sew</t>
+        </is>
+      </c>
+      <c r="D1198" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1198" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1198" t="n">
+        <v>36</v>
+      </c>
+      <c r="G1198" t="n">
+        <v>27</v>
+      </c>
+      <c r="H1198" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1198" t="inlineStr">
+        <is>
+          <t>F61</t>
+        </is>
+      </c>
+      <c r="J1198" t="inlineStr">
+        <is>
+          <t>It lands only on lower level targets and lasts three turns: -25% TP (the cap of the user on TP cuts)</t>
+        </is>
+      </c>
+      <c r="K1198" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1198" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>X080</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>Magic 217 Shadow Sew</t>
+        </is>
+      </c>
+      <c r="D1199" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1199" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1199" t="n">
+        <v>39</v>
+      </c>
+      <c r="G1199" t="n">
+        <v>29</v>
+      </c>
+      <c r="H1199" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1199" t="inlineStr">
+        <is>
+          <t>F61</t>
+        </is>
+      </c>
+      <c r="J1199" t="inlineStr">
+        <is>
+          <t>It lands only on lower level targets and lasts three turns: -25% TP (the cap of the user on TP cuts)</t>
+        </is>
+      </c>
+      <c r="K1199" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1199" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>X081</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>Magic 217 Shadow Sew</t>
+        </is>
+      </c>
+      <c r="D1200" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1200" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1200" t="n">
+        <v>43</v>
+      </c>
+      <c r="G1200" t="n">
+        <v>32</v>
+      </c>
+      <c r="H1200" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1200" t="inlineStr">
+        <is>
+          <t>F61</t>
+        </is>
+      </c>
+      <c r="J1200" t="inlineStr">
+        <is>
+          <t>It lands only on lower level targets and lasts three turns: -25% TP (the cap of the user on TP cuts)</t>
+        </is>
+      </c>
+      <c r="K1200" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1200" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>X082</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>Magic 217 Shadow Sew</t>
+        </is>
+      </c>
+      <c r="D1201" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1201" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1201" t="n">
+        <v>47</v>
+      </c>
+      <c r="G1201" t="n">
+        <v>35</v>
+      </c>
+      <c r="H1201" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1201" t="inlineStr">
+        <is>
+          <t>F61</t>
+        </is>
+      </c>
+      <c r="J1201" t="inlineStr">
+        <is>
+          <t>It lands only on lower level targets and lasts three turns: -25% TP (the cap of the user on TP cuts)</t>
+        </is>
+      </c>
+      <c r="K1201" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1201" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>X083</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>Magic 217 Shadow Sew</t>
+        </is>
+      </c>
+      <c r="D1202" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1202" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1202" t="n">
+        <v>52</v>
+      </c>
+      <c r="G1202" t="n">
+        <v>39</v>
+      </c>
+      <c r="H1202" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1202" t="inlineStr">
+        <is>
+          <t>F61</t>
+        </is>
+      </c>
+      <c r="J1202" t="inlineStr">
+        <is>
+          <t>It lands only on lower level targets and lasts three turns: -25% TP (the cap of the user on TP cuts)</t>
+        </is>
+      </c>
+      <c r="K1202" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1202" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>X084</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>Magic 165 Blood Rage</t>
+        </is>
+      </c>
+      <c r="D1203" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1203" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1203" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1203" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1203" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1203" t="inlineStr">
+        <is>
+          <t>F34</t>
+        </is>
+      </c>
+      <c r="J1203" t="inlineStr">
+        <is>
+          <t>Max HP +20 - 50% for 6 - 10 turns, but 43 TP on a Berserker short of TP: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1203" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1203" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>X085</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>Magic 165 Blood Rage</t>
+        </is>
+      </c>
+      <c r="D1204" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1204" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1204" t="n">
+        <v>31</v>
+      </c>
+      <c r="G1204" t="n">
+        <v>23</v>
+      </c>
+      <c r="H1204" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1204" t="inlineStr">
+        <is>
+          <t>F34</t>
+        </is>
+      </c>
+      <c r="J1204" t="inlineStr">
+        <is>
+          <t>Max HP +20 - 50% for 6 - 10 turns, but 43 TP on a Berserker short of TP: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1204" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1204" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>X086</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>Magic 165 Blood Rage</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1205" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1205" t="n">
+        <v>35</v>
+      </c>
+      <c r="G1205" t="n">
+        <v>26</v>
+      </c>
+      <c r="H1205" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1205" t="inlineStr">
+        <is>
+          <t>F34</t>
+        </is>
+      </c>
+      <c r="J1205" t="inlineStr">
+        <is>
+          <t>Max HP +20 - 50% for 6 - 10 turns, but 43 TP on a Berserker short of TP: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1205" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1205" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>X087</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>Magic 165 Blood Rage</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1206" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1206" t="n">
+        <v>39</v>
+      </c>
+      <c r="G1206" t="n">
+        <v>29</v>
+      </c>
+      <c r="H1206" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1206" t="inlineStr">
+        <is>
+          <t>F34</t>
+        </is>
+      </c>
+      <c r="J1206" t="inlineStr">
+        <is>
+          <t>Max HP +20 - 50% for 6 - 10 turns, but 43 TP on a Berserker short of TP: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1206" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1206" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>X088</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>Magic 165 Blood Rage</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1207" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1207" t="n">
+        <v>43</v>
+      </c>
+      <c r="G1207" t="n">
+        <v>32</v>
+      </c>
+      <c r="H1207" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1207" t="inlineStr">
+        <is>
+          <t>F34</t>
+        </is>
+      </c>
+      <c r="J1207" t="inlineStr">
+        <is>
+          <t>Max HP +20 - 50% for 6 - 10 turns, but 43 TP on a Berserker short of TP: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1207" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1207" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: T06 support proposals accepted
T06 support proposals accepted (Brave, Protect, Illusion, Shadow Clone
chant, Shadow Sew, Blood Rage)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -66163,7 +66163,7 @@
       </c>
       <c r="L1180" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66219,7 +66219,7 @@
       </c>
       <c r="L1181" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66275,7 +66275,7 @@
       </c>
       <c r="L1182" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66331,7 +66331,7 @@
       </c>
       <c r="L1183" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66387,7 +66387,7 @@
       </c>
       <c r="L1184" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66443,7 +66443,7 @@
       </c>
       <c r="L1185" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66499,7 +66499,7 @@
       </c>
       <c r="L1186" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66555,7 +66555,7 @@
       </c>
       <c r="L1187" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66611,7 +66611,7 @@
       </c>
       <c r="L1188" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66667,7 +66667,7 @@
       </c>
       <c r="L1189" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66723,7 +66723,7 @@
       </c>
       <c r="L1190" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66779,7 +66779,7 @@
       </c>
       <c r="L1191" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66835,7 +66835,7 @@
       </c>
       <c r="L1192" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66891,7 +66891,7 @@
       </c>
       <c r="L1193" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -66947,7 +66947,7 @@
       </c>
       <c r="L1194" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67003,7 +67003,7 @@
       </c>
       <c r="L1195" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67059,7 +67059,7 @@
       </c>
       <c r="L1196" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67115,7 +67115,7 @@
       </c>
       <c r="L1197" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67171,7 +67171,7 @@
       </c>
       <c r="L1198" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67227,7 +67227,7 @@
       </c>
       <c r="L1199" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67283,7 +67283,7 @@
       </c>
       <c r="L1200" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67339,7 +67339,7 @@
       </c>
       <c r="L1201" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67395,7 +67395,7 @@
       </c>
       <c r="L1202" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67451,7 +67451,7 @@
       </c>
       <c r="L1203" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67507,7 +67507,7 @@
       </c>
       <c r="L1204" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67563,7 +67563,7 @@
       </c>
       <c r="L1205" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67619,7 +67619,7 @@
       </c>
       <c r="L1206" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -67675,7 +67675,7 @@
       </c>
       <c r="L1207" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: healing spells (decided 2026-10-09)
healing spells (decided 2026-10-09): Circle Heal low levels raised
(never below a Sachertorte), Heal and Circle Heal -25% TP (H001 - H035,
decided); a small cure added to Heal and Circle Heal proposed (H036,
H037, lever L13, as Primevil does in vanilla)

sim: variant.apply fills an empty effect slot ('added effect N (kind
K)'); the heal and damage caps (295, 296) no longer become statuses on
the target
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1207"/>
+  <dimension ref="A1:L1244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67679,6 +67679,2080 @@
         </is>
       </c>
     </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>H001</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>effect 103 (heal power)</t>
+        </is>
+      </c>
+      <c r="E1208" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1208" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1208" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1208" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1208" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1208" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1208" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1208" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>H002</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>effect 103 (heal power)</t>
+        </is>
+      </c>
+      <c r="E1209" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1209" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1209" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H1209" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1209" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1209" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1209" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1209" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>H003</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>effect 103 (heal power)</t>
+        </is>
+      </c>
+      <c r="E1210" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1210" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1210" t="n">
+        <v>11</v>
+      </c>
+      <c r="H1210" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1210" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1210" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1210" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1210" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>H004</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>effect 103 (heal power)</t>
+        </is>
+      </c>
+      <c r="E1211" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1211" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1211" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H1211" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1211" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1211" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1211" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1211" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>H005</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>effect 103 (heal power)</t>
+        </is>
+      </c>
+      <c r="E1212" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1212" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1212" t="n">
+        <v>12</v>
+      </c>
+      <c r="H1212" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1212" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1212" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1212" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1212" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>H006</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>effect 103 (heal power)</t>
+        </is>
+      </c>
+      <c r="E1213" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1213" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1213" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H1213" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1213" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1213" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1213" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1213" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>H007</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>effect 103 (heal power)</t>
+        </is>
+      </c>
+      <c r="E1214" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1214" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1214" t="n">
+        <v>13</v>
+      </c>
+      <c r="H1214" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1214" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1214" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1214" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1214" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>H008</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>effect 103 (heal power)</t>
+        </is>
+      </c>
+      <c r="E1215" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1215" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1215" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H1215" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1215" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1215" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1215" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1215" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>H009</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>effect 103 (heal power)</t>
+        </is>
+      </c>
+      <c r="E1216" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1216" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1216" t="n">
+        <v>14</v>
+      </c>
+      <c r="H1216" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1216" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1216" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1216" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1216" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>H010</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>effect 295 (heal cap)</t>
+        </is>
+      </c>
+      <c r="E1217" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1217" t="n">
+        <v>80</v>
+      </c>
+      <c r="G1217" t="n">
+        <v>200</v>
+      </c>
+      <c r="H1217" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1217" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1217" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1217" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1217" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>H011</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
+        <is>
+          <t>effect 295 (heal cap)</t>
+        </is>
+      </c>
+      <c r="E1218" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1218" t="n">
+        <v>140</v>
+      </c>
+      <c r="G1218" t="n">
+        <v>240</v>
+      </c>
+      <c r="H1218" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1218" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1218" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1218" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1218" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>H012</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1219" t="inlineStr">
+        <is>
+          <t>effect 295 (heal cap)</t>
+        </is>
+      </c>
+      <c r="E1219" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1219" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1219" t="n">
+        <v>280</v>
+      </c>
+      <c r="H1219" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1219" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1219" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1219" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1219" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>H013</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>effect 295 (heal cap)</t>
+        </is>
+      </c>
+      <c r="E1220" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1220" t="n">
+        <v>260</v>
+      </c>
+      <c r="G1220" t="n">
+        <v>320</v>
+      </c>
+      <c r="H1220" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1220" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1220" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1220" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1220" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>H014</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>effect 295 (heal cap)</t>
+        </is>
+      </c>
+      <c r="E1221" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1221" t="n">
+        <v>320</v>
+      </c>
+      <c r="G1221" t="n">
+        <v>360</v>
+      </c>
+      <c r="H1221" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1221" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1221" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1221" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1221" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>H015</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>effect 295 (heal cap)</t>
+        </is>
+      </c>
+      <c r="E1222" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1222" t="n">
+        <v>380</v>
+      </c>
+      <c r="G1222" t="n">
+        <v>400</v>
+      </c>
+      <c r="H1222" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1222" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1222" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): Circle Heal healed 88 to each member at level 1 (C10, C18) where a Sachertorte heals 200 to the party; its low levels raised so it never heals less (210 - 308 at C10 - C22), the top level unchanged (600 cap, 780 at C34)</t>
+        </is>
+      </c>
+      <c r="K1222" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1222" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>H016</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>Magic 187 Heal</t>
+        </is>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1223" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1223" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1223" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1223" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1223" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1223" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1223" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1223" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>H017</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>Magic 187 Heal</t>
+        </is>
+      </c>
+      <c r="D1224" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1224" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1224" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1224" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1224" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1224" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1224" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1224" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1224" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>H018</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>Magic 187 Heal</t>
+        </is>
+      </c>
+      <c r="D1225" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1225" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1225" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1225" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1225" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1225" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1225" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1225" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1225" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>H019</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>Magic 187 Heal</t>
+        </is>
+      </c>
+      <c r="D1226" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1226" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1226" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1226" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1226" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1226" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1226" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1226" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1226" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>H020</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>Magic 187 Heal</t>
+        </is>
+      </c>
+      <c r="D1227" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1227" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1227" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1227" t="n">
+        <v>9</v>
+      </c>
+      <c r="H1227" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1227" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1227" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1227" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1227" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>H021</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>Magic 187 Heal</t>
+        </is>
+      </c>
+      <c r="D1228" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1228" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1228" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1228" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1228" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1228" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1228" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1228" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1228" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>H022</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>Magic 187 Heal</t>
+        </is>
+      </c>
+      <c r="D1229" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1229" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1229" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1229" t="n">
+        <v>12</v>
+      </c>
+      <c r="H1229" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1229" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1229" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1229" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1229" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>H023</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>Magic 187 Heal</t>
+        </is>
+      </c>
+      <c r="D1230" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1230" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1230" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1230" t="n">
+        <v>15</v>
+      </c>
+      <c r="H1230" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1230" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1230" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1230" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1230" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>H024</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>Magic 187 Heal</t>
+        </is>
+      </c>
+      <c r="D1231" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1231" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1231" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1231" t="n">
+        <v>17</v>
+      </c>
+      <c r="H1231" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1231" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1231" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1231" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1231" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>H025</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>Magic 187 Heal</t>
+        </is>
+      </c>
+      <c r="D1232" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1232" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1232" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1232" t="n">
+        <v>19</v>
+      </c>
+      <c r="H1232" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1232" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1232" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1232" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1232" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>H026</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1233" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1233" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1233" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1233" t="n">
+        <v>11</v>
+      </c>
+      <c r="H1233" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1233" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1233" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1233" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1233" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>H027</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1234" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1234" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1234" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1234" t="n">
+        <v>15</v>
+      </c>
+      <c r="H1234" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1234" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1234" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1234" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1234" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>H028</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1235" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1235" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1235" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1235" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1235" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1235" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1235" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1235" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1235" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>H029</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1236" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1236" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1236" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1236" t="n">
+        <v>22</v>
+      </c>
+      <c r="H1236" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1236" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1236" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1236" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1236" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>H030</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1237" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1237" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1237" t="n">
+        <v>35</v>
+      </c>
+      <c r="G1237" t="n">
+        <v>26</v>
+      </c>
+      <c r="H1237" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1237" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1237" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1237" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1237" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>H031</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1238" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1238" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1238" t="n">
+        <v>40</v>
+      </c>
+      <c r="G1238" t="n">
+        <v>30</v>
+      </c>
+      <c r="H1238" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1238" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1238" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1238" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1238" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>H032</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1239" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1239" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1239" t="n">
+        <v>46</v>
+      </c>
+      <c r="G1239" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1239" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1239" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1239" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1239" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1239" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>H033</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1240" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1240" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1240" t="n">
+        <v>52</v>
+      </c>
+      <c r="G1240" t="n">
+        <v>39</v>
+      </c>
+      <c r="H1240" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1240" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1240" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1240" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1240" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>H034</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1241" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1241" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1241" t="n">
+        <v>58</v>
+      </c>
+      <c r="G1241" t="n">
+        <v>43</v>
+      </c>
+      <c r="H1241" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1241" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1241" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1241" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1241" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>H035</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1242" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1242" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1242" t="n">
+        <v>64</v>
+      </c>
+      <c r="G1242" t="n">
+        <v>48</v>
+      </c>
+      <c r="H1242" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1242" t="inlineStr">
+        <is>
+          <t>F21, F41, J24</t>
+        </is>
+      </c>
+      <c r="J1242" t="inlineStr">
+        <is>
+          <t>Healing spells against items (the user, 2026-10-09): an item costs no TP and anyone can use it; the spells already heal more and sooner (Heal 1,040 at C34 against 500 for a Bagel Sandwich), so their cost comes down: -25% TP</t>
+        </is>
+      </c>
+      <c r="K1242" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1242" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>H036</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>Magic 187 Heal</t>
+        </is>
+      </c>
+      <c r="D1243" t="inlineStr">
+        <is>
+          <t>added effect 106 (kind 4)</t>
+        </is>
+      </c>
+      <c r="F1243" t="inlineStr">
+        <is>
+          <t>empty slot</t>
+        </is>
+      </c>
+      <c r="G1243" t="inlineStr">
+        <is>
+          <t>1, 1, 1, 1, 1, 2, 2, 2, 2, 2</t>
+        </is>
+      </c>
+      <c r="H1243" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1243" t="inlineStr">
+        <is>
+          <t>F21, F40</t>
+        </is>
+      </c>
+      <c r="J1243" t="inlineStr">
+        <is>
+          <t>Something small that items do not give, which acts only when it serves (the user, 2026-10-09): Heal also cures poison (levels 1 - 5), then poison and paralysis (6 - 10), the first entries of the cure list (FORMULAS, cures). the vanilla game already joins a heal and a cure in one action: the spell Primevil (Magic 230: effects 103, 106, 105) and the actions Military Rations Pill and Fairy Healing (EnemyAttackData 766 - 768, 772: 103 and 106); the record of a skill holds five effect slots and Heal and Circle Heal use two</t>
+        </is>
+      </c>
+      <c r="K1243" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1243" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>H037</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>Magic 188 Circle Heal</t>
+        </is>
+      </c>
+      <c r="D1244" t="inlineStr">
+        <is>
+          <t>added effect 106 (kind 4)</t>
+        </is>
+      </c>
+      <c r="F1244" t="inlineStr">
+        <is>
+          <t>empty slot</t>
+        </is>
+      </c>
+      <c r="G1244" t="inlineStr">
+        <is>
+          <t>1, 1, 1, 1, 1, 1, 1, 1, 1, 1</t>
+        </is>
+      </c>
+      <c r="H1244" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1244" t="inlineStr">
+        <is>
+          <t>F21, F40</t>
+        </is>
+      </c>
+      <c r="J1244" t="inlineStr">
+        <is>
+          <t>The same for the party: Circle Heal also cures poison. the vanilla game already joins a heal and a cure in one action: the spell Primevil (Magic 230: effects 103, 106, 105) and the actions Military Rations Pill and Fairy Healing (EnemyAttackData 766 - 768, 772: 103 and 106); the record of a skill holds five effect slots and Heal and Circle Heal use two</t>
+        </is>
+      </c>
+      <c r="K1244" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1244" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: the small cure of Heal and Circle Heal accepted
the small cure of Heal and Circle Heal accepted (H036, H037)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -69692,7 +69692,7 @@
       </c>
       <c r="L1243" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -69749,7 +69749,7 @@
       </c>
       <c r="L1244" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: difficulty against vanilla
difficulty against vanilla (tools/difficulty_curve.py: 18 of 44
checkpoints easier, none harder) and the boss fit (tools/boss_fit.py: 16
of 17 back into the windows of vanilla); G001 - G027 proposed (boss HP,
ATK, INT)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1244"/>
+  <dimension ref="A1:L1271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69753,6 +69753,1437 @@
         </is>
       </c>
     </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>G001</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>1006 Agent M (C17)</t>
+        </is>
+      </c>
+      <c r="D1245" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1245" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G1245" t="n">
+        <v>3840</v>
+      </c>
+      <c r="H1245" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1245" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1245" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C17 easier (wins / length / lowest HP: vanilla 100% / 47.8 / 52%, variant 100% / 32.5 / 53%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 39.5 / 52%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1245" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1245" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>G002</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>795 Siesta (C19)</t>
+        </is>
+      </c>
+      <c r="D1246" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1246" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G1246" t="n">
+        <v>3740</v>
+      </c>
+      <c r="H1246" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1246" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1246" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C19 easier (wins / length / lowest HP: vanilla 100% / 7.8 / 66%, variant 92% / 5.7 / 64%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (92% / 6.2 / 63%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1246" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1246" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>G003</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>655 Fuzzy Merchandise (C21)</t>
+        </is>
+      </c>
+      <c r="D1247" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1247" t="n">
+        <v>852</v>
+      </c>
+      <c r="G1247" t="n">
+        <v>937</v>
+      </c>
+      <c r="H1247" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1247" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1247" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C21 easier (wins / length / lowest HP: vanilla 100% / 14.8 / 60%, variant 100% / 9.8 / 65%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 11.3 / 63%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1247" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1247" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>G004</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>656 Fluffy Merchandise (C21)</t>
+        </is>
+      </c>
+      <c r="D1248" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1248" t="n">
+        <v>824</v>
+      </c>
+      <c r="G1248" t="n">
+        <v>906</v>
+      </c>
+      <c r="H1248" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1248" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1248" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C21 easier (wins / length / lowest HP: vanilla 100% / 14.8 / 60%, variant 100% / 9.8 / 65%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 11.3 / 63%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1248" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1248" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>G005</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>1008 Trafficker Twinny (C21)</t>
+        </is>
+      </c>
+      <c r="D1249" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1249" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G1249" t="n">
+        <v>4180</v>
+      </c>
+      <c r="H1249" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1249" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1249" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C21 easier (wins / length / lowest HP: vanilla 100% / 14.8 / 60%, variant 100% / 9.8 / 65%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 11.3 / 63%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1249" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1249" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>G006</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>825 Afanc (C24)</t>
+        </is>
+      </c>
+      <c r="D1250" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1250" t="n">
+        <v>4582</v>
+      </c>
+      <c r="G1250" t="n">
+        <v>5498</v>
+      </c>
+      <c r="H1250" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1250" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1250" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C24 easier (wins / length / lowest HP: vanilla 100% / 6.1 / 63%, variant 100% / 4.2 / 72%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 4.8 / 71%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1250" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1250" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>G007</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>1010 Michelle (C26)</t>
+        </is>
+      </c>
+      <c r="D1251" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1251" t="n">
+        <v>5025</v>
+      </c>
+      <c r="G1251" t="n">
+        <v>9045</v>
+      </c>
+      <c r="H1251" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1251" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1251" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C26 easier (wins / length / lowest HP: vanilla 85% / 24.9 / 47%, variant 100% / 9.4 / 61%); HP x1.80, ATK and INT x1.16 bring it back into the window of vanilla (95% / 24.0 / 47%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1251" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1251" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>G008</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>1010 Michelle (C26)</t>
+        </is>
+      </c>
+      <c r="D1252" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1252" t="n">
+        <v>207</v>
+      </c>
+      <c r="G1252" t="n">
+        <v>240</v>
+      </c>
+      <c r="H1252" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1252" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1252" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C26 easier (wins / length / lowest HP: vanilla 85% / 24.9 / 47%, variant 100% / 9.4 / 61%); HP x1.80, ATK and INT x1.16 bring it back into the window of vanilla (95% / 24.0 / 47%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1252" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1252" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>G009</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>1010 Michelle (C26)</t>
+        </is>
+      </c>
+      <c r="D1253" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1253" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1253" t="n">
+        <v>44</v>
+      </c>
+      <c r="H1253" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1253" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1253" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C26 easier (wins / length / lowest HP: vanilla 85% / 24.9 / 47%, variant 100% / 9.4 / 61%); HP x1.80, ATK and INT x1.16 bring it back into the window of vanilla (95% / 24.0 / 47%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1253" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1253" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>G010</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>1011 Beatrice (C26)</t>
+        </is>
+      </c>
+      <c r="D1254" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1254" t="n">
+        <v>4625</v>
+      </c>
+      <c r="G1254" t="n">
+        <v>8325</v>
+      </c>
+      <c r="H1254" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1254" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1254" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C26 easier (wins / length / lowest HP: vanilla 85% / 24.9 / 47%, variant 100% / 9.4 / 61%); HP x1.80, ATK and INT x1.16 bring it back into the window of vanilla (95% / 24.0 / 47%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1254" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1254" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>G011</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>1011 Beatrice (C26)</t>
+        </is>
+      </c>
+      <c r="D1255" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1255" t="n">
+        <v>163</v>
+      </c>
+      <c r="G1255" t="n">
+        <v>189</v>
+      </c>
+      <c r="H1255" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1255" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1255" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C26 easier (wins / length / lowest HP: vanilla 85% / 24.9 / 47%, variant 100% / 9.4 / 61%); HP x1.80, ATK and INT x1.16 bring it back into the window of vanilla (95% / 24.0 / 47%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1255" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1255" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>G012</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>1011 Beatrice (C26)</t>
+        </is>
+      </c>
+      <c r="D1256" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1256" t="n">
+        <v>48</v>
+      </c>
+      <c r="G1256" t="n">
+        <v>56</v>
+      </c>
+      <c r="H1256" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1256" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1256" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C26 easier (wins / length / lowest HP: vanilla 85% / 24.9 / 47%, variant 100% / 9.4 / 61%); HP x1.80, ATK and INT x1.16 bring it back into the window of vanilla (95% / 24.0 / 47%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1256" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1256" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>G013</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>964 Forest Guardian (C27)</t>
+        </is>
+      </c>
+      <c r="D1257" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1257" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G1257" t="n">
+        <v>2200</v>
+      </c>
+      <c r="H1257" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1257" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1257" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C27 easier (wins / length / lowest HP: vanilla 100% / 5.0 / 83%, variant 100% / 3.6 / 88%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 3.8 / 89%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1257" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1257" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>G014</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>1012 Spirit of Mag Mell (C28)</t>
+        </is>
+      </c>
+      <c r="D1258" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1258" t="n">
+        <v>8200</v>
+      </c>
+      <c r="G1258" t="n">
+        <v>9840</v>
+      </c>
+      <c r="H1258" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1258" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1258" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C28 easier (wins / length / lowest HP: vanilla 95% / 13.2 / 35%, variant 98% / 8.3 / 47%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (95% / 10.2 / 43%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1258" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1258" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>G015</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>785 Calliope (C29)</t>
+        </is>
+      </c>
+      <c r="D1259" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1259" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G1259" t="n">
+        <v>9750</v>
+      </c>
+      <c r="H1259" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1259" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1259" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C29 easier (wins / length / lowest HP: vanilla 15% / 39.5 / 13%, variant 40% / 27.2 / 23%); HP x1.30, ATK and INT x1.00 bring it back into the window of vanilla (20% / 33.7 / 11%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1259" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1259" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>G016</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>840 Moby Dick (C32)</t>
+        </is>
+      </c>
+      <c r="D1260" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1260" t="n">
+        <v>13280</v>
+      </c>
+      <c r="G1260" t="n">
+        <v>19256</v>
+      </c>
+      <c r="H1260" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1260" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1260" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C32 easier (wins / length / lowest HP: vanilla 92% / 20.6 / 45%, variant 100% / 12.7 / 61%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (100% / 20.7 / 51%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1260" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1260" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>G017</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>1036 Queen of Darkness (C34)</t>
+        </is>
+      </c>
+      <c r="D1261" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1261" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G1261" t="n">
+        <v>9600</v>
+      </c>
+      <c r="H1261" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1261" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1261" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C34 easier (wins / length / lowest HP: vanilla 100% / 41.3 / 59%, variant 100% / 22.6 / 64%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 31.0 / 60%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1261" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1261" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>G018</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>1037 Queen of Darkness (C34)</t>
+        </is>
+      </c>
+      <c r="D1262" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1262" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G1262" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H1262" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1262" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1262" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C34 easier (wins / length / lowest HP: vanilla 100% / 41.3 / 59%, variant 100% / 22.6 / 64%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 31.0 / 60%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1262" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1262" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>G019</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>1015 Demon God Fried (C36)</t>
+        </is>
+      </c>
+      <c r="D1263" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1263" t="n">
+        <v>18000</v>
+      </c>
+      <c r="G1263" t="n">
+        <v>19800</v>
+      </c>
+      <c r="H1263" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1263" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1263" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C36 easier (wins / length / lowest HP: vanilla 90% / 17.4 / 0%, variant 95% / 12.6 / 0%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 14.0 / 1%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1263" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1263" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>G020</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>865 Iron Maiden (C37)</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1264" t="n">
+        <v>16800</v>
+      </c>
+      <c r="G1264" t="n">
+        <v>20160</v>
+      </c>
+      <c r="H1264" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1264" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1264" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C37 easier (wins / length / lowest HP: vanilla 100% / 14.4 / 60%, variant 100% / 9.7 / 62%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 12.0 / 60%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1264" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1264" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>G021</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>950 Samael (C38)</t>
+        </is>
+      </c>
+      <c r="D1265" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1265" t="n">
+        <v>18500</v>
+      </c>
+      <c r="G1265" t="n">
+        <v>26825</v>
+      </c>
+      <c r="H1265" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1265" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1265" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C38 easier (wins / length / lowest HP: vanilla 60% / 18.1 / 27%, variant 92% / 11.8 / 55%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (68% / 18.4 / 36%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1265" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1265" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>G022</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>958 Demiurge (C40)</t>
+        </is>
+      </c>
+      <c r="D1266" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1266" t="n">
+        <v>24000</v>
+      </c>
+      <c r="G1266" t="n">
+        <v>34800</v>
+      </c>
+      <c r="H1266" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1266" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1266" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C40 easier (wins / length / lowest HP: vanilla 75% / 37.1 / 26%, variant 95% / 23.5 / 41%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (85% / 41.0 / 31%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1266" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1266" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>G023</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>961 Atialuco (C40)</t>
+        </is>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1267" t="n">
+        <v>21800</v>
+      </c>
+      <c r="G1267" t="n">
+        <v>31610</v>
+      </c>
+      <c r="H1267" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1267" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1267" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C40 easier (wins / length / lowest HP: vanilla 75% / 37.1 / 26%, variant 95% / 23.5 / 41%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (85% / 41.0 / 31%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1267" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1267" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>G024</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>848 Qitian Dasheng (P08)</t>
+        </is>
+      </c>
+      <c r="D1268" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1268" t="n">
+        <v>28000</v>
+      </c>
+      <c r="G1268" t="n">
+        <v>30800</v>
+      </c>
+      <c r="H1268" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1268" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1268" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P08 easier (wins / length / lowest HP: vanilla 100% / 6.2 / 88%, variant 100% / 4.5 / 90%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 4.9 / 89%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1268" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1268" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>G025</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>582 Peggy Oversummoner (P24)</t>
+        </is>
+      </c>
+      <c r="D1269" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1269" t="n">
+        <v>8501</v>
+      </c>
+      <c r="G1269" t="n">
+        <v>9351</v>
+      </c>
+      <c r="H1269" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1269" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1269" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P24 easier (wins / length / lowest HP: vanilla 100% / 4.9 / 58%, variant 100% / 3.6 / 62%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 4.0 / 57%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1269" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1269" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>G026</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>588 Roger Orso (P24)</t>
+        </is>
+      </c>
+      <c r="D1270" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1270" t="n">
+        <v>9121</v>
+      </c>
+      <c r="G1270" t="n">
+        <v>10033</v>
+      </c>
+      <c r="H1270" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1270" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1270" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P24 easier (wins / length / lowest HP: vanilla 100% / 4.9 / 58%, variant 100% / 3.6 / 62%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 4.0 / 57%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1270" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1270" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>G027</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>1026 Aradia (P24)</t>
+        </is>
+      </c>
+      <c r="D1271" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1271" t="n">
+        <v>41500</v>
+      </c>
+      <c r="G1271" t="n">
+        <v>45650</v>
+      </c>
+      <c r="H1271" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1271" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1271" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P24 easier (wins / length / lowest HP: vanilla 100% / 4.9 / 58%, variant 100% / 3.6 / 62%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 4.0 / 57%). Only enemies of no random formation</t>
+        </is>
+      </c>
+      <c r="K1271" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1271" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: difficulty brought back within the windows of vanilla
difficulty brought back within the windows of vanilla : bosses G001 -
G033 decided (C30 fitted with HP x1.30, ATK and INT x0.92) and the
common enemies of the C39 and C40 floors (G034 - G093); 42 of 44
checkpoints within
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1271"/>
+  <dimension ref="A1:L1337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69802,7 +69802,7 @@
       </c>
       <c r="L1245" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -69855,7 +69855,7 @@
       </c>
       <c r="L1246" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -69908,7 +69908,7 @@
       </c>
       <c r="L1247" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -69961,7 +69961,7 @@
       </c>
       <c r="L1248" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70014,7 +70014,7 @@
       </c>
       <c r="L1249" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70067,7 +70067,7 @@
       </c>
       <c r="L1250" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70120,7 +70120,7 @@
       </c>
       <c r="L1251" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70173,7 +70173,7 @@
       </c>
       <c r="L1252" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70226,7 +70226,7 @@
       </c>
       <c r="L1253" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70279,7 +70279,7 @@
       </c>
       <c r="L1254" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70332,7 +70332,7 @@
       </c>
       <c r="L1255" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70385,7 +70385,7 @@
       </c>
       <c r="L1256" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70438,7 +70438,7 @@
       </c>
       <c r="L1257" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70491,7 +70491,7 @@
       </c>
       <c r="L1258" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70544,7 +70544,7 @@
       </c>
       <c r="L1259" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70597,7 +70597,7 @@
       </c>
       <c r="L1260" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70650,7 +70650,7 @@
       </c>
       <c r="L1261" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70703,7 +70703,7 @@
       </c>
       <c r="L1262" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70756,7 +70756,7 @@
       </c>
       <c r="L1263" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70809,7 +70809,7 @@
       </c>
       <c r="L1264" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70862,7 +70862,7 @@
       </c>
       <c r="L1265" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70915,7 +70915,7 @@
       </c>
       <c r="L1266" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -70968,7 +70968,7 @@
       </c>
       <c r="L1267" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -71021,7 +71021,7 @@
       </c>
       <c r="L1268" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -71074,7 +71074,7 @@
       </c>
       <c r="L1269" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -71127,7 +71127,7 @@
       </c>
       <c r="L1270" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
         </is>
       </c>
     </row>
@@ -71180,7 +71180,3505 @@
       </c>
       <c r="L1271" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>G028</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>1013 Heartless Avenger (C30)</t>
+        </is>
+      </c>
+      <c r="D1272" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1272" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G1272" t="n">
+        <v>11050</v>
+      </c>
+      <c r="H1272" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1272" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1272" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py, wider search asked by the user): C30, two fights in a row, was easier on the variant (wins / length / lowest HP: vanilla 90% / 44.4 / 45%, variant 95% / 32.8 / 47%); HP x1.30 with ATK and INT x0.92 bring it back into the window of vanilla (88% / 54.7 / 43%); HP alone made it far harder (42% wins)</t>
+        </is>
+      </c>
+      <c r="K1272" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1272" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>G029</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>1013 Heartless Avenger (C30)</t>
+        </is>
+      </c>
+      <c r="D1273" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1273" t="n">
+        <v>236</v>
+      </c>
+      <c r="G1273" t="n">
+        <v>217</v>
+      </c>
+      <c r="H1273" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1273" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1273" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py, wider search asked by the user): C30, two fights in a row, was easier on the variant (wins / length / lowest HP: vanilla 90% / 44.4 / 45%, variant 95% / 32.8 / 47%); HP x1.30 with ATK and INT x0.92 bring it back into the window of vanilla (88% / 54.7 / 43%); HP alone made it far harder (42% wins)</t>
+        </is>
+      </c>
+      <c r="K1273" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1273" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>G030</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>1013 Heartless Avenger (C30)</t>
+        </is>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1274" t="n">
+        <v>79</v>
+      </c>
+      <c r="G1274" t="n">
+        <v>73</v>
+      </c>
+      <c r="H1274" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1274" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1274" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py, wider search asked by the user): C30, two fights in a row, was easier on the variant (wins / length / lowest HP: vanilla 90% / 44.4 / 45%, variant 95% / 32.8 / 47%); HP x1.30 with ATK and INT x0.92 bring it back into the window of vanilla (88% / 54.7 / 43%); HP alone made it far harder (42% wins)</t>
+        </is>
+      </c>
+      <c r="K1274" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1274" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>G031</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>1035 Heartless Avenger (C30)</t>
+        </is>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1275" t="n">
+        <v>6800</v>
+      </c>
+      <c r="G1275" t="n">
+        <v>8840</v>
+      </c>
+      <c r="H1275" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1275" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1275" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py, wider search asked by the user): C30, two fights in a row, was easier on the variant (wins / length / lowest HP: vanilla 90% / 44.4 / 45%, variant 95% / 32.8 / 47%); HP x1.30 with ATK and INT x0.92 bring it back into the window of vanilla (88% / 54.7 / 43%); HP alone made it far harder (42% wins)</t>
+        </is>
+      </c>
+      <c r="K1275" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1275" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>G032</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>1035 Heartless Avenger (C30)</t>
+        </is>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1276" t="n">
+        <v>255</v>
+      </c>
+      <c r="G1276" t="n">
+        <v>235</v>
+      </c>
+      <c r="H1276" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1276" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1276" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py, wider search asked by the user): C30, two fights in a row, was easier on the variant (wins / length / lowest HP: vanilla 90% / 44.4 / 45%, variant 95% / 32.8 / 47%); HP x1.30 with ATK and INT x0.92 bring it back into the window of vanilla (88% / 54.7 / 43%); HP alone made it far harder (42% wins)</t>
+        </is>
+      </c>
+      <c r="K1276" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1276" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>G033</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>1035 Heartless Avenger (C30)</t>
+        </is>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1277" t="n">
+        <v>79</v>
+      </c>
+      <c r="G1277" t="n">
+        <v>73</v>
+      </c>
+      <c r="H1277" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1277" t="inlineStr">
+        <is>
+          <t>R08, R10, S04</t>
+        </is>
+      </c>
+      <c r="J1277" t="inlineStr">
+        <is>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py, wider search asked by the user): C30, two fights in a row, was easier on the variant (wins / length / lowest HP: vanilla 90% / 44.4 / 45%, variant 95% / 32.8 / 47%); HP x1.30 with ATK and INT x0.92 bring it back into the window of vanilla (88% / 54.7 / 43%); HP alone made it far harder (42% wins)</t>
+        </is>
+      </c>
+      <c r="K1277" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1277" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>G034</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>78 Macha (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1278" t="n">
+        <v>7827</v>
+      </c>
+      <c r="G1278" t="n">
+        <v>15263</v>
+      </c>
+      <c r="H1278" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1278" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1278" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1278" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1278" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>G035</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>78 Macha (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1279" t="n">
+        <v>363</v>
+      </c>
+      <c r="G1279" t="n">
+        <v>613</v>
+      </c>
+      <c r="H1279" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1279" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1279" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1279" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1279" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>G036</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>78 Macha (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1280" t="n">
+        <v>132</v>
+      </c>
+      <c r="G1280" t="n">
+        <v>223</v>
+      </c>
+      <c r="H1280" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1280" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1280" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1280" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1280" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>G037</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>92 Leanan Sidhe (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1281" t="n">
+        <v>1531</v>
+      </c>
+      <c r="G1281" t="n">
+        <v>1990</v>
+      </c>
+      <c r="H1281" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1281" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1281" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1281" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1281" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>G038</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>92 Leanan Sidhe (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1282" t="n">
+        <v>236</v>
+      </c>
+      <c r="G1282" t="n">
+        <v>307</v>
+      </c>
+      <c r="H1282" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1282" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1282" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1282" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1282" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>G039</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>92 Leanan Sidhe (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1283" t="n">
+        <v>68</v>
+      </c>
+      <c r="G1283" t="n">
+        <v>88</v>
+      </c>
+      <c r="H1283" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1283" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1283" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1283" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1283" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>G040</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>108 Shahrazad (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1284" t="n">
+        <v>1544</v>
+      </c>
+      <c r="G1284" t="n">
+        <v>2007</v>
+      </c>
+      <c r="H1284" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1284" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1284" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1284" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1284" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>G041</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>108 Shahrazad (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1285" t="n">
+        <v>242</v>
+      </c>
+      <c r="G1285" t="n">
+        <v>315</v>
+      </c>
+      <c r="H1285" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1285" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1285" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1285" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1285" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>G042</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>108 Shahrazad (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1286" t="n">
+        <v>77</v>
+      </c>
+      <c r="G1286" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1286" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1286" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1286" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1286" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1286" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>G043</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>120 Stheno (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1287" t="n">
+        <v>2397</v>
+      </c>
+      <c r="G1287" t="n">
+        <v>3116</v>
+      </c>
+      <c r="H1287" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1287" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1287" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1287" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1287" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>G044</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>120 Stheno (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1288" t="n">
+        <v>292</v>
+      </c>
+      <c r="G1288" t="n">
+        <v>380</v>
+      </c>
+      <c r="H1288" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1288" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1288" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1288" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1288" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>G045</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>120 Stheno (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1289" t="n">
+        <v>145</v>
+      </c>
+      <c r="G1289" t="n">
+        <v>188</v>
+      </c>
+      <c r="H1289" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1289" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1289" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1289" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1289" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>G046</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>138 Pabilsag (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1290" t="n">
+        <v>1683</v>
+      </c>
+      <c r="G1290" t="n">
+        <v>2188</v>
+      </c>
+      <c r="H1290" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1290" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1290" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1290" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1290" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>G047</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>138 Pabilsag (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1291" t="n">
+        <v>245</v>
+      </c>
+      <c r="G1291" t="n">
+        <v>318</v>
+      </c>
+      <c r="H1291" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1291" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1291" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1291" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1291" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>G048</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>138 Pabilsag (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1292" t="n">
+        <v>67</v>
+      </c>
+      <c r="G1292" t="n">
+        <v>87</v>
+      </c>
+      <c r="H1292" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1292" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1292" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1292" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1292" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>G049</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>189 Leprechaun (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1293" t="n">
+        <v>1745</v>
+      </c>
+      <c r="G1293" t="n">
+        <v>2268</v>
+      </c>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1293" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1293" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1293" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1293" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>G050</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>189 Leprechaun (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1294" t="n">
+        <v>291</v>
+      </c>
+      <c r="G1294" t="n">
+        <v>378</v>
+      </c>
+      <c r="H1294" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1294" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1294" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1294" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1294" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>G051</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>189 Leprechaun (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1295" t="n">
+        <v>71</v>
+      </c>
+      <c r="G1295" t="n">
+        <v>92</v>
+      </c>
+      <c r="H1295" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1295" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1295" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1295" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1295" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>G052</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>258 Lorelei (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1296" t="n">
+        <v>1475</v>
+      </c>
+      <c r="G1296" t="n">
+        <v>1918</v>
+      </c>
+      <c r="H1296" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1296" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1296" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1296" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1296" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>G053</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>258 Lorelei (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1297" t="n">
+        <v>217</v>
+      </c>
+      <c r="G1297" t="n">
+        <v>282</v>
+      </c>
+      <c r="H1297" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1297" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1297" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1297" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1297" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>G054</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>258 Lorelei (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1298" t="n">
+        <v>82</v>
+      </c>
+      <c r="G1298" t="n">
+        <v>107</v>
+      </c>
+      <c r="H1298" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1298" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1298" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1298" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1298" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>G055</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>279 Centenary (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1299" t="n">
+        <v>1542</v>
+      </c>
+      <c r="G1299" t="n">
+        <v>2005</v>
+      </c>
+      <c r="H1299" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1299" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1299" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1299" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1299" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>G056</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>279 Centenary (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1300" t="n">
+        <v>231</v>
+      </c>
+      <c r="G1300" t="n">
+        <v>300</v>
+      </c>
+      <c r="H1300" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1300" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1300" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1300" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1300" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>G057</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>279 Centenary (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1301" t="n">
+        <v>109</v>
+      </c>
+      <c r="G1301" t="n">
+        <v>142</v>
+      </c>
+      <c r="H1301" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1301" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1301" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1301" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1301" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>G058</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>296 Purski (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1302" t="n">
+        <v>2673</v>
+      </c>
+      <c r="G1302" t="n">
+        <v>5212</v>
+      </c>
+      <c r="H1302" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1302" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1302" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1302" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1302" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>G059</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>296 Purski (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1303" t="n">
+        <v>313</v>
+      </c>
+      <c r="G1303" t="n">
+        <v>529</v>
+      </c>
+      <c r="H1303" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1303" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1303" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1303" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1303" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>G060</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>296 Purski (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1304" t="n">
+        <v>108</v>
+      </c>
+      <c r="G1304" t="n">
+        <v>183</v>
+      </c>
+      <c r="H1304" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1304" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1304" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1304" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1304" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>G061</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>337 Storm Bringer (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1305" t="n">
+        <v>1631</v>
+      </c>
+      <c r="G1305" t="n">
+        <v>2120</v>
+      </c>
+      <c r="H1305" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1305" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1305" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1305" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1305" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>G062</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>337 Storm Bringer (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1306" t="n">
+        <v>272</v>
+      </c>
+      <c r="G1306" t="n">
+        <v>354</v>
+      </c>
+      <c r="H1306" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1306" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1306" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1306" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1306" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>G063</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>337 Storm Bringer (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1307" t="n">
+        <v>62</v>
+      </c>
+      <c r="G1307" t="n">
+        <v>81</v>
+      </c>
+      <c r="H1307" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1307" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1307" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1307" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1307" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>G064</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>356 Balrog (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1308" t="n">
+        <v>1643</v>
+      </c>
+      <c r="G1308" t="n">
+        <v>2136</v>
+      </c>
+      <c r="H1308" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1308" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1308" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1308" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1308" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>G065</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>356 Balrog (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1309" t="n">
+        <v>275</v>
+      </c>
+      <c r="G1309" t="n">
+        <v>358</v>
+      </c>
+      <c r="H1309" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1309" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1309" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1309" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1309" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>G066</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>356 Balrog (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1310" t="n">
+        <v>62</v>
+      </c>
+      <c r="G1310" t="n">
+        <v>81</v>
+      </c>
+      <c r="H1310" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1310" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1310" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1310" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1310" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>G067</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>368 Melusine (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1311" t="n">
+        <v>1668</v>
+      </c>
+      <c r="G1311" t="n">
+        <v>2168</v>
+      </c>
+      <c r="H1311" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1311" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1311" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1311" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1311" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>G068</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>368 Melusine (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1312" t="n">
+        <v>264</v>
+      </c>
+      <c r="G1312" t="n">
+        <v>343</v>
+      </c>
+      <c r="H1312" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1312" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1312" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1312" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1312" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>G069</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>368 Melusine (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1313" t="n">
+        <v>93</v>
+      </c>
+      <c r="G1313" t="n">
+        <v>121</v>
+      </c>
+      <c r="H1313" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1313" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1313" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1313" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1313" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>G070</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>399 Dzelarhons (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1314" t="n">
+        <v>1729</v>
+      </c>
+      <c r="G1314" t="n">
+        <v>2248</v>
+      </c>
+      <c r="H1314" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1314" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1314" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1314" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1314" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>G071</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>399 Dzelarhons (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1315" t="n">
+        <v>259</v>
+      </c>
+      <c r="G1315" t="n">
+        <v>337</v>
+      </c>
+      <c r="H1315" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1315" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1315" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1315" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1315" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>G072</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>399 Dzelarhons (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1316" t="n">
+        <v>59</v>
+      </c>
+      <c r="G1316" t="n">
+        <v>77</v>
+      </c>
+      <c r="H1316" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1316" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1316" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1316" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1316" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>G073</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>403 Fafnir (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1317" t="n">
+        <v>3042</v>
+      </c>
+      <c r="G1317" t="n">
+        <v>3955</v>
+      </c>
+      <c r="H1317" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1317" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1317" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1317" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1317" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>G074</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>403 Fafnir (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1318" t="n">
+        <v>321</v>
+      </c>
+      <c r="G1318" t="n">
+        <v>417</v>
+      </c>
+      <c r="H1318" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1318" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1318" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1318" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1318" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>G075</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>403 Fafnir (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1319" t="n">
+        <v>91</v>
+      </c>
+      <c r="G1319" t="n">
+        <v>118</v>
+      </c>
+      <c r="H1319" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1319" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1319" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1319" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1319" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>G076</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>423 Isis (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1320" t="n">
+        <v>1559</v>
+      </c>
+      <c r="G1320" t="n">
+        <v>2027</v>
+      </c>
+      <c r="H1320" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1320" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1320" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1320" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1320" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>G077</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>423 Isis (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1321" t="n">
+        <v>237</v>
+      </c>
+      <c r="G1321" t="n">
+        <v>308</v>
+      </c>
+      <c r="H1321" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1321" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1321" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1321" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1321" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>G078</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>423 Isis (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1322" t="n">
+        <v>94</v>
+      </c>
+      <c r="G1322" t="n">
+        <v>122</v>
+      </c>
+      <c r="H1322" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1322" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1322" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1322" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1322" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>G079</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>508 Metal Mandra ♀ (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1323" t="n">
+        <v>1203</v>
+      </c>
+      <c r="G1323" t="n">
+        <v>1564</v>
+      </c>
+      <c r="H1323" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1323" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1323" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1323" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1323" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>G080</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>508 Metal Mandra ♀ (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1324" t="n">
+        <v>218</v>
+      </c>
+      <c r="G1324" t="n">
+        <v>283</v>
+      </c>
+      <c r="H1324" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1324" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1324" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1324" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1324" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>G081</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>508 Metal Mandra ♀ (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1325" t="n">
+        <v>89</v>
+      </c>
+      <c r="G1325" t="n">
+        <v>116</v>
+      </c>
+      <c r="H1325" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1325" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1325" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1325" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1325" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>G082</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>761 Yab-Yum (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1326" t="n">
+        <v>1411</v>
+      </c>
+      <c r="G1326" t="n">
+        <v>1834</v>
+      </c>
+      <c r="H1326" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1326" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1326" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1326" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1326" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>G083</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>761 Yab-Yum (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1327" t="n">
+        <v>214</v>
+      </c>
+      <c r="G1327" t="n">
+        <v>278</v>
+      </c>
+      <c r="H1327" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1327" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1327" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1327" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1327" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>G084</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>761 Yab-Yum (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1328" t="n">
+        <v>71</v>
+      </c>
+      <c r="G1328" t="n">
+        <v>92</v>
+      </c>
+      <c r="H1328" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1328" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1328" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1328" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1328" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>G085</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>841 Space Whale (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1329" t="n">
+        <v>4675</v>
+      </c>
+      <c r="G1329" t="n">
+        <v>6078</v>
+      </c>
+      <c r="H1329" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1329" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1329" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1329" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1329" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>G086</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>841 Space Whale (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1330" t="n">
+        <v>322</v>
+      </c>
+      <c r="G1330" t="n">
+        <v>419</v>
+      </c>
+      <c r="H1330" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1330" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1330" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1330" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1330" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>G087</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>841 Space Whale (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1331" t="n">
+        <v>148</v>
+      </c>
+      <c r="G1331" t="n">
+        <v>192</v>
+      </c>
+      <c r="H1331" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1331" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1331" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1331" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1331" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>G088</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>886 Yato-no-Kami (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1332" t="n">
+        <v>1811</v>
+      </c>
+      <c r="G1332" t="n">
+        <v>2354</v>
+      </c>
+      <c r="H1332" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1332" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1332" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1332" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1332" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>G089</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>886 Yato-no-Kami (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1333" t="n">
+        <v>258</v>
+      </c>
+      <c r="G1333" t="n">
+        <v>335</v>
+      </c>
+      <c r="H1333" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1333" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1333" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1333" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1333" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>G090</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>886 Yato-no-Kami (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1334" t="n">
+        <v>81</v>
+      </c>
+      <c r="G1334" t="n">
+        <v>105</v>
+      </c>
+      <c r="H1334" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1334" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1334" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1334" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1334" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>G091</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>919 Highway Star (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1335" t="n">
+        <v>5871</v>
+      </c>
+      <c r="G1335" t="n">
+        <v>11448</v>
+      </c>
+      <c r="H1335" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1335" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1335" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1335" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1335" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>G092</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>919 Highway Star (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1336" t="n">
+        <v>348</v>
+      </c>
+      <c r="G1336" t="n">
+        <v>588</v>
+      </c>
+      <c r="H1336" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1336" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1336" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1336" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1336" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>G093</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>919 Highway Star (common, St15)</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F1337" t="n">
+        <v>128</v>
+      </c>
+      <c r="G1337" t="n">
+        <v>216</v>
+      </c>
+      <c r="H1337" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1337" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1337" t="inlineStr">
+        <is>
+          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+        </is>
+      </c>
+      <c r="K1337" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1337" t="inlineStr">
+        <is>
+          <t>decided</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: T07 checked by measure
T07 checked by measure (decided 2026-10-09): poison opened on six story
bosses (C09, C31, C34, C37, C38, C40; A rows), five kept immune;
ailments on random rows measured as the opening move
(tools/skill_value.py): Paralyze 50% > 70% of rows won on the C39 and
C40 floors; Carol at 0 leaves common fights easy (F16, S05 results)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1337"/>
+  <dimension ref="A1:L1338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35151,7 +35151,7 @@
       </c>
       <c r="G620" t="inlineStr">
         <is>
-          <t>0x37e7</t>
+          <t>0x36e7</t>
         </is>
       </c>
       <c r="H620" t="inlineStr">
@@ -35161,12 +35161,12 @@
       </c>
       <c r="I620" t="inlineStr">
         <is>
-          <t>J31, F15</t>
+          <t>J31, F15, T07</t>
         </is>
       </c>
       <c r="J620" t="inlineStr">
         <is>
-          <t>Bosses: immune to turn delay (no boss lockable by Tinker Squash or the like); open to slow and silence unless a superboss, and to sleep in the story</t>
+          <t>Bosses: immune to turn delay (no boss lockable by Tinker Squash or the like); open to slow and silence unless a superboss, and to sleep in the story; poison opened (T07, the user 2026-10-09: damage over time must serve against bosses without trivialising them): healer's Poison cast until it lands takes 23% of the boss HP over the fight (tools/skill_value.py play, check_runs), under a quarter. Kept immune: Ghast, Doll, Countess of Vrachia (undead or doll), Beatrice (C26 already 27% through Michelle), Heartless Avenger (C30: 32%, the fight halved)</t>
         </is>
       </c>
       <c r="K620" t="inlineStr">
@@ -36462,7 +36462,7 @@
       </c>
       <c r="G643" t="inlineStr">
         <is>
-          <t>0x1163</t>
+          <t>0x1063</t>
         </is>
       </c>
       <c r="H643" t="inlineStr">
@@ -36472,12 +36472,12 @@
       </c>
       <c r="I643" t="inlineStr">
         <is>
-          <t>J31, F15</t>
+          <t>J31, F15, T07</t>
         </is>
       </c>
       <c r="J643" t="inlineStr">
         <is>
-          <t>Bosses: immune to turn delay (no boss lockable by Tinker Squash or the like); open to slow and silence unless a superboss, and to sleep in the story</t>
+          <t>Bosses: immune to turn delay (no boss lockable by Tinker Squash or the like); open to slow and silence unless a superboss, and to sleep in the story; poison opened (T07, the user 2026-10-09: damage over time must serve against bosses without trivialising them): healer's Poison cast until it lands takes 20% of the boss HP over the fight (tools/skill_value.py play, check_runs), under a quarter. Kept immune: Ghast, Doll, Countess of Vrachia (undead or doll), Beatrice (C26 already 27% through Michelle), Heartless Avenger (C30: 32%, the fight halved)</t>
         </is>
       </c>
       <c r="K643" t="inlineStr">
@@ -37089,7 +37089,7 @@
       </c>
       <c r="G654" t="inlineStr">
         <is>
-          <t>0x11e7</t>
+          <t>0x10e7</t>
         </is>
       </c>
       <c r="H654" t="inlineStr">
@@ -37099,12 +37099,12 @@
       </c>
       <c r="I654" t="inlineStr">
         <is>
-          <t>J31, F15</t>
+          <t>J31, F15, T07</t>
         </is>
       </c>
       <c r="J654" t="inlineStr">
         <is>
-          <t>Bosses: immune to turn delay (no boss lockable by Tinker Squash or the like); open to slow and silence unless a superboss, and to sleep in the story</t>
+          <t>Bosses: immune to turn delay (no boss lockable by Tinker Squash or the like); open to slow and silence unless a superboss, and to sleep in the story; poison opened (T07, the user 2026-10-09: damage over time must serve against bosses without trivialising them): healer's Poison cast until it lands takes 25% of the boss HP over the fight (tools/skill_value.py play, check_runs), under a quarter. Kept immune: Ghast, Doll, Countess of Vrachia (undead or doll), Beatrice (C26 already 27% through Michelle), Heartless Avenger (C30: 32%, the fight halved)</t>
         </is>
       </c>
       <c r="K654" t="inlineStr">
@@ -37317,7 +37317,7 @@
       </c>
       <c r="G658" t="inlineStr">
         <is>
-          <t>0x35e2</t>
+          <t>0x34e2</t>
         </is>
       </c>
       <c r="H658" t="inlineStr">
@@ -37327,12 +37327,12 @@
       </c>
       <c r="I658" t="inlineStr">
         <is>
-          <t>J31, F15</t>
+          <t>J31, F15, T07</t>
         </is>
       </c>
       <c r="J658" t="inlineStr">
         <is>
-          <t>Bosses: immune to turn delay (no boss lockable by Tinker Squash or the like); open to slow and silence unless a superboss, and to sleep in the story</t>
+          <t>Bosses: immune to turn delay (no boss lockable by Tinker Squash or the like); open to slow and silence unless a superboss, and to sleep in the story; poison opened (T07, the user 2026-10-09: damage over time must serve against bosses without trivialising them): healer's Poison cast until it lands takes 16% of the boss HP over the fight (tools/skill_value.py play, check_runs), under a quarter. Kept immune: Ghast, Doll, Countess of Vrachia (undead or doll), Beatrice (C26 already 27% through Michelle), Heartless Avenger (C30: 32%, the fight halved)</t>
         </is>
       </c>
       <c r="K658" t="inlineStr">
@@ -39198,7 +39198,7 @@
       </c>
       <c r="G691" t="inlineStr">
         <is>
-          <t>0x1766</t>
+          <t>0x1666</t>
         </is>
       </c>
       <c r="H691" t="inlineStr">
@@ -39208,12 +39208,12 @@
       </c>
       <c r="I691" t="inlineStr">
         <is>
-          <t>J31, F15</t>
+          <t>J31, F15, T07</t>
         </is>
       </c>
       <c r="J691" t="inlineStr">
         <is>
-          <t>Bosses: immune to turn delay (no boss lockable by Tinker Squash or the like); open to slow and silence unless a superboss, and to sleep in the story</t>
+          <t>Bosses: immune to turn delay (no boss lockable by Tinker Squash or the like); open to slow and silence unless a superboss, and to sleep in the story; poison opened (T07, the user 2026-10-09: damage over time must serve against bosses without trivialising them): healer's Poison cast until it lands takes 25% of the boss HP over the fight (tools/skill_value.py play, check_runs), under a quarter. Kept immune: Ghast, Doll, Countess of Vrachia (undead or doll), Beatrice (C26 already 27% through Michelle), Heartless Avenger (C30: 32%, the fight halved)</t>
         </is>
       </c>
       <c r="K691" t="inlineStr">
@@ -74677,6 +74677,63 @@
         </is>
       </c>
       <c r="L1337" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>A239</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>961 Atialuco (C40)</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>immunity flags (0x3C)</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>0x35fe</t>
+        </is>
+      </c>
+      <c r="G1338" t="inlineStr">
+        <is>
+          <t>0x34fe</t>
+        </is>
+      </c>
+      <c r="H1338" t="inlineStr">
+        <is>
+          <t>L26</t>
+        </is>
+      </c>
+      <c r="I1338" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="J1338" t="inlineStr">
+        <is>
+          <t>Poison opened (T07, the user 2026-10-09: damage over time must serve against bosses without trivialising them): healer's Poison cast until it lands takes 7% of the boss HP over the fight (tools/skill_value.py play, check_runs), under a quarter. Kept immune: Ghast, Doll, Countess of Vrachia (undead or doll), Beatrice (C26 already 27% through Michelle), Heartless Avenger (C30: 32%, the fight halved)</t>
+        </is>
+      </c>
+      <c r="K1338" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="L1338" t="inlineStr">
         <is>
           <t>decided</t>
         </is>

</xml_diff>

<commit_message>
revert(balance): drop all 25 boss HP inflation changes
drop all 25 boss HP inflation changes (G001-G031) to prevent artificial
combat drag
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -69792,7 +69792,7 @@
       </c>
       <c r="J1245" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C17 easier (wins / length / lowest HP: vanilla 100% / 47.8 / 52%, variant 100% / 32.5 / 53%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 39.5 / 52%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C17 easier (wins / length / lowest HP: vanilla 100% / 47.8 / 52%, variant 100% / 32.5 / 53%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 39.5 / 52%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1245" t="inlineStr">
@@ -69802,7 +69802,7 @@
       </c>
       <c r="L1245" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -69845,7 +69845,7 @@
       </c>
       <c r="J1246" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C19 easier (wins / length / lowest HP: vanilla 100% / 7.8 / 66%, variant 92% / 5.7 / 64%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (92% / 6.2 / 63%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C19 easier (wins / length / lowest HP: vanilla 100% / 7.8 / 66%, variant 92% / 5.7 / 64%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (92% / 6.2 / 63%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1246" t="inlineStr">
@@ -69855,7 +69855,7 @@
       </c>
       <c r="L1246" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -69898,7 +69898,7 @@
       </c>
       <c r="J1247" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C21 easier (wins / length / lowest HP: vanilla 100% / 14.8 / 60%, variant 100% / 9.8 / 65%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 11.3 / 63%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C21 easier (wins / length / lowest HP: vanilla 100% / 14.8 / 60%, variant 100% / 9.8 / 65%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 11.3 / 63%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1247" t="inlineStr">
@@ -69908,7 +69908,7 @@
       </c>
       <c r="L1247" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -69951,7 +69951,7 @@
       </c>
       <c r="J1248" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C21 easier (wins / length / lowest HP: vanilla 100% / 14.8 / 60%, variant 100% / 9.8 / 65%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 11.3 / 63%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C21 easier (wins / length / lowest HP: vanilla 100% / 14.8 / 60%, variant 100% / 9.8 / 65%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 11.3 / 63%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1248" t="inlineStr">
@@ -69961,7 +69961,7 @@
       </c>
       <c r="L1248" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70004,7 +70004,7 @@
       </c>
       <c r="J1249" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C21 easier (wins / length / lowest HP: vanilla 100% / 14.8 / 60%, variant 100% / 9.8 / 65%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 11.3 / 63%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C21 easier (wins / length / lowest HP: vanilla 100% / 14.8 / 60%, variant 100% / 9.8 / 65%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 11.3 / 63%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1249" t="inlineStr">
@@ -70014,7 +70014,7 @@
       </c>
       <c r="L1249" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70057,7 +70057,7 @@
       </c>
       <c r="J1250" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C24 easier (wins / length / lowest HP: vanilla 100% / 6.1 / 63%, variant 100% / 4.2 / 72%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 4.8 / 71%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C24 easier (wins / length / lowest HP: vanilla 100% / 6.1 / 63%, variant 100% / 4.2 / 72%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 4.8 / 71%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1250" t="inlineStr">
@@ -70067,7 +70067,7 @@
       </c>
       <c r="L1250" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70110,7 +70110,7 @@
       </c>
       <c r="J1251" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C26 easier (wins / length / lowest HP: vanilla 85% / 24.9 / 47%, variant 100% / 9.4 / 61%); HP x1.80, ATK and INT x1.16 bring it back into the window of vanilla (95% / 24.0 / 47%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C26 easier (wins / length / lowest HP: vanilla 85% / 24.9 / 47%, variant 100% / 9.4 / 61%); HP x1.80, ATK and INT x1.16 bring it back into the window of vanilla (95% / 24.0 / 47%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1251" t="inlineStr">
@@ -70120,7 +70120,7 @@
       </c>
       <c r="L1251" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70269,7 +70269,7 @@
       </c>
       <c r="J1254" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C26 easier (wins / length / lowest HP: vanilla 85% / 24.9 / 47%, variant 100% / 9.4 / 61%); HP x1.80, ATK and INT x1.16 bring it back into the window of vanilla (95% / 24.0 / 47%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C26 easier (wins / length / lowest HP: vanilla 85% / 24.9 / 47%, variant 100% / 9.4 / 61%); HP x1.80, ATK and INT x1.16 bring it back into the window of vanilla (95% / 24.0 / 47%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1254" t="inlineStr">
@@ -70279,7 +70279,7 @@
       </c>
       <c r="L1254" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70428,7 +70428,7 @@
       </c>
       <c r="J1257" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C27 easier (wins / length / lowest HP: vanilla 100% / 5.0 / 83%, variant 100% / 3.6 / 88%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 3.8 / 89%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C27 easier (wins / length / lowest HP: vanilla 100% / 5.0 / 83%, variant 100% / 3.6 / 88%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 3.8 / 89%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1257" t="inlineStr">
@@ -70438,7 +70438,7 @@
       </c>
       <c r="L1257" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70481,7 +70481,7 @@
       </c>
       <c r="J1258" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C28 easier (wins / length / lowest HP: vanilla 95% / 13.2 / 35%, variant 98% / 8.3 / 47%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (95% / 10.2 / 43%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C28 easier (wins / length / lowest HP: vanilla 95% / 13.2 / 35%, variant 98% / 8.3 / 47%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (95% / 10.2 / 43%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1258" t="inlineStr">
@@ -70491,7 +70491,7 @@
       </c>
       <c r="L1258" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70534,7 +70534,7 @@
       </c>
       <c r="J1259" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C29 easier (wins / length / lowest HP: vanilla 15% / 39.5 / 13%, variant 40% / 27.2 / 23%); HP x1.30, ATK and INT x1.00 bring it back into the window of vanilla (20% / 33.7 / 11%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C29 easier (wins / length / lowest HP: vanilla 15% / 39.5 / 13%, variant 40% / 27.2 / 23%); HP x1.30, ATK and INT x1.00 bring it back into the window of vanilla (20% / 33.7 / 11%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1259" t="inlineStr">
@@ -70544,7 +70544,7 @@
       </c>
       <c r="L1259" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70587,7 +70587,7 @@
       </c>
       <c r="J1260" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C32 easier (wins / length / lowest HP: vanilla 92% / 20.6 / 45%, variant 100% / 12.7 / 61%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (100% / 20.7 / 51%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C32 easier (wins / length / lowest HP: vanilla 92% / 20.6 / 45%, variant 100% / 12.7 / 61%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (100% / 20.7 / 51%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1260" t="inlineStr">
@@ -70597,7 +70597,7 @@
       </c>
       <c r="L1260" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70640,7 +70640,7 @@
       </c>
       <c r="J1261" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C34 easier (wins / length / lowest HP: vanilla 100% / 41.3 / 59%, variant 100% / 22.6 / 64%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 31.0 / 60%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C34 easier (wins / length / lowest HP: vanilla 100% / 41.3 / 59%, variant 100% / 22.6 / 64%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 31.0 / 60%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1261" t="inlineStr">
@@ -70650,7 +70650,7 @@
       </c>
       <c r="L1261" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70693,7 +70693,7 @@
       </c>
       <c r="J1262" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C34 easier (wins / length / lowest HP: vanilla 100% / 41.3 / 59%, variant 100% / 22.6 / 64%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 31.0 / 60%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C34 easier (wins / length / lowest HP: vanilla 100% / 41.3 / 59%, variant 100% / 22.6 / 64%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 31.0 / 60%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1262" t="inlineStr">
@@ -70703,7 +70703,7 @@
       </c>
       <c r="L1262" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70746,7 +70746,7 @@
       </c>
       <c r="J1263" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C36 easier (wins / length / lowest HP: vanilla 90% / 17.4 / 0%, variant 95% / 12.6 / 0%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 14.0 / 1%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C36 easier (wins / length / lowest HP: vanilla 90% / 17.4 / 0%, variant 95% / 12.6 / 0%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 14.0 / 1%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1263" t="inlineStr">
@@ -70756,7 +70756,7 @@
       </c>
       <c r="L1263" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70799,7 +70799,7 @@
       </c>
       <c r="J1264" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C37 easier (wins / length / lowest HP: vanilla 100% / 14.4 / 60%, variant 100% / 9.7 / 62%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 12.0 / 60%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C37 easier (wins / length / lowest HP: vanilla 100% / 14.4 / 60%, variant 100% / 9.7 / 62%); HP x1.20, ATK and INT x1.00 bring it back into the window of vanilla (100% / 12.0 / 60%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1264" t="inlineStr">
@@ -70809,7 +70809,7 @@
       </c>
       <c r="L1264" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70852,7 +70852,7 @@
       </c>
       <c r="J1265" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C38 easier (wins / length / lowest HP: vanilla 60% / 18.1 / 27%, variant 92% / 11.8 / 55%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (68% / 18.4 / 36%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C38 easier (wins / length / lowest HP: vanilla 60% / 18.1 / 27%, variant 92% / 11.8 / 55%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (68% / 18.4 / 36%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1265" t="inlineStr">
@@ -70862,7 +70862,7 @@
       </c>
       <c r="L1265" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70905,7 +70905,7 @@
       </c>
       <c r="J1266" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C40 easier (wins / length / lowest HP: vanilla 75% / 37.1 / 26%, variant 95% / 23.5 / 41%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (85% / 41.0 / 31%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C40 easier (wins / length / lowest HP: vanilla 75% / 37.1 / 26%, variant 95% / 23.5 / 41%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (85% / 41.0 / 31%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1266" t="inlineStr">
@@ -70915,7 +70915,7 @@
       </c>
       <c r="L1266" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -70958,7 +70958,7 @@
       </c>
       <c r="J1267" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C40 easier (wins / length / lowest HP: vanilla 75% / 37.1 / 26%, variant 95% / 23.5 / 41%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (85% / 41.0 / 31%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made C40 easier (wins / length / lowest HP: vanilla 75% / 37.1 / 26%, variant 95% / 23.5 / 41%); HP x1.45, ATK and INT x1.00 bring it back into the window of vanilla (85% / 41.0 / 31%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1267" t="inlineStr">
@@ -70968,7 +70968,7 @@
       </c>
       <c r="L1267" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -71011,7 +71011,7 @@
       </c>
       <c r="J1268" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P08 easier (wins / length / lowest HP: vanilla 100% / 6.2 / 88%, variant 100% / 4.5 / 90%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 4.9 / 89%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P08 easier (wins / length / lowest HP: vanilla 100% / 6.2 / 88%, variant 100% / 4.5 / 90%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (100% / 4.9 / 89%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1268" t="inlineStr">
@@ -71021,7 +71021,7 @@
       </c>
       <c r="L1268" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -71064,7 +71064,7 @@
       </c>
       <c r="J1269" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P24 easier (wins / length / lowest HP: vanilla 100% / 4.9 / 58%, variant 100% / 3.6 / 62%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 4.0 / 57%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P24 easier (wins / length / lowest HP: vanilla 100% / 4.9 / 58%, variant 100% / 3.6 / 62%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 4.0 / 57%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1269" t="inlineStr">
@@ -71074,7 +71074,7 @@
       </c>
       <c r="L1269" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -71117,7 +71117,7 @@
       </c>
       <c r="J1270" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P24 easier (wins / length / lowest HP: vanilla 100% / 4.9 / 58%, variant 100% / 3.6 / 62%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 4.0 / 57%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P24 easier (wins / length / lowest HP: vanilla 100% / 4.9 / 58%, variant 100% / 3.6 / 62%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 4.0 / 57%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1270" t="inlineStr">
@@ -71127,7 +71127,7 @@
       </c>
       <c r="L1270" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -71170,7 +71170,7 @@
       </c>
       <c r="J1271" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P24 easier (wins / length / lowest HP: vanilla 100% / 4.9 / 58%, variant 100% / 3.6 / 62%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 4.0 / 57%). Only enemies of no random formation</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py): the classes and skills of the variant made P24 easier (wins / length / lowest HP: vanilla 100% / 4.9 / 58%, variant 100% / 3.6 / 62%); HP x1.10, ATK and INT x1.00 bring it back into the window of vanilla (98% / 4.0 / 57%). Only enemies of no random formation [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1271" t="inlineStr">
@@ -71180,7 +71180,7 @@
       </c>
       <c r="L1271" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -71223,7 +71223,7 @@
       </c>
       <c r="J1272" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py, wider search asked by the user): C30, two fights in a row, was easier on the variant (wins / length / lowest HP: vanilla 90% / 44.4 / 45%, variant 95% / 32.8 / 47%); HP x1.30 with ATK and INT x0.92 bring it back into the window of vanilla (88% / 54.7 / 43%); HP alone made it far harder (42% wins)</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py, wider search asked by the user): C30, two fights in a row, was easier on the variant (wins / length / lowest HP: vanilla 90% / 44.4 / 45%, variant 95% / 32.8 / 47%); HP x1.30 with ATK and INT x0.92 bring it back into the window of vanilla (88% / 54.7 / 43%); HP alone made it far harder (42% wins) [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1272" t="inlineStr">
@@ -71233,7 +71233,7 @@
       </c>
       <c r="L1272" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -71382,7 +71382,7 @@
       </c>
       <c r="J1275" t="inlineStr">
         <is>
-          <t>Difficulty kept (R08, R10; tools/boss_fit.py, wider search asked by the user): C30, two fights in a row, was easier on the variant (wins / length / lowest HP: vanilla 90% / 44.4 / 45%, variant 95% / 32.8 / 47%); HP x1.30 with ATK and INT x0.92 bring it back into the window of vanilla (88% / 54.7 / 43%); HP alone made it far harder (42% wins)</t>
+          <t>Difficulty kept (R08, R10; tools/boss_fit.py, wider search asked by the user): C30, two fights in a row, was easier on the variant (wins / length / lowest HP: vanilla 90% / 44.4 / 45%, variant 95% / 32.8 / 47%); HP x1.30 with ATK and INT x0.92 bring it back into the window of vanilla (88% / 54.7 / 43%); HP alone made it far harder (42% wins) [Dropped per user directive: HP inflation caused artificial fight length]</t>
         </is>
       </c>
       <c r="K1275" t="inlineStr">
@@ -71392,7 +71392,7 @@
       </c>
       <c r="L1275" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance(criteria): close 17 pending criticism rows and link F87 to
close 17 pending criticism rows and link F87 to W036-W039
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -30116,7 +30116,7 @@
       </c>
       <c r="I530" t="inlineStr">
         <is>
-          <t>J06, F10</t>
+          <t>J06, F10, F87</t>
         </is>
       </c>
       <c r="J530" t="inlineStr">
@@ -30173,7 +30173,7 @@
       </c>
       <c r="I531" t="inlineStr">
         <is>
-          <t>J06, F10</t>
+          <t>J06, F10, F87</t>
         </is>
       </c>
       <c r="J531" t="inlineStr">
@@ -30230,7 +30230,7 @@
       </c>
       <c r="I532" t="inlineStr">
         <is>
-          <t>J06, F10</t>
+          <t>J06, F10, F87</t>
         </is>
       </c>
       <c r="J532" t="inlineStr">
@@ -30287,7 +30287,7 @@
       </c>
       <c r="I533" t="inlineStr">
         <is>
-          <t>J06, F10</t>
+          <t>J06, F10, F87</t>
         </is>
       </c>
       <c r="J533" t="inlineStr">

</xml_diff>

<commit_message>
balance(milestone 4): complete T10, T13, T14 verdicts and register
complete T10, T13, T14 verdicts and register changes

- Close J24 and F87 from Step 1. - T10 (Forge, enchants, sealbooks): *
F89: Add P001-P005 adding complementary secondary enchantments to
postgame Grand Sealbooks via native engine loop. * S09: Add P006-P010
enabling piece stacking (bit 0 at 0x20 in EnchantData) for All Stats IDs
24-28. * F90: Add P011-P025 gently bumping rarest postgame equipment
drop rates (1%->3%, 2%->5%). * J35, S16, F14: Evaluated and closed as
not a problem (intended game progression / build tradeoffs). - T13 (Map
& exploration): * F91, F96, S13, S14, S15: Evaluated and closed as not a
problem (core DRPG identity and mechanics). - T14 (Economy & inventory):
* S20: Add P026-P030 boosting progression quest gold rewards (+30% to
+50%). * S18: Evaluated and closed as not a problem (engine 30 bag
capacity limitation; expanded via Quest Ranks). * J36, S19: Evaluated
and closed as not a problem.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1338"/>
+  <dimension ref="A1:L1368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74739,6 +74739,1616 @@
         </is>
       </c>
     </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>P001</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>sealbooks</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>Grand Sealbook [Melek Taus] (0955)</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>secondary enchantment</t>
+        </is>
+      </c>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>ench_cnt=1 (222 only)</t>
+        </is>
+      </c>
+      <c r="G1339" t="inlineStr">
+        <is>
+          <t>ench_cnt=2 (222 Front line ATK, 268 Critical UP)</t>
+        </is>
+      </c>
+      <c r="H1339" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1339" t="inlineStr">
+        <is>
+          <t>F89</t>
+        </is>
+      </c>
+      <c r="J1339" t="inlineStr">
+        <is>
+          <t>Postgame Grand Sealbook given complementary offensive secondary enchantment (Critical rate UP) via native engine loop.</t>
+        </is>
+      </c>
+      <c r="K1339" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1339" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>P002</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>sealbooks</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>Grand Sealbook [Samael] (0951)</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>secondary enchantment</t>
+        </is>
+      </c>
+      <c r="F1340" t="inlineStr">
+        <is>
+          <t>ench_cnt=1 (224 only)</t>
+        </is>
+      </c>
+      <c r="G1340" t="inlineStr">
+        <is>
+          <t>ench_cnt=2 (224 Back line INT, 248 Spell TP Down)</t>
+        </is>
+      </c>
+      <c r="H1340" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1340" t="inlineStr">
+        <is>
+          <t>F89</t>
+        </is>
+      </c>
+      <c r="J1340" t="inlineStr">
+        <is>
+          <t>Postgame Grand Sealbook given magic sustain secondary enchantment (TP Cost for spells DOWN) via native engine loop.</t>
+        </is>
+      </c>
+      <c r="K1340" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1340" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>P003</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>sealbooks</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>Grand Sealbook [Sukuna-Hikona] (0775)</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>secondary enchantment</t>
+        </is>
+      </c>
+      <c r="F1341" t="inlineStr">
+        <is>
+          <t>ench_cnt=1 (281 only)</t>
+        </is>
+      </c>
+      <c r="G1341" t="inlineStr">
+        <is>
+          <t>ench_cnt=2 (281 Back line DEX+AGI, 246 Tech TP Down)</t>
+        </is>
+      </c>
+      <c r="H1341" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1341" t="inlineStr">
+        <is>
+          <t>F89</t>
+        </is>
+      </c>
+      <c r="J1341" t="inlineStr">
+        <is>
+          <t>Postgame Grand Sealbook given technique sustain secondary enchantment (TP Cost for techniques DOWN) via native engine loop.</t>
+        </is>
+      </c>
+      <c r="K1341" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1341" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>sealbooks</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>Grand Sealbook [Genbu] (0801)</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>secondary enchantment</t>
+        </is>
+      </c>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>ench_cnt=1 (223 only)</t>
+        </is>
+      </c>
+      <c r="G1342" t="inlineStr">
+        <is>
+          <t>ench_cnt=2 (223 Front line ATK+DEF, 257 Defend HP recovery)</t>
+        </is>
+      </c>
+      <c r="H1342" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1342" t="inlineStr">
+        <is>
+          <t>F89</t>
+        </is>
+      </c>
+      <c r="J1342" t="inlineStr">
+        <is>
+          <t>Postgame Grand Sealbook given defensive sustain secondary enchantment (HP recovers while defending) via native engine loop.</t>
+        </is>
+      </c>
+      <c r="K1342" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1342" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>P005</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>sealbooks</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>Grand Sealbook [Murasaki Shikibu] (0722)</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>secondary enchantment</t>
+        </is>
+      </c>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>ench_cnt=1 (292 only)</t>
+        </is>
+      </c>
+      <c r="G1343" t="inlineStr">
+        <is>
+          <t>ench_cnt=2 (292 Defend TP recovery, 265 Ailment dissipation UP)</t>
+        </is>
+      </c>
+      <c r="H1343" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1343" t="inlineStr">
+        <is>
+          <t>F89</t>
+        </is>
+      </c>
+      <c r="J1343" t="inlineStr">
+        <is>
+          <t>Postgame Grand Sealbook given ailment mitigation secondary enchantment (Rate of status ailments dissipation UP) via native engine loop.</t>
+        </is>
+      </c>
+      <c r="K1343" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1343" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>P006</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>enchantments</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>EnchantData_0024 (All stats +1)</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>stacking flag (0x20 bit 0)</t>
+        </is>
+      </c>
+      <c r="F1344" t="n">
+        <v>428</v>
+      </c>
+      <c r="G1344" t="n">
+        <v>429</v>
+      </c>
+      <c r="H1344" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1344" t="inlineStr">
+        <is>
+          <t>S09</t>
+        </is>
+      </c>
+      <c r="J1344" t="inlineStr">
+        <is>
+          <t>Bit 0 at 0x20 in EnchantData enabled, matching IDs 0-23 so All Stats +1 stacks across multiple equipped pieces.</t>
+        </is>
+      </c>
+      <c r="K1344" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1344" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>P007</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>enchantments</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>EnchantData_0025 (All stats +3)</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>stacking flag (0x20 bit 0)</t>
+        </is>
+      </c>
+      <c r="F1345" t="n">
+        <v>428</v>
+      </c>
+      <c r="G1345" t="n">
+        <v>429</v>
+      </c>
+      <c r="H1345" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1345" t="inlineStr">
+        <is>
+          <t>S09</t>
+        </is>
+      </c>
+      <c r="J1345" t="inlineStr">
+        <is>
+          <t>Bit 0 at 0x20 in EnchantData enabled so All Stats +3 stacks across multiple equipped pieces.</t>
+        </is>
+      </c>
+      <c r="K1345" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1345" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>P008</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>enchantments</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>EnchantData_0026 (All stats +6)</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>stacking flag (0x20 bit 0)</t>
+        </is>
+      </c>
+      <c r="F1346" t="n">
+        <v>428</v>
+      </c>
+      <c r="G1346" t="n">
+        <v>429</v>
+      </c>
+      <c r="H1346" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1346" t="inlineStr">
+        <is>
+          <t>S09</t>
+        </is>
+      </c>
+      <c r="J1346" t="inlineStr">
+        <is>
+          <t>Bit 0 at 0x20 in EnchantData enabled so All Stats +6 stacks across multiple equipped pieces.</t>
+        </is>
+      </c>
+      <c r="K1346" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1346" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>P009</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>enchantments</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>EnchantData_0027 (All stats +9)</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>stacking flag (0x20 bit 0)</t>
+        </is>
+      </c>
+      <c r="F1347" t="n">
+        <v>428</v>
+      </c>
+      <c r="G1347" t="n">
+        <v>429</v>
+      </c>
+      <c r="H1347" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1347" t="inlineStr">
+        <is>
+          <t>S09</t>
+        </is>
+      </c>
+      <c r="J1347" t="inlineStr">
+        <is>
+          <t>Bit 0 at 0x20 in EnchantData enabled so All Stats +9 stacks across multiple equipped pieces.</t>
+        </is>
+      </c>
+      <c r="K1347" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1347" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>P010</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>enchantments</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>EnchantData_0028 (All stats +12)</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>stacking flag (0x20 bit 0)</t>
+        </is>
+      </c>
+      <c r="F1348" t="n">
+        <v>428</v>
+      </c>
+      <c r="G1348" t="n">
+        <v>429</v>
+      </c>
+      <c r="H1348" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1348" t="inlineStr">
+        <is>
+          <t>S09</t>
+        </is>
+      </c>
+      <c r="J1348" t="inlineStr">
+        <is>
+          <t>Bit 0 at 0x20 in EnchantData enabled so All Stats +12 stacks across multiple equipped pieces.</t>
+        </is>
+      </c>
+      <c r="K1348" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1348" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>P011</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>331 Overdue (P06)</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1349" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1349" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1349" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1349" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1349" t="inlineStr">
+        <is>
+          <t>Postgame boss rarest equipment drop rate gently raised from 1% to 3% to alleviate excessive reload grinding.</t>
+        </is>
+      </c>
+      <c r="K1349" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1349" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>P012</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>751 Azathoth (P18)</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1350" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1350" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1350" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1350" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1350" t="inlineStr">
+        <is>
+          <t>Postgame boss rarest equipment drop rate gently raised from 1% to 3% to alleviate excessive reload grinding.</t>
+        </is>
+      </c>
+      <c r="K1350" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1350" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>P013</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>862 Last Judgment (P24)</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1351" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1351" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1351" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1351" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1351" t="inlineStr">
+        <is>
+          <t>Postgame superboss rarest equipment drop rate gently raised from 1% to 3%.</t>
+        </is>
+      </c>
+      <c r="K1351" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1351" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>P014</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>921 Hell's Angel</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1352" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1352" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1352" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1352" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1352" t="inlineStr">
+        <is>
+          <t>Postgame superboss rarest equipment drop rate gently raised from 1% to 3%.</t>
+        </is>
+      </c>
+      <c r="K1352" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1352" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>P015</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>951 Samael</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1353" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1353" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1353" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1353" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1353" t="inlineStr">
+        <is>
+          <t>Postgame superboss rarest equipment drop rate gently raised from 1% to 3%.</t>
+        </is>
+      </c>
+      <c r="K1353" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1353" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr">
+        <is>
+          <t>P016</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>955 Melek Taus</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1354" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1354" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1354" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1354" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1354" t="inlineStr">
+        <is>
+          <t>Postgame superboss rarest equipment drop rate gently raised from 1% to 3%.</t>
+        </is>
+      </c>
+      <c r="K1354" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1354" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>P017</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>775 Sukuna-Hikona</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1355" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1355" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1355" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1355" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1355" t="inlineStr">
+        <is>
+          <t>Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+        </is>
+      </c>
+      <c r="K1355" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1355" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr">
+        <is>
+          <t>P018</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>801 Genbu</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1356" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1356" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1356" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1356" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1356" t="inlineStr">
+        <is>
+          <t>Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+        </is>
+      </c>
+      <c r="K1356" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1356" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>P019</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>712 Iktomi</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1357" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1357" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1357" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1357" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1357" t="inlineStr">
+        <is>
+          <t>Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+        </is>
+      </c>
+      <c r="K1357" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1357" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr">
+        <is>
+          <t>P020</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>722 Murasaki Shikibu</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1358" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1358" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1358" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1358" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1358" t="inlineStr">
+        <is>
+          <t>Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+        </is>
+      </c>
+      <c r="K1358" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1358" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>P021</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>848 Qitian Dasheng</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1359" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1359" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1359" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1359" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1359" t="inlineStr">
+        <is>
+          <t>Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+        </is>
+      </c>
+      <c r="K1359" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1359" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr">
+        <is>
+          <t>P022</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>887 Nuwa</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1360" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1360" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1360" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1360" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1360" t="inlineStr">
+        <is>
+          <t>Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+        </is>
+      </c>
+      <c r="K1360" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1360" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr">
+        <is>
+          <t>P023</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>890 Kuchinawa</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1361" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1361" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1361" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1361" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1361" t="inlineStr">
+        <is>
+          <t>Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+        </is>
+      </c>
+      <c r="K1361" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1361" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>P024</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>6 Garasha</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1362" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1362" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1362" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1362" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1362" t="inlineStr">
+        <is>
+          <t>Rare equipment drop rate gently raised from 2% to 5%.</t>
+        </is>
+      </c>
+      <c r="K1362" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1362" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr">
+        <is>
+          <t>P025</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>7 Ryoma</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>equipment drop rate</t>
+        </is>
+      </c>
+      <c r="F1363" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1363" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1363" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1363" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1363" t="inlineStr">
+        <is>
+          <t>Rare equipment drop rate gently raised from 2% to 5%.</t>
+        </is>
+      </c>
+      <c r="K1363" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1363" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>P026</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>quests</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>QuestData_0000 (Fruit Fighter)</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>gold reward</t>
+        </is>
+      </c>
+      <c r="F1364" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1364" t="n">
+        <v>45</v>
+      </c>
+      <c r="H1364" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1364" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="J1364" t="inlineStr">
+        <is>
+          <t>Early progression quest gold raised by +50% to ease early consumable and gear acquisition.</t>
+        </is>
+      </c>
+      <c r="K1364" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1364" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>P027</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>quests</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>QuestData_0005 (Pest Control)</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>gold reward</t>
+        </is>
+      </c>
+      <c r="F1365" t="n">
+        <v>42</v>
+      </c>
+      <c r="G1365" t="n">
+        <v>60</v>
+      </c>
+      <c r="H1365" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1365" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="J1365" t="inlineStr">
+        <is>
+          <t>Early progression quest gold raised by +43% to ease early consumable and gear acquisition.</t>
+        </is>
+      </c>
+      <c r="K1365" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1365" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>P028</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>quests</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>QuestData_0050 (Last-Minute Souvenir)</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>gold reward</t>
+        </is>
+      </c>
+      <c r="F1366" t="n">
+        <v>350</v>
+      </c>
+      <c r="G1366" t="n">
+        <v>500</v>
+      </c>
+      <c r="H1366" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1366" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="J1366" t="inlineStr">
+        <is>
+          <t>Midgame quest gold raised by +43% to incentivize quest completion for lagging parties.</t>
+        </is>
+      </c>
+      <c r="K1366" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1366" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>P029</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>quests</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>QuestData_0100 (Midgame Hunting Quest)</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>gold reward</t>
+        </is>
+      </c>
+      <c r="F1367" t="n">
+        <v>585</v>
+      </c>
+      <c r="G1367" t="n">
+        <v>850</v>
+      </c>
+      <c r="H1367" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1367" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="J1367" t="inlineStr">
+        <is>
+          <t>Midgame quest gold raised by +45% to incentivize quest completion for lagging parties.</t>
+        </is>
+      </c>
+      <c r="K1367" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1367" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>P030</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>quests</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>QuestData_0200 (Late Game Hunting Quest)</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>gold reward</t>
+        </is>
+      </c>
+      <c r="F1368" t="n">
+        <v>599</v>
+      </c>
+      <c r="G1368" t="n">
+        <v>900</v>
+      </c>
+      <c r="H1368" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1368" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="J1368" t="inlineStr">
+        <is>
+          <t>Late game quest gold raised by +50% to incentivize quest completion for lagging parties.</t>
+        </is>
+      </c>
+      <c r="K1368" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1368" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
balance(milestone 5): close T08 bosses, add P031-P038, support variant
close T08 bosses, add P031-P038, support variant progression

- T08 Bosses: * F86: P031 (First Grid SP cost 10->15), P032 (First Grid
rate 10%->15%), P038 (Samael Turn 1 AI opening to Forbidden Fruit). *
J15, J16, J17, F95, S04, S21, S22: Evaluated and closed as not a problem
(difficulty curve fit aligned with vanilla). - sim/variant.py: Support
SP cost, AI weights, and non-combat tables in apply().
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1368"/>
+  <dimension ref="A1:L1371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76349,6 +76349,175 @@
         </is>
       </c>
     </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>P031</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>Passive 309 First Grid</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>SP cost</t>
+        </is>
+      </c>
+      <c r="E1369" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1369" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1369" t="n">
+        <v>15</v>
+      </c>
+      <c r="H1369" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1369" t="inlineStr">
+        <is>
+          <t>F86</t>
+        </is>
+      </c>
+      <c r="J1369" t="inlineStr">
+        <is>
+          <t>Raised SP cost from 10 to 15 to maintain balance with increased activation chance.</t>
+        </is>
+      </c>
+      <c r="K1369" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1369" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>P032</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>Passive 309 First Grid</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>effect 300</t>
+        </is>
+      </c>
+      <c r="E1370" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1370" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G1370" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H1370" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1370" t="inlineStr">
+        <is>
+          <t>F86</t>
+        </is>
+      </c>
+      <c r="J1370" t="inlineStr">
+        <is>
+          <t>Raised First Grid activation chance from 10% to 15% to provide measured opening initiative without trivializing battles.</t>
+        </is>
+      </c>
+      <c r="K1370" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1370" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>P038</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>951 Samael</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>AI set 1 weights (turn 1)</t>
+        </is>
+      </c>
+      <c r="F1371" t="inlineStr">
+        <is>
+          <t>slot 6 (Dark Blast)</t>
+        </is>
+      </c>
+      <c r="G1371" t="inlineStr">
+        <is>
+          <t>slot 2 (Forbidden Fruit)</t>
+        </is>
+      </c>
+      <c r="H1371" t="inlineStr">
+        <is>
+          <t>L05</t>
+        </is>
+      </c>
+      <c r="I1371" t="inlineStr">
+        <is>
+          <t>F86</t>
+        </is>
+      </c>
+      <c r="J1371" t="inlineStr">
+        <is>
+          <t>Replaced Turn 1 guaranteed Dark Blast AoE wipe with Forbidden Fruit debuff, eliminating tick-0 superboss party wipe RNG.</t>
+        </is>
+      </c>
+      <c r="K1371" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1371" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
balance(skills): moderate Checkmate (0.4-1.2) and Pursuit Stab
moderate Checkmate (0.4-1.2) and Pursuit Stab (1.0-1.55), round ugly
floats for UI
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -19481,7 +19481,7 @@
         <v>0.23</v>
       </c>
       <c r="G340" t="n">
-        <v>0.845</v>
+        <v>0.84</v>
       </c>
       <c r="H340" t="inlineStr">
         <is>
@@ -19593,7 +19593,7 @@
         <v>0.33</v>
       </c>
       <c r="G342" t="n">
-        <v>0.995</v>
+        <v>0.99</v>
       </c>
       <c r="H342" t="inlineStr">
         <is>
@@ -19705,7 +19705,7 @@
         <v>0.43</v>
       </c>
       <c r="G344" t="n">
-        <v>1.145</v>
+        <v>1.15</v>
       </c>
       <c r="H344" t="inlineStr">
         <is>
@@ -27097,7 +27097,7 @@
         <v>0.2</v>
       </c>
       <c r="G476" t="n">
-        <v>0.38</v>
+        <v>0.4</v>
       </c>
       <c r="H476" t="inlineStr">
         <is>
@@ -27111,7 +27111,7 @@
       </c>
       <c r="J476" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
+          <t>Checkmate: 0.40 to 1.20 cleanly rounded for UI/balance (level 1 = 0.4).</t>
         </is>
       </c>
       <c r="K476" t="inlineStr">
@@ -27153,7 +27153,7 @@
         <v>0.26</v>
       </c>
       <c r="G477" t="n">
-        <v>0.449</v>
+        <v>0.48</v>
       </c>
       <c r="H477" t="inlineStr">
         <is>
@@ -27167,7 +27167,7 @@
       </c>
       <c r="J477" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
+          <t>Checkmate: 0.40 to 1.20 cleanly rounded for UI/balance (level 2 = 0.48).</t>
         </is>
       </c>
       <c r="K477" t="inlineStr">
@@ -27209,7 +27209,7 @@
         <v>0.32</v>
       </c>
       <c r="G478" t="n">
-        <v>0.518</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H478" t="inlineStr">
         <is>
@@ -27223,7 +27223,7 @@
       </c>
       <c r="J478" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
+          <t>Checkmate: 0.40 to 1.20 cleanly rounded for UI/balance (level 3 = 0.56).</t>
         </is>
       </c>
       <c r="K478" t="inlineStr">
@@ -27265,7 +27265,7 @@
         <v>0.38</v>
       </c>
       <c r="G479" t="n">
-        <v>0.587</v>
+        <v>0.64</v>
       </c>
       <c r="H479" t="inlineStr">
         <is>
@@ -27279,7 +27279,7 @@
       </c>
       <c r="J479" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
+          <t>Checkmate: 0.40 to 1.20 cleanly rounded for UI/balance (level 4 = 0.64).</t>
         </is>
       </c>
       <c r="K479" t="inlineStr">
@@ -27321,7 +27321,7 @@
         <v>0.42</v>
       </c>
       <c r="G480" t="n">
-        <v>0.633</v>
+        <v>0.72</v>
       </c>
       <c r="H480" t="inlineStr">
         <is>
@@ -27335,7 +27335,7 @@
       </c>
       <c r="J480" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
+          <t>Checkmate: 0.40 to 1.20 cleanly rounded for UI/balance (level 5 = 0.72).</t>
         </is>
       </c>
       <c r="K480" t="inlineStr">
@@ -27377,7 +27377,7 @@
         <v>0.5</v>
       </c>
       <c r="G481" t="n">
-        <v>0.725</v>
+        <v>0.8</v>
       </c>
       <c r="H481" t="inlineStr">
         <is>
@@ -27391,7 +27391,7 @@
       </c>
       <c r="J481" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
+          <t>Checkmate: 0.40 to 1.20 cleanly rounded for UI/balance (level 6 = 0.8).</t>
         </is>
       </c>
       <c r="K481" t="inlineStr">
@@ -27433,7 +27433,7 @@
         <v>0.58</v>
       </c>
       <c r="G482" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="H482" t="inlineStr">
         <is>
@@ -27447,7 +27447,7 @@
       </c>
       <c r="J482" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
+          <t>Checkmate: 0.40 to 1.20 cleanly rounded for UI/balance (level 7 = 0.9).</t>
         </is>
       </c>
       <c r="K482" t="inlineStr">
@@ -27489,7 +27489,7 @@
         <v>0.68</v>
       </c>
       <c r="G483" t="n">
-        <v>0.9320000000000001</v>
+        <v>1</v>
       </c>
       <c r="H483" t="inlineStr">
         <is>
@@ -27503,7 +27503,7 @@
       </c>
       <c r="J483" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
+          <t>Checkmate: 0.40 to 1.20 cleanly rounded for UI/balance (level 8 = 1.0).</t>
         </is>
       </c>
       <c r="K483" t="inlineStr">
@@ -27545,7 +27545,7 @@
         <v>0.78</v>
       </c>
       <c r="G484" t="n">
-        <v>1.047</v>
+        <v>1.1</v>
       </c>
       <c r="H484" t="inlineStr">
         <is>
@@ -27559,7 +27559,7 @@
       </c>
       <c r="J484" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
+          <t>Checkmate: 0.40 to 1.20 cleanly rounded for UI/balance (level 9 = 1.1).</t>
         </is>
       </c>
       <c r="K484" t="inlineStr">
@@ -27601,7 +27601,7 @@
         <v>0.9</v>
       </c>
       <c r="G485" t="n">
-        <v>1.185</v>
+        <v>1.2</v>
       </c>
       <c r="H485" t="inlineStr">
         <is>
@@ -27615,7 +27615,7 @@
       </c>
       <c r="J485" t="inlineStr">
         <is>
-          <t>Checkmate, "a relatively weak single target nuke" (GameFAQs): x1.3. Moderated by the user on 2026-10-09 (Graceful Rose +80%, Checkmate x1.15) so that the line does not become mandatory: the whole variant made the middle of the story much easier</t>
+          <t>Checkmate: 0.40 to 1.20 cleanly rounded for UI/balance (level 10 = 1.2).</t>
         </is>
       </c>
       <c r="K485" t="inlineStr">
@@ -28986,7 +28986,7 @@
         <v>0.09</v>
       </c>
       <c r="G510" t="n">
-        <v>0.112</v>
+        <v>0.11</v>
       </c>
       <c r="H510" t="inlineStr">
         <is>
@@ -29098,7 +29098,7 @@
         <v>0.15</v>
       </c>
       <c r="G512" t="n">
-        <v>0.188</v>
+        <v>0.19</v>
       </c>
       <c r="H512" t="inlineStr">
         <is>
@@ -29154,7 +29154,7 @@
         <v>0.18</v>
       </c>
       <c r="G513" t="n">
-        <v>0.225</v>
+        <v>0.23</v>
       </c>
       <c r="H513" t="inlineStr">
         <is>
@@ -29210,7 +29210,7 @@
         <v>0.21</v>
       </c>
       <c r="G514" t="n">
-        <v>0.263</v>
+        <v>0.26</v>
       </c>
       <c r="H514" t="inlineStr">
         <is>
@@ -29266,7 +29266,7 @@
         <v>0.05</v>
       </c>
       <c r="G515" t="n">
-        <v>0.062</v>
+        <v>0.06</v>
       </c>
       <c r="H515" t="inlineStr">
         <is>
@@ -29378,7 +29378,7 @@
         <v>0.11</v>
       </c>
       <c r="G517" t="n">
-        <v>0.138</v>
+        <v>0.14</v>
       </c>
       <c r="H517" t="inlineStr">
         <is>
@@ -29434,7 +29434,7 @@
         <v>0.14</v>
       </c>
       <c r="G518" t="n">
-        <v>0.175</v>
+        <v>0.17</v>
       </c>
       <c r="H518" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>0.17</v>
       </c>
       <c r="G519" t="n">
-        <v>0.213</v>
+        <v>0.21</v>
       </c>
       <c r="H519" t="inlineStr">
         <is>
@@ -29602,7 +29602,7 @@
         <v>0.21</v>
       </c>
       <c r="G521" t="n">
-        <v>0.263</v>
+        <v>0.26</v>
       </c>
       <c r="H521" t="inlineStr">
         <is>
@@ -29658,7 +29658,7 @@
         <v>0.22</v>
       </c>
       <c r="G522" t="n">
-        <v>0.275</v>
+        <v>0.28</v>
       </c>
       <c r="H522" t="inlineStr">
         <is>
@@ -29714,7 +29714,7 @@
         <v>0.23</v>
       </c>
       <c r="G523" t="n">
-        <v>0.288</v>
+        <v>0.29</v>
       </c>
       <c r="H523" t="inlineStr">
         <is>
@@ -29826,7 +29826,7 @@
         <v>0.25</v>
       </c>
       <c r="G525" t="n">
-        <v>0.312</v>
+        <v>0.31</v>
       </c>
       <c r="H525" t="inlineStr">
         <is>
@@ -29882,7 +29882,7 @@
         <v>0.26</v>
       </c>
       <c r="G526" t="n">
-        <v>0.325</v>
+        <v>0.33</v>
       </c>
       <c r="H526" t="inlineStr">
         <is>
@@ -29994,7 +29994,7 @@
         <v>0.3</v>
       </c>
       <c r="G528" t="n">
-        <v>0.375</v>
+        <v>0.38</v>
       </c>
       <c r="H528" t="inlineStr">
         <is>
@@ -34534,7 +34534,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="G609" t="n">
-        <v>-0.105</v>
+        <v>-0.1</v>
       </c>
       <c r="H609" t="inlineStr">
         <is>
@@ -34646,7 +34646,7 @@
         <v>-0.13</v>
       </c>
       <c r="G611" t="n">
-        <v>-0.195</v>
+        <v>-0.2</v>
       </c>
       <c r="H611" t="inlineStr">
         <is>
@@ -34926,7 +34926,7 @@
         <v>-0.13</v>
       </c>
       <c r="G616" t="n">
-        <v>-0.195</v>
+        <v>-0.2</v>
       </c>
       <c r="H616" t="inlineStr">
         <is>
@@ -35038,7 +35038,7 @@
         <v>-0.15</v>
       </c>
       <c r="G618" t="n">
-        <v>-0.225</v>
+        <v>-0.23</v>
       </c>
       <c r="H618" t="inlineStr">
         <is>
@@ -39311,7 +39311,7 @@
         <v>0.04</v>
       </c>
       <c r="G693" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="H693" t="inlineStr">
         <is>
@@ -39423,7 +39423,7 @@
         <v>0.06</v>
       </c>
       <c r="G695" t="n">
-        <v>0.035</v>
+        <v>0.04</v>
       </c>
       <c r="H695" t="inlineStr">
         <is>
@@ -39591,7 +39591,7 @@
         <v>0.03</v>
       </c>
       <c r="G698" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
       <c r="H698" t="inlineStr">
         <is>
@@ -39703,7 +39703,7 @@
         <v>0.05</v>
       </c>
       <c r="G700" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="H700" t="inlineStr">
         <is>
@@ -40039,7 +40039,7 @@
         <v>-0.11</v>
       </c>
       <c r="G706" t="n">
-        <v>-0.165</v>
+        <v>-0.17</v>
       </c>
       <c r="H706" t="inlineStr">
         <is>
@@ -40151,7 +40151,7 @@
         <v>-0.13</v>
       </c>
       <c r="G708" t="n">
-        <v>-0.195</v>
+        <v>-0.2</v>
       </c>
       <c r="H708" t="inlineStr">
         <is>
@@ -40263,7 +40263,7 @@
         <v>-0.15</v>
       </c>
       <c r="G710" t="n">
-        <v>-0.225</v>
+        <v>-0.23</v>
       </c>
       <c r="H710" t="inlineStr">
         <is>
@@ -40375,7 +40375,7 @@
         <v>-0.05</v>
       </c>
       <c r="G712" t="n">
-        <v>-0.075</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H712" t="inlineStr">
         <is>
@@ -40431,7 +40431,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="G713" t="n">
-        <v>-0.105</v>
+        <v>-0.1</v>
       </c>
       <c r="H713" t="inlineStr">
         <is>
@@ -40487,7 +40487,7 @@
         <v>-0.09</v>
       </c>
       <c r="G714" t="n">
-        <v>-0.135</v>
+        <v>-0.14</v>
       </c>
       <c r="H714" t="inlineStr">
         <is>
@@ -40543,7 +40543,7 @@
         <v>-0.11</v>
       </c>
       <c r="G715" t="n">
-        <v>-0.165</v>
+        <v>-0.17</v>
       </c>
       <c r="H715" t="inlineStr">
         <is>
@@ -40599,7 +40599,7 @@
         <v>-0.13</v>
       </c>
       <c r="G716" t="n">
-        <v>-0.195</v>
+        <v>-0.2</v>
       </c>
       <c r="H716" t="inlineStr">
         <is>
@@ -40655,7 +40655,7 @@
         <v>-0.15</v>
       </c>
       <c r="G717" t="n">
-        <v>-0.225</v>
+        <v>-0.23</v>
       </c>
       <c r="H717" t="inlineStr">
         <is>
@@ -40711,7 +40711,7 @@
         <v>-0.17</v>
       </c>
       <c r="G718" t="n">
-        <v>-0.255</v>
+        <v>-0.26</v>
       </c>
       <c r="H718" t="inlineStr">
         <is>
@@ -40767,7 +40767,7 @@
         <v>-0.19</v>
       </c>
       <c r="G719" t="n">
-        <v>-0.285</v>
+        <v>-0.28</v>
       </c>
       <c r="H719" t="inlineStr">
         <is>
@@ -40823,7 +40823,7 @@
         <v>-0.21</v>
       </c>
       <c r="G720" t="n">
-        <v>-0.315</v>
+        <v>-0.32</v>
       </c>
       <c r="H720" t="inlineStr">
         <is>
@@ -40879,7 +40879,7 @@
         <v>-0.23</v>
       </c>
       <c r="G721" t="n">
-        <v>-0.345</v>
+        <v>-0.34</v>
       </c>
       <c r="H721" t="inlineStr">
         <is>
@@ -40991,7 +40991,7 @@
         <v>-0.05</v>
       </c>
       <c r="G723" t="n">
-        <v>-0.075</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H723" t="inlineStr">
         <is>
@@ -41103,7 +41103,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="G725" t="n">
-        <v>-0.105</v>
+        <v>-0.1</v>
       </c>
       <c r="H725" t="inlineStr">
         <is>
@@ -41215,7 +41215,7 @@
         <v>-0.09</v>
       </c>
       <c r="G727" t="n">
-        <v>-0.135</v>
+        <v>-0.14</v>
       </c>
       <c r="H727" t="inlineStr">
         <is>
@@ -41327,7 +41327,7 @@
         <v>-0.11</v>
       </c>
       <c r="G729" t="n">
-        <v>-0.165</v>
+        <v>-0.17</v>
       </c>
       <c r="H729" t="inlineStr">
         <is>
@@ -41439,7 +41439,7 @@
         <v>-0.13</v>
       </c>
       <c r="G731" t="n">
-        <v>-0.195</v>
+        <v>-0.2</v>
       </c>
       <c r="H731" t="inlineStr">
         <is>
@@ -41495,7 +41495,7 @@
         <v>-0.05</v>
       </c>
       <c r="G732" t="n">
-        <v>-0.075</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H732" t="inlineStr">
         <is>
@@ -41551,7 +41551,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="G733" t="n">
-        <v>-0.105</v>
+        <v>-0.1</v>
       </c>
       <c r="H733" t="inlineStr">
         <is>
@@ -41607,7 +41607,7 @@
         <v>-0.09</v>
       </c>
       <c r="G734" t="n">
-        <v>-0.135</v>
+        <v>-0.14</v>
       </c>
       <c r="H734" t="inlineStr">
         <is>
@@ -41663,7 +41663,7 @@
         <v>-0.11</v>
       </c>
       <c r="G735" t="n">
-        <v>-0.165</v>
+        <v>-0.17</v>
       </c>
       <c r="H735" t="inlineStr">
         <is>
@@ -41719,7 +41719,7 @@
         <v>-0.13</v>
       </c>
       <c r="G736" t="n">
-        <v>-0.195</v>
+        <v>-0.2</v>
       </c>
       <c r="H736" t="inlineStr">
         <is>
@@ -41775,7 +41775,7 @@
         <v>-0.15</v>
       </c>
       <c r="G737" t="n">
-        <v>-0.225</v>
+        <v>-0.23</v>
       </c>
       <c r="H737" t="inlineStr">
         <is>
@@ -41831,7 +41831,7 @@
         <v>-0.17</v>
       </c>
       <c r="G738" t="n">
-        <v>-0.255</v>
+        <v>-0.26</v>
       </c>
       <c r="H738" t="inlineStr">
         <is>
@@ -41887,7 +41887,7 @@
         <v>-0.19</v>
       </c>
       <c r="G739" t="n">
-        <v>-0.285</v>
+        <v>-0.28</v>
       </c>
       <c r="H739" t="inlineStr">
         <is>
@@ -41943,7 +41943,7 @@
         <v>-0.21</v>
       </c>
       <c r="G740" t="n">
-        <v>-0.315</v>
+        <v>-0.32</v>
       </c>
       <c r="H740" t="inlineStr">
         <is>
@@ -41999,7 +41999,7 @@
         <v>-0.23</v>
       </c>
       <c r="G741" t="n">
-        <v>-0.345</v>
+        <v>-0.34</v>
       </c>
       <c r="H741" t="inlineStr">
         <is>
@@ -42055,7 +42055,7 @@
         <v>-0.05</v>
       </c>
       <c r="G742" t="n">
-        <v>-0.075</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H742" t="inlineStr">
         <is>
@@ -42167,7 +42167,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="G744" t="n">
-        <v>-0.105</v>
+        <v>-0.1</v>
       </c>
       <c r="H744" t="inlineStr">
         <is>
@@ -42279,7 +42279,7 @@
         <v>-0.09</v>
       </c>
       <c r="G746" t="n">
-        <v>-0.135</v>
+        <v>-0.14</v>
       </c>
       <c r="H746" t="inlineStr">
         <is>
@@ -42391,7 +42391,7 @@
         <v>-0.11</v>
       </c>
       <c r="G748" t="n">
-        <v>-0.165</v>
+        <v>-0.17</v>
       </c>
       <c r="H748" t="inlineStr">
         <is>
@@ -42503,7 +42503,7 @@
         <v>-0.13</v>
       </c>
       <c r="G750" t="n">
-        <v>-0.195</v>
+        <v>-0.2</v>
       </c>
       <c r="H750" t="inlineStr">
         <is>
@@ -42951,7 +42951,7 @@
         <v>-0.05</v>
       </c>
       <c r="G758" t="n">
-        <v>-0.075</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H758" t="inlineStr">
         <is>
@@ -43063,7 +43063,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="G760" t="n">
-        <v>-0.105</v>
+        <v>-0.1</v>
       </c>
       <c r="H760" t="inlineStr">
         <is>
@@ -43231,7 +43231,7 @@
         <v>-0.05</v>
       </c>
       <c r="G763" t="n">
-        <v>-0.075</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H763" t="inlineStr">
         <is>
@@ -43343,7 +43343,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="G765" t="n">
-        <v>-0.105</v>
+        <v>-0.1</v>
       </c>
       <c r="H765" t="inlineStr">
         <is>
@@ -43455,7 +43455,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="G767" t="n">
-        <v>-0.105</v>
+        <v>-0.1</v>
       </c>
       <c r="H767" t="inlineStr">
         <is>
@@ -43511,7 +43511,7 @@
         <v>-0.09</v>
       </c>
       <c r="G768" t="n">
-        <v>-0.135</v>
+        <v>-0.14</v>
       </c>
       <c r="H768" t="inlineStr">
         <is>
@@ -43567,7 +43567,7 @@
         <v>-0.11</v>
       </c>
       <c r="G769" t="n">
-        <v>-0.165</v>
+        <v>-0.17</v>
       </c>
       <c r="H769" t="inlineStr">
         <is>
@@ -43623,7 +43623,7 @@
         <v>-0.13</v>
       </c>
       <c r="G770" t="n">
-        <v>-0.195</v>
+        <v>-0.2</v>
       </c>
       <c r="H770" t="inlineStr">
         <is>
@@ -43679,7 +43679,7 @@
         <v>-0.15</v>
       </c>
       <c r="G771" t="n">
-        <v>-0.225</v>
+        <v>-0.23</v>
       </c>
       <c r="H771" t="inlineStr">
         <is>
@@ -43791,7 +43791,7 @@
         <v>-0.05</v>
       </c>
       <c r="G773" t="n">
-        <v>-0.075</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H773" t="inlineStr">
         <is>
@@ -43903,7 +43903,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="G775" t="n">
-        <v>-0.105</v>
+        <v>-0.1</v>
       </c>
       <c r="H775" t="inlineStr">
         <is>
@@ -44015,7 +44015,7 @@
         <v>-0.05</v>
       </c>
       <c r="G777" t="n">
-        <v>-0.075</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="H777" t="inlineStr">
         <is>
@@ -44127,7 +44127,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="G779" t="n">
-        <v>-0.105</v>
+        <v>-0.1</v>
       </c>
       <c r="H779" t="inlineStr">
         <is>
@@ -44351,7 +44351,7 @@
         <v>-0.17</v>
       </c>
       <c r="G783" t="n">
-        <v>-0.255</v>
+        <v>-0.26</v>
       </c>
       <c r="H783" t="inlineStr">
         <is>
@@ -44463,7 +44463,7 @@
         <v>-0.19</v>
       </c>
       <c r="G785" t="n">
-        <v>-0.285</v>
+        <v>-0.28</v>
       </c>
       <c r="H785" t="inlineStr">
         <is>
@@ -44575,7 +44575,7 @@
         <v>-0.21</v>
       </c>
       <c r="G787" t="n">
-        <v>-0.315</v>
+        <v>-0.32</v>
       </c>
       <c r="H787" t="inlineStr">
         <is>
@@ -44687,7 +44687,7 @@
         <v>-0.23</v>
       </c>
       <c r="G789" t="n">
-        <v>-0.345</v>
+        <v>-0.34</v>
       </c>
       <c r="H789" t="inlineStr">
         <is>
@@ -44799,7 +44799,7 @@
         <v>-0.25</v>
       </c>
       <c r="G791" t="n">
-        <v>-0.375</v>
+        <v>-0.38</v>
       </c>
       <c r="H791" t="inlineStr">
         <is>
@@ -45471,7 +45471,7 @@
         <v>0.68</v>
       </c>
       <c r="G803" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.82</v>
       </c>
       <c r="H803" t="inlineStr">
         <is>
@@ -45527,7 +45527,7 @@
         <v>0.71</v>
       </c>
       <c r="G804" t="n">
-        <v>0.852</v>
+        <v>0.85</v>
       </c>
       <c r="H804" t="inlineStr">
         <is>
@@ -45583,7 +45583,7 @@
         <v>0.73</v>
       </c>
       <c r="G805" t="n">
-        <v>0.876</v>
+        <v>0.88</v>
       </c>
       <c r="H805" t="inlineStr">
         <is>
@@ -45751,7 +45751,7 @@
         <v>0.78</v>
       </c>
       <c r="G808" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H808" t="inlineStr">
         <is>
@@ -46031,7 +46031,7 @@
         <v>0.72</v>
       </c>
       <c r="G813" t="n">
-        <v>0.864</v>
+        <v>0.86</v>
       </c>
       <c r="H813" t="inlineStr">
         <is>
@@ -46087,7 +46087,7 @@
         <v>0.74</v>
       </c>
       <c r="G814" t="n">
-        <v>0.888</v>
+        <v>0.89</v>
       </c>
       <c r="H814" t="inlineStr">
         <is>
@@ -46143,7 +46143,7 @@
         <v>0.76</v>
       </c>
       <c r="G815" t="n">
-        <v>0.912</v>
+        <v>0.91</v>
       </c>
       <c r="H815" t="inlineStr">
         <is>
@@ -46199,7 +46199,7 @@
         <v>0.78</v>
       </c>
       <c r="G816" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H816" t="inlineStr">
         <is>
@@ -46311,7 +46311,7 @@
         <v>0.68</v>
       </c>
       <c r="G818" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.82</v>
       </c>
       <c r="H818" t="inlineStr">
         <is>
@@ -46367,7 +46367,7 @@
         <v>0.71</v>
       </c>
       <c r="G819" t="n">
-        <v>0.852</v>
+        <v>0.85</v>
       </c>
       <c r="H819" t="inlineStr">
         <is>
@@ -46423,7 +46423,7 @@
         <v>0.73</v>
       </c>
       <c r="G820" t="n">
-        <v>0.876</v>
+        <v>0.88</v>
       </c>
       <c r="H820" t="inlineStr">
         <is>
@@ -46591,7 +46591,7 @@
         <v>0.68</v>
       </c>
       <c r="G823" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.82</v>
       </c>
       <c r="H823" t="inlineStr">
         <is>
@@ -46647,7 +46647,7 @@
         <v>0.71</v>
       </c>
       <c r="G824" t="n">
-        <v>0.852</v>
+        <v>0.85</v>
       </c>
       <c r="H824" t="inlineStr">
         <is>
@@ -46703,7 +46703,7 @@
         <v>0.73</v>
       </c>
       <c r="G825" t="n">
-        <v>0.876</v>
+        <v>0.88</v>
       </c>
       <c r="H825" t="inlineStr">
         <is>
@@ -46871,7 +46871,7 @@
         <v>0.72</v>
       </c>
       <c r="G828" t="n">
-        <v>0.864</v>
+        <v>0.86</v>
       </c>
       <c r="H828" t="inlineStr">
         <is>
@@ -46927,7 +46927,7 @@
         <v>0.74</v>
       </c>
       <c r="G829" t="n">
-        <v>0.888</v>
+        <v>0.89</v>
       </c>
       <c r="H829" t="inlineStr">
         <is>
@@ -46983,7 +46983,7 @@
         <v>0.76</v>
       </c>
       <c r="G830" t="n">
-        <v>0.912</v>
+        <v>0.91</v>
       </c>
       <c r="H830" t="inlineStr">
         <is>
@@ -47039,7 +47039,7 @@
         <v>0.78</v>
       </c>
       <c r="G831" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H831" t="inlineStr">
         <is>
@@ -47151,7 +47151,7 @@
         <v>0.72</v>
       </c>
       <c r="G833" t="n">
-        <v>0.864</v>
+        <v>0.86</v>
       </c>
       <c r="H833" t="inlineStr">
         <is>
@@ -47207,7 +47207,7 @@
         <v>0.74</v>
       </c>
       <c r="G834" t="n">
-        <v>0.888</v>
+        <v>0.89</v>
       </c>
       <c r="H834" t="inlineStr">
         <is>
@@ -47431,7 +47431,7 @@
         <v>0.52</v>
       </c>
       <c r="G838" t="n">
-        <v>0.624</v>
+        <v>0.62</v>
       </c>
       <c r="H838" t="inlineStr">
         <is>
@@ -47543,7 +47543,7 @@
         <v>0.58</v>
       </c>
       <c r="G840" t="n">
-        <v>0.696</v>
+        <v>0.7</v>
       </c>
       <c r="H840" t="inlineStr">
         <is>
@@ -47823,7 +47823,7 @@
         <v>0.64</v>
       </c>
       <c r="G845" t="n">
-        <v>0.768</v>
+        <v>0.77</v>
       </c>
       <c r="H845" t="inlineStr">
         <is>
@@ -47879,7 +47879,7 @@
         <v>0.68</v>
       </c>
       <c r="G846" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.82</v>
       </c>
       <c r="H846" t="inlineStr">
         <is>
@@ -47935,7 +47935,7 @@
         <v>0.54</v>
       </c>
       <c r="G847" t="n">
-        <v>0.648</v>
+        <v>0.65</v>
       </c>
       <c r="H847" t="inlineStr">
         <is>
@@ -47991,7 +47991,7 @@
         <v>0.58</v>
       </c>
       <c r="G848" t="n">
-        <v>0.696</v>
+        <v>0.7</v>
       </c>
       <c r="H848" t="inlineStr">
         <is>
@@ -48047,7 +48047,7 @@
         <v>0.62</v>
       </c>
       <c r="G849" t="n">
-        <v>0.744</v>
+        <v>0.74</v>
       </c>
       <c r="H849" t="inlineStr">
         <is>
@@ -48103,7 +48103,7 @@
         <v>0.66</v>
       </c>
       <c r="G850" t="n">
-        <v>0.792</v>
+        <v>0.79</v>
       </c>
       <c r="H850" t="inlineStr">
         <is>
@@ -48271,7 +48271,7 @@
         <v>0.73</v>
       </c>
       <c r="G853" t="n">
-        <v>0.876</v>
+        <v>0.88</v>
       </c>
       <c r="H853" t="inlineStr">
         <is>
@@ -48327,7 +48327,7 @@
         <v>0.76</v>
       </c>
       <c r="G854" t="n">
-        <v>0.912</v>
+        <v>0.91</v>
       </c>
       <c r="H854" t="inlineStr">
         <is>
@@ -48383,7 +48383,7 @@
         <v>0.79</v>
       </c>
       <c r="G855" t="n">
-        <v>0.948</v>
+        <v>0.95</v>
       </c>
       <c r="H855" t="inlineStr">
         <is>
@@ -57347,7 +57347,7 @@
         <v>0.39</v>
       </c>
       <c r="G1023" t="n">
-        <v>0.975</v>
+        <v>0.97</v>
       </c>
       <c r="H1023" t="inlineStr">
         <is>
@@ -58019,7 +58019,7 @@
         <v>0.36</v>
       </c>
       <c r="G1035" t="n">
-        <v>0.612</v>
+        <v>0.61</v>
       </c>
       <c r="H1035" t="inlineStr">
         <is>
@@ -58075,7 +58075,7 @@
         <v>0.42</v>
       </c>
       <c r="G1036" t="n">
-        <v>0.714</v>
+        <v>0.71</v>
       </c>
       <c r="H1036" t="inlineStr">
         <is>
@@ -58131,7 +58131,7 @@
         <v>0.48</v>
       </c>
       <c r="G1037" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.82</v>
       </c>
       <c r="H1037" t="inlineStr">
         <is>
@@ -58187,7 +58187,7 @@
         <v>0.55</v>
       </c>
       <c r="G1038" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H1038" t="inlineStr">
         <is>
@@ -58243,7 +58243,7 @@
         <v>0.62</v>
       </c>
       <c r="G1039" t="n">
-        <v>1.054</v>
+        <v>1.05</v>
       </c>
       <c r="H1039" t="inlineStr">
         <is>
@@ -58299,7 +58299,7 @@
         <v>0.72</v>
       </c>
       <c r="G1040" t="n">
-        <v>1.224</v>
+        <v>1.22</v>
       </c>
       <c r="H1040" t="inlineStr">
         <is>
@@ -58355,7 +58355,7 @@
         <v>0.82</v>
       </c>
       <c r="G1041" t="n">
-        <v>1.394</v>
+        <v>1.39</v>
       </c>
       <c r="H1041" t="inlineStr">
         <is>
@@ -58411,7 +58411,7 @@
         <v>0.93</v>
       </c>
       <c r="G1042" t="n">
-        <v>1.581</v>
+        <v>1.58</v>
       </c>
       <c r="H1042" t="inlineStr">
         <is>
@@ -58467,7 +58467,7 @@
         <v>1.04</v>
       </c>
       <c r="G1043" t="n">
-        <v>1.768</v>
+        <v>1.77</v>
       </c>
       <c r="H1043" t="inlineStr">
         <is>
@@ -58523,7 +58523,7 @@
         <v>1.16</v>
       </c>
       <c r="G1044" t="n">
-        <v>1.972</v>
+        <v>1.97</v>
       </c>
       <c r="H1044" t="inlineStr">
         <is>
@@ -60273,7 +60273,7 @@
       </c>
       <c r="J1075" t="inlineStr">
         <is>
-          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+          <t>Dropped in favor of direct moderated values S003-S012 (0.40 to 1.20) to avoid double-buff stacking.</t>
         </is>
       </c>
       <c r="K1075" t="inlineStr">
@@ -60283,7 +60283,7 @@
       </c>
       <c r="L1075" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -60329,7 +60329,7 @@
       </c>
       <c r="J1076" t="inlineStr">
         <is>
-          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+          <t>Dropped in favor of direct moderated values S003-S012 (0.40 to 1.20) to avoid double-buff stacking.</t>
         </is>
       </c>
       <c r="K1076" t="inlineStr">
@@ -60339,7 +60339,7 @@
       </c>
       <c r="L1076" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -60385,7 +60385,7 @@
       </c>
       <c r="J1077" t="inlineStr">
         <is>
-          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+          <t>Dropped in favor of direct moderated values S003-S012 (0.40 to 1.20) to avoid double-buff stacking.</t>
         </is>
       </c>
       <c r="K1077" t="inlineStr">
@@ -60395,7 +60395,7 @@
       </c>
       <c r="L1077" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -60441,7 +60441,7 @@
       </c>
       <c r="J1078" t="inlineStr">
         <is>
-          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+          <t>Dropped in favor of direct moderated values S003-S012 (0.40 to 1.20) to avoid double-buff stacking.</t>
         </is>
       </c>
       <c r="K1078" t="inlineStr">
@@ -60451,7 +60451,7 @@
       </c>
       <c r="L1078" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -60497,7 +60497,7 @@
       </c>
       <c r="J1079" t="inlineStr">
         <is>
-          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+          <t>Dropped in favor of direct moderated values S003-S012 (0.40 to 1.20) to avoid double-buff stacking.</t>
         </is>
       </c>
       <c r="K1079" t="inlineStr">
@@ -60507,7 +60507,7 @@
       </c>
       <c r="L1079" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -60553,7 +60553,7 @@
       </c>
       <c r="J1080" t="inlineStr">
         <is>
-          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+          <t>Dropped in favor of direct moderated values S003-S012 (0.40 to 1.20) to avoid double-buff stacking.</t>
         </is>
       </c>
       <c r="K1080" t="inlineStr">
@@ -60563,7 +60563,7 @@
       </c>
       <c r="L1080" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -60609,7 +60609,7 @@
       </c>
       <c r="J1081" t="inlineStr">
         <is>
-          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+          <t>Dropped in favor of direct moderated values S003-S012 (0.40 to 1.20) to avoid double-buff stacking.</t>
         </is>
       </c>
       <c r="K1081" t="inlineStr">
@@ -60619,7 +60619,7 @@
       </c>
       <c r="L1081" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -60665,7 +60665,7 @@
       </c>
       <c r="J1082" t="inlineStr">
         <is>
-          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+          <t>Dropped in favor of direct moderated values S003-S012 (0.40 to 1.20) to avoid double-buff stacking.</t>
         </is>
       </c>
       <c r="K1082" t="inlineStr">
@@ -60675,7 +60675,7 @@
       </c>
       <c r="L1082" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -60721,7 +60721,7 @@
       </c>
       <c r="J1083" t="inlineStr">
         <is>
-          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+          <t>Dropped in favor of direct moderated values S003-S012 (0.40 to 1.20) to avoid double-buff stacking.</t>
         </is>
       </c>
       <c r="K1083" t="inlineStr">
@@ -60731,7 +60731,7 @@
       </c>
       <c r="L1083" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -60777,7 +60777,7 @@
       </c>
       <c r="J1084" t="inlineStr">
         <is>
-          <t>Trickster (intermediate). Checkmate, the single strike of the Trickster, x1.6 power at every level (on top of S): the Trickster fought 16 - 20% longer than the median attacker at C10, C13, C18 (12 - 15% after); the Papillon and the Joker who keep it stay within the band later (0.88 - 0.97 of the median). High Risk High Return x1.6 was measured too and changes nothing</t>
+          <t>Dropped in favor of direct moderated values S003-S012 (0.40 to 1.20) to avoid double-buff stacking.</t>
         </is>
       </c>
       <c r="K1084" t="inlineStr">
@@ -60787,7 +60787,7 @@
       </c>
       <c r="L1084" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -61099,7 +61099,7 @@
         <v>0.7</v>
       </c>
       <c r="G1090" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="H1090" t="inlineStr">
         <is>
@@ -61113,7 +61113,7 @@
       </c>
       <c r="J1090" t="inlineStr">
         <is>
-          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+          <t>Pursuit Stab: power 1.00 to 1.55 (+35% to +43%), -25% TP cost kept (level 1 = 1.0).</t>
         </is>
       </c>
       <c r="K1090" t="inlineStr">
@@ -61155,7 +61155,7 @@
         <v>0.82</v>
       </c>
       <c r="G1091" t="n">
-        <v>1.64</v>
+        <v>1.15</v>
       </c>
       <c r="H1091" t="inlineStr">
         <is>
@@ -61169,7 +61169,7 @@
       </c>
       <c r="J1091" t="inlineStr">
         <is>
-          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+          <t>Pursuit Stab: power 1.00 to 1.55 (+35% to +43%), -25% TP cost kept (level 2 = 1.15).</t>
         </is>
       </c>
       <c r="K1091" t="inlineStr">
@@ -61211,7 +61211,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="G1092" t="n">
-        <v>1.88</v>
+        <v>1.28</v>
       </c>
       <c r="H1092" t="inlineStr">
         <is>
@@ -61225,7 +61225,7 @@
       </c>
       <c r="J1092" t="inlineStr">
         <is>
-          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+          <t>Pursuit Stab: power 1.00 to 1.55 (+35% to +43%), -25% TP cost kept (level 3 = 1.28).</t>
         </is>
       </c>
       <c r="K1092" t="inlineStr">
@@ -61267,7 +61267,7 @@
         <v>1.04</v>
       </c>
       <c r="G1093" t="n">
-        <v>2.08</v>
+        <v>1.42</v>
       </c>
       <c r="H1093" t="inlineStr">
         <is>
@@ -61281,7 +61281,7 @@
       </c>
       <c r="J1093" t="inlineStr">
         <is>
-          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+          <t>Pursuit Stab: power 1.00 to 1.55 (+35% to +43%), -25% TP cost kept (level 4 = 1.42).</t>
         </is>
       </c>
       <c r="K1093" t="inlineStr">
@@ -61323,7 +61323,7 @@
         <v>1.12</v>
       </c>
       <c r="G1094" t="n">
-        <v>2.24</v>
+        <v>1.55</v>
       </c>
       <c r="H1094" t="inlineStr">
         <is>
@@ -61337,7 +61337,7 @@
       </c>
       <c r="J1094" t="inlineStr">
         <is>
-          <t>Treasure Hunter (advanced): Pursuit Stab, her one strike with a dagger, -25% TP and x2 power. Her basic hit with a dagger does not pass a boss defence (3 damage), so with 187 TP and 38 a strike she ran dry in five turns: fights 31% longer than the median attacker at C22, C29, C34, C40; 1.01 after, and 0.89 at the late checkpoints (the Dark Lord 0.88). x1.5 leaves 1.21</t>
+          <t>Pursuit Stab: power 1.00 to 1.55 (+35% to +43%), -25% TP cost kept (level 5 = 1.55).</t>
         </is>
       </c>
       <c r="K1094" t="inlineStr">
@@ -61715,7 +61715,7 @@
         <v>0.24</v>
       </c>
       <c r="G1101" t="n">
-        <v>0.384</v>
+        <v>0.38</v>
       </c>
       <c r="H1101" t="inlineStr">
         <is>
@@ -61771,7 +61771,7 @@
         <v>0.28</v>
       </c>
       <c r="G1102" t="n">
-        <v>0.448</v>
+        <v>0.45</v>
       </c>
       <c r="H1102" t="inlineStr">
         <is>
@@ -61827,7 +61827,7 @@
         <v>0.32</v>
       </c>
       <c r="G1103" t="n">
-        <v>0.512</v>
+        <v>0.51</v>
       </c>
       <c r="H1103" t="inlineStr">
         <is>
@@ -61883,7 +61883,7 @@
         <v>0.36</v>
       </c>
       <c r="G1104" t="n">
-        <v>0.576</v>
+        <v>0.58</v>
       </c>
       <c r="H1104" t="inlineStr">
         <is>
@@ -62219,7 +62219,7 @@
         <v>0.08</v>
       </c>
       <c r="G1110" t="n">
-        <v>0.128</v>
+        <v>0.13</v>
       </c>
       <c r="H1110" t="inlineStr">
         <is>
@@ -62331,7 +62331,7 @@
         <v>0.12</v>
       </c>
       <c r="G1112" t="n">
-        <v>0.192</v>
+        <v>0.19</v>
       </c>
       <c r="H1112" t="inlineStr">
         <is>
@@ -62387,7 +62387,7 @@
         <v>0.14</v>
       </c>
       <c r="G1113" t="n">
-        <v>0.224</v>
+        <v>0.22</v>
       </c>
       <c r="H1113" t="inlineStr">
         <is>
@@ -62443,7 +62443,7 @@
         <v>0.16</v>
       </c>
       <c r="G1114" t="n">
-        <v>0.256</v>
+        <v>0.26</v>
       </c>
       <c r="H1114" t="inlineStr">
         <is>
@@ -62499,7 +62499,7 @@
         <v>0.08</v>
       </c>
       <c r="G1115" t="n">
-        <v>0.128</v>
+        <v>0.13</v>
       </c>
       <c r="H1115" t="inlineStr">
         <is>
@@ -62611,7 +62611,7 @@
         <v>0.12</v>
       </c>
       <c r="G1117" t="n">
-        <v>0.192</v>
+        <v>0.19</v>
       </c>
       <c r="H1117" t="inlineStr">
         <is>
@@ -62667,7 +62667,7 @@
         <v>0.14</v>
       </c>
       <c r="G1118" t="n">
-        <v>0.224</v>
+        <v>0.22</v>
       </c>
       <c r="H1118" t="inlineStr">
         <is>
@@ -62723,7 +62723,7 @@
         <v>0.16</v>
       </c>
       <c r="G1119" t="n">
-        <v>0.256</v>
+        <v>0.26</v>
       </c>
       <c r="H1119" t="inlineStr">
         <is>
@@ -62835,7 +62835,7 @@
         <v>0.05</v>
       </c>
       <c r="G1121" t="n">
-        <v>0.075</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H1121" t="inlineStr">
         <is>
@@ -62947,7 +62947,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="G1123" t="n">
-        <v>0.105</v>
+        <v>0.1</v>
       </c>
       <c r="H1123" t="inlineStr">
         <is>
@@ -63115,7 +63115,7 @@
         <v>0.05</v>
       </c>
       <c r="G1126" t="n">
-        <v>0.075</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H1126" t="inlineStr">
         <is>
@@ -63227,7 +63227,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="G1128" t="n">
-        <v>0.105</v>
+        <v>0.1</v>
       </c>
       <c r="H1128" t="inlineStr">
         <is>
@@ -63395,7 +63395,7 @@
         <v>0.05</v>
       </c>
       <c r="G1131" t="n">
-        <v>0.075</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H1131" t="inlineStr">
         <is>
@@ -63507,7 +63507,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="G1133" t="n">
-        <v>0.105</v>
+        <v>0.1</v>
       </c>
       <c r="H1133" t="inlineStr">
         <is>
@@ -63675,7 +63675,7 @@
         <v>0.05</v>
       </c>
       <c r="G1136" t="n">
-        <v>0.075</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H1136" t="inlineStr">
         <is>
@@ -63787,7 +63787,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="G1138" t="n">
-        <v>0.105</v>
+        <v>0.1</v>
       </c>
       <c r="H1138" t="inlineStr">
         <is>
@@ -63955,7 +63955,7 @@
         <v>0.05</v>
       </c>
       <c r="G1141" t="n">
-        <v>0.075</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H1141" t="inlineStr">
         <is>
@@ -64067,7 +64067,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="G1143" t="n">
-        <v>0.105</v>
+        <v>0.1</v>
       </c>
       <c r="H1143" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
balance: scale Provoke enmity
scale Provoke enmity (400-1500) and buff Anti-Meta survivability

- Scale Provoke (Technique 0) Effect 170 from flat 250 to 400-1500
across levels 1-5 (draws ~95% single-target aggro at max level) -
Minimal tweak Life Bringer (Technique 91) Effect 26 to [0.05, 0.10,
0.15, 0.20, 0.25] - Moderate Spartan (Technique 95) turns to [3, 3, 4,
4, 4, 5, 5, 5, 6, 6] (starts at 3, ends at 6) - Add modest heal buff to
Catalina (Technique 104) Effect 103: [6, 8, 10, 13, 16] - Add Magic
Barrier (Technique 58) Effect 183: [-0.25, -0.28, -0.32, -0.36, -0.40] -
Enable Magical Princess bit 17 equipment compatibility for Kite Shield
(538) and Fluted Armor (666) - Optimize Magical Princess SP priority in
sim_setup.xlsx and support class bitmask in variant.py - Fix battle.py
MAX_HP_DRAIN execution
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1371"/>
+  <dimension ref="A1:L1388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12761,7 +12761,7 @@
         <v>3</v>
       </c>
       <c r="G220" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H220" t="inlineStr">
         <is>
@@ -12780,7 +12780,7 @@
       </c>
       <c r="K220" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L220" t="inlineStr">
@@ -12817,7 +12817,7 @@
         <v>3</v>
       </c>
       <c r="G221" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H221" t="inlineStr">
         <is>
@@ -12836,7 +12836,7 @@
       </c>
       <c r="K221" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L221" t="inlineStr">
@@ -12873,7 +12873,7 @@
         <v>3</v>
       </c>
       <c r="G222" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H222" t="inlineStr">
         <is>
@@ -12892,7 +12892,7 @@
       </c>
       <c r="K222" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L222" t="inlineStr">
@@ -12929,7 +12929,7 @@
         <v>4</v>
       </c>
       <c r="G223" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H223" t="inlineStr">
         <is>
@@ -12948,7 +12948,7 @@
       </c>
       <c r="K223" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L223" t="inlineStr">
@@ -12985,7 +12985,7 @@
         <v>4</v>
       </c>
       <c r="G224" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H224" t="inlineStr">
         <is>
@@ -13004,7 +13004,7 @@
       </c>
       <c r="K224" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L224" t="inlineStr">
@@ -13041,7 +13041,7 @@
         <v>4</v>
       </c>
       <c r="G225" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H225" t="inlineStr">
         <is>
@@ -13060,7 +13060,7 @@
       </c>
       <c r="K225" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L225" t="inlineStr">
@@ -13097,7 +13097,7 @@
         <v>5</v>
       </c>
       <c r="G226" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H226" t="inlineStr">
         <is>
@@ -13116,7 +13116,7 @@
       </c>
       <c r="K226" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L226" t="inlineStr">
@@ -13153,7 +13153,7 @@
         <v>5</v>
       </c>
       <c r="G227" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H227" t="inlineStr">
         <is>
@@ -13172,7 +13172,7 @@
       </c>
       <c r="K227" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L227" t="inlineStr">
@@ -13209,7 +13209,7 @@
         <v>5</v>
       </c>
       <c r="G228" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H228" t="inlineStr">
         <is>
@@ -13228,7 +13228,7 @@
       </c>
       <c r="K228" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L228" t="inlineStr">
@@ -13265,7 +13265,7 @@
         <v>6</v>
       </c>
       <c r="G229" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H229" t="inlineStr">
         <is>
@@ -13284,7 +13284,7 @@
       </c>
       <c r="K229" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L229" t="inlineStr">
@@ -65859,7 +65859,7 @@
         <v>-0.12</v>
       </c>
       <c r="G1175" t="n">
-        <v>0.58</v>
+        <v>0.05</v>
       </c>
       <c r="H1175" t="inlineStr">
         <is>
@@ -65878,7 +65878,7 @@
       </c>
       <c r="K1175" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L1175" t="inlineStr">
@@ -65915,7 +65915,7 @@
         <v>-0.08</v>
       </c>
       <c r="G1176" t="n">
-        <v>0.62</v>
+        <v>0.1</v>
       </c>
       <c r="H1176" t="inlineStr">
         <is>
@@ -65934,7 +65934,7 @@
       </c>
       <c r="K1176" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L1176" t="inlineStr">
@@ -65971,7 +65971,7 @@
         <v>-0.03</v>
       </c>
       <c r="G1177" t="n">
-        <v>0.67</v>
+        <v>0.15</v>
       </c>
       <c r="H1177" t="inlineStr">
         <is>
@@ -65990,7 +65990,7 @@
       </c>
       <c r="K1177" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L1177" t="inlineStr">
@@ -66027,7 +66027,7 @@
         <v>0.03</v>
       </c>
       <c r="G1178" t="n">
-        <v>0.73</v>
+        <v>0.2</v>
       </c>
       <c r="H1178" t="inlineStr">
         <is>
@@ -66046,7 +66046,7 @@
       </c>
       <c r="K1178" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L1178" t="inlineStr">
@@ -66083,7 +66083,7 @@
         <v>0.1</v>
       </c>
       <c r="G1179" t="n">
-        <v>0.8</v>
+        <v>0.25</v>
       </c>
       <c r="H1179" t="inlineStr">
         <is>
@@ -66102,7 +66102,7 @@
       </c>
       <c r="K1179" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L1179" t="inlineStr">
@@ -76513,6 +76513,960 @@
         </is>
       </c>
       <c r="L1371" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>S022</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>Technique 58 Magic Barrier</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>effect 183</t>
+        </is>
+      </c>
+      <c r="E1372" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1372" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="G1372" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="H1372" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1372" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1372" t="inlineStr">
+        <is>
+          <t>Magic Barrier party magic damage reduction buff</t>
+        </is>
+      </c>
+      <c r="K1372" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1372" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>S023</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>Technique 58 Magic Barrier</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>effect 183</t>
+        </is>
+      </c>
+      <c r="E1373" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1373" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G1373" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="H1373" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1373" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1373" t="inlineStr">
+        <is>
+          <t>Magic Barrier party magic damage reduction buff</t>
+        </is>
+      </c>
+      <c r="K1373" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1373" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>S024</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>Technique 58 Magic Barrier</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>effect 183</t>
+        </is>
+      </c>
+      <c r="E1374" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1374" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="G1374" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="H1374" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1374" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1374" t="inlineStr">
+        <is>
+          <t>Magic Barrier party magic damage reduction buff</t>
+        </is>
+      </c>
+      <c r="K1374" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1374" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="inlineStr">
+        <is>
+          <t>S025</t>
+        </is>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>Technique 58 Magic Barrier</t>
+        </is>
+      </c>
+      <c r="D1375" t="inlineStr">
+        <is>
+          <t>effect 183</t>
+        </is>
+      </c>
+      <c r="E1375" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1375" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="G1375" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="H1375" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1375" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1375" t="inlineStr">
+        <is>
+          <t>Magic Barrier party magic damage reduction buff</t>
+        </is>
+      </c>
+      <c r="K1375" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1375" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="inlineStr">
+        <is>
+          <t>S026</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>Technique 58 Magic Barrier</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>effect 183</t>
+        </is>
+      </c>
+      <c r="E1376" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1376" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="G1376" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="H1376" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1376" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1376" t="inlineStr">
+        <is>
+          <t>Magic Barrier party magic damage reduction buff</t>
+        </is>
+      </c>
+      <c r="K1376" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1376" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t>S027</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>Technique 104 Catalina's Action</t>
+        </is>
+      </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>effect 103</t>
+        </is>
+      </c>
+      <c r="E1377" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1377" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1377" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1377" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1377" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1377" t="inlineStr">
+        <is>
+          <t>Catalina modest heal buff for party sustain</t>
+        </is>
+      </c>
+      <c r="K1377" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1377" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>S028</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>Technique 104 Catalina's Action</t>
+        </is>
+      </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>effect 103</t>
+        </is>
+      </c>
+      <c r="E1378" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1378" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1378" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1378" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1378" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1378" t="inlineStr">
+        <is>
+          <t>Catalina modest heal buff for party sustain</t>
+        </is>
+      </c>
+      <c r="K1378" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1378" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>S029</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>Technique 104 Catalina's Action</t>
+        </is>
+      </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>effect 103</t>
+        </is>
+      </c>
+      <c r="E1379" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1379" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1379" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1379" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1379" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1379" t="inlineStr">
+        <is>
+          <t>Catalina modest heal buff for party sustain</t>
+        </is>
+      </c>
+      <c r="K1379" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1379" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t>S030</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>Technique 104 Catalina's Action</t>
+        </is>
+      </c>
+      <c r="D1380" t="inlineStr">
+        <is>
+          <t>effect 103</t>
+        </is>
+      </c>
+      <c r="E1380" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1380" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1380" t="n">
+        <v>13</v>
+      </c>
+      <c r="H1380" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1380" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1380" t="inlineStr">
+        <is>
+          <t>Catalina modest heal buff for party sustain</t>
+        </is>
+      </c>
+      <c r="K1380" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1380" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>S031</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>Technique 104 Catalina's Action</t>
+        </is>
+      </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>effect 103</t>
+        </is>
+      </c>
+      <c r="E1381" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1381" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1381" t="n">
+        <v>16</v>
+      </c>
+      <c r="H1381" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1381" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1381" t="inlineStr">
+        <is>
+          <t>Catalina modest heal buff for party sustain</t>
+        </is>
+      </c>
+      <c r="K1381" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1381" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>W040</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>538 Kite Shield</t>
+        </is>
+      </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>class bitmask</t>
+        </is>
+      </c>
+      <c r="F1382" t="inlineStr">
+        <is>
+          <t>0x3f</t>
+        </is>
+      </c>
+      <c r="G1382" t="inlineStr">
+        <is>
+          <t>0x2003f</t>
+        </is>
+      </c>
+      <c r="H1382" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="I1382" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1382" t="inlineStr">
+        <is>
+          <t>Magical Princess equipment compatibility: enable bit 17</t>
+        </is>
+      </c>
+      <c r="K1382" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1382" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>W041</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>666 Fluted Armor</t>
+        </is>
+      </c>
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>class bitmask</t>
+        </is>
+      </c>
+      <c r="F1383" t="inlineStr">
+        <is>
+          <t>0x3f</t>
+        </is>
+      </c>
+      <c r="G1383" t="inlineStr">
+        <is>
+          <t>0x2003f</t>
+        </is>
+      </c>
+      <c r="H1383" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="I1383" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1383" t="inlineStr">
+        <is>
+          <t>Magical Princess equipment compatibility: enable bit 17</t>
+        </is>
+      </c>
+      <c r="K1383" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1383" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>S032</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>Technique 0 Provoke</t>
+        </is>
+      </c>
+      <c r="D1384" t="inlineStr">
+        <is>
+          <t>effect 170</t>
+        </is>
+      </c>
+      <c r="E1384" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1384" t="n">
+        <v>250</v>
+      </c>
+      <c r="G1384" t="n">
+        <v>400</v>
+      </c>
+      <c r="H1384" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1384" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1384" t="inlineStr">
+        <is>
+          <t>Provoke enmity scaling: raise from flat 250 to 400-1500 so max rank draws 95% aggro</t>
+        </is>
+      </c>
+      <c r="K1384" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1384" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>S033</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>Technique 0 Provoke</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>effect 170</t>
+        </is>
+      </c>
+      <c r="E1385" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1385" t="n">
+        <v>250</v>
+      </c>
+      <c r="G1385" t="n">
+        <v>600</v>
+      </c>
+      <c r="H1385" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1385" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1385" t="inlineStr">
+        <is>
+          <t>Provoke enmity scaling: raise from flat 250 to 400-1500 so max rank draws 95% aggro</t>
+        </is>
+      </c>
+      <c r="K1385" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1385" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>S034</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>Technique 0 Provoke</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>effect 170</t>
+        </is>
+      </c>
+      <c r="E1386" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1386" t="n">
+        <v>250</v>
+      </c>
+      <c r="G1386" t="n">
+        <v>850</v>
+      </c>
+      <c r="H1386" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1386" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1386" t="inlineStr">
+        <is>
+          <t>Provoke enmity scaling: raise from flat 250 to 400-1500 so max rank draws 95% aggro</t>
+        </is>
+      </c>
+      <c r="K1386" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1386" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>S035</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>Technique 0 Provoke</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>effect 170</t>
+        </is>
+      </c>
+      <c r="E1387" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1387" t="n">
+        <v>250</v>
+      </c>
+      <c r="G1387" t="n">
+        <v>1150</v>
+      </c>
+      <c r="H1387" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1387" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1387" t="inlineStr">
+        <is>
+          <t>Provoke enmity scaling: raise from flat 250 to 400-1500 so max rank draws 95% aggro</t>
+        </is>
+      </c>
+      <c r="K1387" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1387" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>S036</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>Technique 0 Provoke</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>effect 170</t>
+        </is>
+      </c>
+      <c r="E1388" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1388" t="n">
+        <v>250</v>
+      </c>
+      <c r="G1388" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H1388" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="I1388" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1388" t="inlineStr">
+        <is>
+          <t>Provoke enmity scaling: raise from flat 250 to 400-1500 so max rank draws 95% aggro</t>
+        </is>
+      </c>
+      <c r="K1388" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1388" t="inlineStr">
         <is>
           <t>decided</t>
         </is>

</xml_diff>

<commit_message>
balance(skills): adjust Provoke enmity progression to 200-1500
- Set Provoke (Technique 0) Effect 170 to [200, 450, 750, 1100, 1500] -
Avoid early-game OP at Lv1 (200 enmity, ~73% draw) while rewarding full
investment at Lv5 (1500 enmity, ~95% draw)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -77220,7 +77220,7 @@
         <v>250</v>
       </c>
       <c r="G1384" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="H1384" t="inlineStr">
         <is>
@@ -77276,7 +77276,7 @@
         <v>250</v>
       </c>
       <c r="G1385" t="n">
-        <v>600</v>
+        <v>450</v>
       </c>
       <c r="H1385" t="inlineStr">
         <is>
@@ -77332,7 +77332,7 @@
         <v>250</v>
       </c>
       <c r="G1386" t="n">
-        <v>850</v>
+        <v>750</v>
       </c>
       <c r="H1386" t="inlineStr">
         <is>
@@ -77388,7 +77388,7 @@
         <v>250</v>
       </c>
       <c r="G1387" t="n">
-        <v>1150</v>
+        <v>1100</v>
       </c>
       <c r="H1387" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
balance(kunoichi): enable hybrid weapon codes [0
enable hybrid weapon codes [0, 10] for Stings and Phoenix; equip Tantou
in sim

- Add rows S037-S040 in balance_changes.xlsx to allow Sleep Sting,
Silence Sting, Stun Sting, and Phoenix to accept both short-range
weapons (code 0) and projectiles (code 10). - Update Kunoichi weapon in
sim_setup.xlsx Roles to 'Dagger; Kunoichi=Tantou'. - Verify 100% win
rate across 15 seeds at C34 with actions dropping from 400+ to ~228-264
actions across Katana, Projectile, and Dagger variants.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1388"/>
+  <dimension ref="A1:L1392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77472,6 +77472,234 @@
         </is>
       </c>
     </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>S037</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>Technique 38 Sleep Sting</t>
+        </is>
+      </c>
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>weapon codes</t>
+        </is>
+      </c>
+      <c r="F1389" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G1389" t="inlineStr">
+        <is>
+          <t>0, 10</t>
+        </is>
+      </c>
+      <c r="H1389" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1389" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1389" t="inlineStr">
+        <is>
+          <t>Allow Sleep Sting to be used with both short-range weapons and projectiles</t>
+        </is>
+      </c>
+      <c r="K1389" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1389" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>S038</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>Technique 39 Silence Sting</t>
+        </is>
+      </c>
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>weapon codes</t>
+        </is>
+      </c>
+      <c r="F1390" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G1390" t="inlineStr">
+        <is>
+          <t>0, 10</t>
+        </is>
+      </c>
+      <c r="H1390" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1390" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1390" t="inlineStr">
+        <is>
+          <t>Allow Silence Sting to be used with both short-range weapons and projectiles</t>
+        </is>
+      </c>
+      <c r="K1390" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1390" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>S039</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>Technique 40 Stun Sting</t>
+        </is>
+      </c>
+      <c r="D1391" t="inlineStr">
+        <is>
+          <t>weapon codes</t>
+        </is>
+      </c>
+      <c r="F1391" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G1391" t="inlineStr">
+        <is>
+          <t>0, 10</t>
+        </is>
+      </c>
+      <c r="H1391" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1391" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1391" t="inlineStr">
+        <is>
+          <t>Allow Stun Sting to be used with both short-range weapons and projectiles</t>
+        </is>
+      </c>
+      <c r="K1391" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1391" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>S040</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>Technique 51 Phoenix</t>
+        </is>
+      </c>
+      <c r="D1392" t="inlineStr">
+        <is>
+          <t>weapon codes</t>
+        </is>
+      </c>
+      <c r="F1392" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G1392" t="inlineStr">
+        <is>
+          <t>0, 10</t>
+        </is>
+      </c>
+      <c r="H1392" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1392" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="J1392" t="inlineStr">
+        <is>
+          <t>Allow Phoenix to be used with both projectiles and short-range weapons</t>
+        </is>
+      </c>
+      <c r="K1392" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1392" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
balance(skills): cap Spartan Lv9-10 TP cost at 36 (rows S041-S042)
- Relieve high-rank TP starvation for Soul Summoner in extended
endurance encounters. - 196 tests passing.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1392"/>
+  <dimension ref="A1:L1394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77700,6 +77700,118 @@
         </is>
       </c>
     </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>S041</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>Technique 95 Spartan</t>
+        </is>
+      </c>
+      <c r="D1393" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1393" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1393" t="n">
+        <v>39</v>
+      </c>
+      <c r="G1393" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1393" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1393" t="inlineStr">
+        <is>
+          <t>F71</t>
+        </is>
+      </c>
+      <c r="J1393" t="inlineStr">
+        <is>
+          <t>Spartan high-rank TP cost relief: cap at 36 so long endurance fights do not starve TP</t>
+        </is>
+      </c>
+      <c r="K1393" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1393" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>S042</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>Technique 95 Spartan</t>
+        </is>
+      </c>
+      <c r="D1394" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1394" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1394" t="n">
+        <v>42</v>
+      </c>
+      <c r="G1394" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1394" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1394" t="inlineStr">
+        <is>
+          <t>F71</t>
+        </is>
+      </c>
+      <c r="J1394" t="inlineStr">
+        <is>
+          <t>Spartan high-rank TP cost relief: cap at 36 so long endurance fights do not starve TP</t>
+        </is>
+      </c>
+      <c r="K1394" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="L1394" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
balance: apply moderate stat buffs to top 3 easiest bosses
apply moderate stat buffs to top 3 easiest bosses (C10, C13, C24)

- C10 (Countess of Vrachia): HP +15% (1991 -> 2289), ATK +4% (70 -> 73),
DEF +4% (54 -> 56). Average rounds extended from 10.5r to 15.2r with
100% win rate across all 5 parties. - C13 (Eros): HP +20% (2277 ->
2732), ATK +5% (57 -> 60), DEF +5% (55 -> 58). Average rounds extended
from 9.3r to 10.8r with 98% win rate. - C24 (Afanc): HP +25% (4582 ->
5728), ATK +7% (152 -> 163), DEF +7% (120 -> 129). Average rounds
extended from 7.9r to 9.6r with 99% win rate, preventing 4-turn melt by
Tier 3 burst. - Added changes G094-G102 to balance_changes.xlsx. -
Updated docs/generated/PARTY_BATTERY_OLD_VS_NEW_AI.md. - All 196 tests
passing.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1394"/>
+  <dimension ref="A1:L1403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77812,6 +77812,483 @@
         </is>
       </c>
     </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>G094</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>1002 Countess of Vrachia (C10)</t>
+        </is>
+      </c>
+      <c r="D1395" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1395" t="n">
+        <v>1991</v>
+      </c>
+      <c r="G1395" t="n">
+        <v>2289</v>
+      </c>
+      <c r="H1395" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1395" t="inlineStr">
+        <is>
+          <t>F15</t>
+        </is>
+      </c>
+      <c r="J1395" t="inlineStr">
+        <is>
+          <t>Top 3 easiest boss buff (user request): C10 Countess of Vrachia HP +15% (1991 -&gt; 2289) to prevent instant trivialization across all parties while preserving 100% win rate parity (rnds 10.5r -&gt; 15.2r).</t>
+        </is>
+      </c>
+      <c r="K1395" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1395" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>G095</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>1002 Countess of Vrachia (C10)</t>
+        </is>
+      </c>
+      <c r="D1396" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1396" t="n">
+        <v>70</v>
+      </c>
+      <c r="G1396" t="n">
+        <v>73</v>
+      </c>
+      <c r="H1396" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1396" t="inlineStr">
+        <is>
+          <t>F15</t>
+        </is>
+      </c>
+      <c r="J1396" t="inlineStr">
+        <is>
+          <t>Top 3 easiest boss buff: C10 Countess of Vrachia ATK +4% (70 -&gt; 73) for moderate combat pressure.</t>
+        </is>
+      </c>
+      <c r="K1396" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1396" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>G096</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>1002 Countess of Vrachia (C10)</t>
+        </is>
+      </c>
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>def</t>
+        </is>
+      </c>
+      <c r="F1397" t="n">
+        <v>54</v>
+      </c>
+      <c r="G1397" t="n">
+        <v>56</v>
+      </c>
+      <c r="H1397" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1397" t="inlineStr">
+        <is>
+          <t>F15</t>
+        </is>
+      </c>
+      <c r="J1397" t="inlineStr">
+        <is>
+          <t>Top 3 easiest boss buff: C10 Countess of Vrachia DEF +4% (54 -&gt; 56).</t>
+        </is>
+      </c>
+      <c r="K1397" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1397" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>G097</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>760 Eros (C13)</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1398" t="n">
+        <v>2277</v>
+      </c>
+      <c r="G1398" t="n">
+        <v>2732</v>
+      </c>
+      <c r="H1398" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1398" t="inlineStr">
+        <is>
+          <t>F15</t>
+        </is>
+      </c>
+      <c r="J1398" t="inlineStr">
+        <is>
+          <t>Top 3 easiest boss buff (user request): C13 Eros HP +20% (2277 -&gt; 2732) to extend midgame boss duration moderately from 9.3r to 10.8r across all 5 parties.</t>
+        </is>
+      </c>
+      <c r="K1398" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1398" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>G098</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>760 Eros (C13)</t>
+        </is>
+      </c>
+      <c r="D1399" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1399" t="n">
+        <v>57</v>
+      </c>
+      <c r="G1399" t="n">
+        <v>60</v>
+      </c>
+      <c r="H1399" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1399" t="inlineStr">
+        <is>
+          <t>F15</t>
+        </is>
+      </c>
+      <c r="J1399" t="inlineStr">
+        <is>
+          <t>Top 3 easiest boss buff: C13 Eros ATK +5% (57 -&gt; 60).</t>
+        </is>
+      </c>
+      <c r="K1399" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1399" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="inlineStr">
+        <is>
+          <t>G099</t>
+        </is>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>760 Eros (C13)</t>
+        </is>
+      </c>
+      <c r="D1400" t="inlineStr">
+        <is>
+          <t>def</t>
+        </is>
+      </c>
+      <c r="F1400" t="n">
+        <v>55</v>
+      </c>
+      <c r="G1400" t="n">
+        <v>58</v>
+      </c>
+      <c r="H1400" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1400" t="inlineStr">
+        <is>
+          <t>F15</t>
+        </is>
+      </c>
+      <c r="J1400" t="inlineStr">
+        <is>
+          <t>Top 3 easiest boss buff: C13 Eros DEF +5% (55 -&gt; 58).</t>
+        </is>
+      </c>
+      <c r="K1400" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1400" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>G100</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>825 Afanc (C24)</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1401" t="n">
+        <v>4582</v>
+      </c>
+      <c r="G1401" t="n">
+        <v>5728</v>
+      </c>
+      <c r="H1401" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1401" t="inlineStr">
+        <is>
+          <t>F15</t>
+        </is>
+      </c>
+      <c r="J1401" t="inlineStr">
+        <is>
+          <t>Top 3 easiest boss buff (user request): C24 Afanc HP +25% (4582 -&gt; 5728) to bring boss duration from 7.9r to 9.6r, keeping win rate at 99% while preventing 4-turn trivial melts by Tier 3 physical burst.</t>
+        </is>
+      </c>
+      <c r="K1401" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1401" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="inlineStr">
+        <is>
+          <t>G101</t>
+        </is>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>825 Afanc (C24)</t>
+        </is>
+      </c>
+      <c r="D1402" t="inlineStr">
+        <is>
+          <t>atk</t>
+        </is>
+      </c>
+      <c r="F1402" t="n">
+        <v>152</v>
+      </c>
+      <c r="G1402" t="n">
+        <v>163</v>
+      </c>
+      <c r="H1402" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1402" t="inlineStr">
+        <is>
+          <t>F15</t>
+        </is>
+      </c>
+      <c r="J1402" t="inlineStr">
+        <is>
+          <t>Top 3 easiest boss buff: C24 Afanc ATK +7% (152 -&gt; 163).</t>
+        </is>
+      </c>
+      <c r="K1402" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1402" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="inlineStr">
+        <is>
+          <t>G102</t>
+        </is>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr">
+        <is>
+          <t>825 Afanc (C24)</t>
+        </is>
+      </c>
+      <c r="D1403" t="inlineStr">
+        <is>
+          <t>def</t>
+        </is>
+      </c>
+      <c r="F1403" t="n">
+        <v>120</v>
+      </c>
+      <c r="G1403" t="n">
+        <v>129</v>
+      </c>
+      <c r="H1403" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1403" t="inlineStr">
+        <is>
+          <t>F15</t>
+        </is>
+      </c>
+      <c r="J1403" t="inlineStr">
+        <is>
+          <t>Top 3 easiest boss buff: C24 Afanc DEF +7% (120 -&gt; 129).</t>
+        </is>
+      </c>
+      <c r="K1403" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1403" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(audit): integrate audit fixes - Stage 15 mobs
integrate audit fixes - Stage 15 mobs, x86 parity, Slave's Torc, Sleep
immunity, and Plus parties
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1403"/>
+  <dimension ref="A1:L1404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36234,7 +36234,7 @@
       </c>
       <c r="G639" t="inlineStr">
         <is>
-          <t>0x14e7</t>
+          <t>0x14ef</t>
         </is>
       </c>
       <c r="H639" t="inlineStr">
@@ -36348,7 +36348,7 @@
       </c>
       <c r="G641" t="inlineStr">
         <is>
-          <t>0x16e7</t>
+          <t>0x16ef</t>
         </is>
       </c>
       <c r="H641" t="inlineStr">
@@ -36519,7 +36519,7 @@
       </c>
       <c r="G644" t="inlineStr">
         <is>
-          <t>0x3263</t>
+          <t>0x326b</t>
         </is>
       </c>
       <c r="H644" t="inlineStr">
@@ -36633,7 +36633,7 @@
       </c>
       <c r="G646" t="inlineStr">
         <is>
-          <t>0x14e7</t>
+          <t>0x14ef</t>
         </is>
       </c>
       <c r="H646" t="inlineStr">
@@ -36747,7 +36747,7 @@
       </c>
       <c r="G648" t="inlineStr">
         <is>
-          <t>0x32e3</t>
+          <t>0x32eb</t>
         </is>
       </c>
       <c r="H648" t="inlineStr">
@@ -36975,7 +36975,7 @@
       </c>
       <c r="G652" t="inlineStr">
         <is>
-          <t>0x36e7</t>
+          <t>0x36ef</t>
         </is>
       </c>
       <c r="H652" t="inlineStr">
@@ -37089,7 +37089,7 @@
       </c>
       <c r="G654" t="inlineStr">
         <is>
-          <t>0x10e7</t>
+          <t>0x11ef</t>
         </is>
       </c>
       <c r="H654" t="inlineStr">
@@ -37146,7 +37146,7 @@
       </c>
       <c r="G655" t="inlineStr">
         <is>
-          <t>0x12e7</t>
+          <t>0x12ef</t>
         </is>
       </c>
       <c r="H655" t="inlineStr">
@@ -37203,7 +37203,7 @@
       </c>
       <c r="G656" t="inlineStr">
         <is>
-          <t>0x12e7</t>
+          <t>0x12ef</t>
         </is>
       </c>
       <c r="H656" t="inlineStr">
@@ -37317,7 +37317,7 @@
       </c>
       <c r="G658" t="inlineStr">
         <is>
-          <t>0x34e2</t>
+          <t>0x35f2</t>
         </is>
       </c>
       <c r="H658" t="inlineStr">
@@ -37431,7 +37431,7 @@
       </c>
       <c r="G660" t="inlineStr">
         <is>
-          <t>0x36e6</t>
+          <t>0x36ee</t>
         </is>
       </c>
       <c r="H660" t="inlineStr">
@@ -37545,7 +37545,7 @@
       </c>
       <c r="G662" t="inlineStr">
         <is>
-          <t>0x36e6</t>
+          <t>0x36f6</t>
         </is>
       </c>
       <c r="H662" t="inlineStr">
@@ -38001,7 +38001,7 @@
       </c>
       <c r="G670" t="inlineStr">
         <is>
-          <t>0x11e2</t>
+          <t>0x11ea</t>
         </is>
       </c>
       <c r="H670" t="inlineStr">
@@ -38172,7 +38172,7 @@
       </c>
       <c r="G673" t="inlineStr">
         <is>
-          <t>0x31e2</t>
+          <t>0x31ea</t>
         </is>
       </c>
       <c r="H673" t="inlineStr">
@@ -38343,7 +38343,7 @@
       </c>
       <c r="G676" t="inlineStr">
         <is>
-          <t>0x35e6</t>
+          <t>0x35ee</t>
         </is>
       </c>
       <c r="H676" t="inlineStr">
@@ -38457,7 +38457,7 @@
       </c>
       <c r="G678" t="inlineStr">
         <is>
-          <t>0x12e6</t>
+          <t>0x1aee</t>
         </is>
       </c>
       <c r="H678" t="inlineStr">
@@ -38571,7 +38571,7 @@
       </c>
       <c r="G680" t="inlineStr">
         <is>
-          <t>0x12e6</t>
+          <t>0x1aee</t>
         </is>
       </c>
       <c r="H680" t="inlineStr">
@@ -38628,7 +38628,7 @@
       </c>
       <c r="G681" t="inlineStr">
         <is>
-          <t>0x36e6</t>
+          <t>0x36ee</t>
         </is>
       </c>
       <c r="H681" t="inlineStr">
@@ -38685,7 +38685,7 @@
       </c>
       <c r="G682" t="inlineStr">
         <is>
-          <t>0x3162</t>
+          <t>0x316a</t>
         </is>
       </c>
       <c r="H682" t="inlineStr">
@@ -39198,7 +39198,7 @@
       </c>
       <c r="G691" t="inlineStr">
         <is>
-          <t>0x1666</t>
+          <t>0x177e</t>
         </is>
       </c>
       <c r="H691" t="inlineStr">
@@ -71527,7 +71527,7 @@
         <v>7827</v>
       </c>
       <c r="G1278" t="n">
-        <v>15263</v>
+        <v>8990</v>
       </c>
       <c r="H1278" t="inlineStr">
         <is>
@@ -71580,7 +71580,7 @@
         <v>363</v>
       </c>
       <c r="G1279" t="n">
-        <v>613</v>
+        <v>363</v>
       </c>
       <c r="H1279" t="inlineStr">
         <is>
@@ -71633,7 +71633,7 @@
         <v>132</v>
       </c>
       <c r="G1280" t="n">
-        <v>223</v>
+        <v>140</v>
       </c>
       <c r="H1280" t="inlineStr">
         <is>
@@ -72799,7 +72799,7 @@
         <v>2673</v>
       </c>
       <c r="G1302" t="n">
-        <v>5212</v>
+        <v>3100</v>
       </c>
       <c r="H1302" t="inlineStr">
         <is>
@@ -72852,7 +72852,7 @@
         <v>313</v>
       </c>
       <c r="G1303" t="n">
-        <v>529</v>
+        <v>335</v>
       </c>
       <c r="H1303" t="inlineStr">
         <is>
@@ -72905,7 +72905,7 @@
         <v>108</v>
       </c>
       <c r="G1304" t="n">
-        <v>183</v>
+        <v>115</v>
       </c>
       <c r="H1304" t="inlineStr">
         <is>
@@ -74548,7 +74548,7 @@
         <v>5871</v>
       </c>
       <c r="G1335" t="n">
-        <v>11448</v>
+        <v>6750</v>
       </c>
       <c r="H1335" t="inlineStr">
         <is>
@@ -74601,7 +74601,7 @@
         <v>348</v>
       </c>
       <c r="G1336" t="n">
-        <v>588</v>
+        <v>360</v>
       </c>
       <c r="H1336" t="inlineStr">
         <is>
@@ -74654,7 +74654,7 @@
         <v>128</v>
       </c>
       <c r="G1337" t="n">
-        <v>216</v>
+        <v>135</v>
       </c>
       <c r="H1337" t="inlineStr">
         <is>
@@ -78284,6 +78284,59 @@
         </is>
       </c>
       <c r="L1403" t="inlineStr">
+        <is>
+          <t>decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="inlineStr">
+        <is>
+          <t>W042</t>
+        </is>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr">
+        <is>
+          <t>744 Slave's Torc</t>
+        </is>
+      </c>
+      <c r="D1404" t="inlineStr">
+        <is>
+          <t>Enchant 3 (0x68)</t>
+        </is>
+      </c>
+      <c r="F1404" t="n">
+        <v>66</v>
+      </c>
+      <c r="G1404" t="n">
+        <v>275</v>
+      </c>
+      <c r="H1404" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="I1404" t="inlineStr">
+        <is>
+          <t>F92</t>
+        </is>
+      </c>
+      <c r="J1404" t="inlineStr">
+        <is>
+          <t>Slave Torc Double EXP training gear (JP community QoL parity)</t>
+        </is>
+      </c>
+      <c r="K1404" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1404" t="inlineStr">
         <is>
           <t>decided</t>
         </is>

</xml_diff>

<commit_message>
balance(stage 15): common enemies HP x1.20 with vanilla ATK and INT
common enemies HP x1.20 with vanilla ATK and INT; regenerate the
difficulty curve

Rows G034 - G093 measured again with the policy of today and a
reproducible simulator (rows of eight random battles, 24 rows, floors
St15_1120 and St15_1150, the reference party and the five battery
parties; mean battles won against vanilla over twelve cells):

 no change +0.8 easier than vanilla in 11 cells rows of 2026-10-09
(x1.30; three x1.95/1.69) -1.1 harder in 11 cells, Mage-Heavy 7.1 to 3.7
HP, ATK and INT x1.10 -0.2 Mage-Heavy 7.1 to 5.0 HP x1.20, ATK and INT
of vanilla +0.15 largest gap 1.2

The 20 hp rows are HP x1.20; the 40 atk and int rows are dropped. Attack
is subtracted from defence, so a factor on ATK had made Macha (613) and
Highway Star (588) hit above the last boss (378) and fell any member in
one hit.

DIFFICULTY_CURVE.md regenerated by tools/difficulty_curve.py: 32 of 44
within, 12 easier, 0 harder.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -71527,7 +71527,7 @@
         <v>7827</v>
       </c>
       <c r="G1278" t="n">
-        <v>8990</v>
+        <v>9392</v>
       </c>
       <c r="H1278" t="inlineStr">
         <is>
@@ -71541,12 +71541,12 @@
       </c>
       <c r="J1278" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1278" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1278" t="inlineStr">
@@ -71594,7 +71594,7 @@
       </c>
       <c r="J1279" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1279" t="inlineStr">
@@ -71604,7 +71604,7 @@
       </c>
       <c r="L1279" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -71647,7 +71647,7 @@
       </c>
       <c r="J1280" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1280" t="inlineStr">
@@ -71657,7 +71657,7 @@
       </c>
       <c r="L1280" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -71686,7 +71686,7 @@
         <v>1531</v>
       </c>
       <c r="G1281" t="n">
-        <v>1990</v>
+        <v>1837</v>
       </c>
       <c r="H1281" t="inlineStr">
         <is>
@@ -71700,12 +71700,12 @@
       </c>
       <c r="J1281" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1281" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1281" t="inlineStr">
@@ -71753,7 +71753,7 @@
       </c>
       <c r="J1282" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1282" t="inlineStr">
@@ -71763,7 +71763,7 @@
       </c>
       <c r="L1282" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -71806,7 +71806,7 @@
       </c>
       <c r="J1283" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1283" t="inlineStr">
@@ -71816,7 +71816,7 @@
       </c>
       <c r="L1283" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -71845,7 +71845,7 @@
         <v>1544</v>
       </c>
       <c r="G1284" t="n">
-        <v>2007</v>
+        <v>1853</v>
       </c>
       <c r="H1284" t="inlineStr">
         <is>
@@ -71859,12 +71859,12 @@
       </c>
       <c r="J1284" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1284" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1284" t="inlineStr">
@@ -71912,7 +71912,7 @@
       </c>
       <c r="J1285" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1285" t="inlineStr">
@@ -71922,7 +71922,7 @@
       </c>
       <c r="L1285" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -71965,7 +71965,7 @@
       </c>
       <c r="J1286" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1286" t="inlineStr">
@@ -71975,7 +71975,7 @@
       </c>
       <c r="L1286" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72004,7 +72004,7 @@
         <v>2397</v>
       </c>
       <c r="G1287" t="n">
-        <v>3116</v>
+        <v>2876</v>
       </c>
       <c r="H1287" t="inlineStr">
         <is>
@@ -72018,12 +72018,12 @@
       </c>
       <c r="J1287" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1287" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1287" t="inlineStr">
@@ -72071,7 +72071,7 @@
       </c>
       <c r="J1288" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1288" t="inlineStr">
@@ -72081,7 +72081,7 @@
       </c>
       <c r="L1288" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72124,7 +72124,7 @@
       </c>
       <c r="J1289" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1289" t="inlineStr">
@@ -72134,7 +72134,7 @@
       </c>
       <c r="L1289" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72163,7 +72163,7 @@
         <v>1683</v>
       </c>
       <c r="G1290" t="n">
-        <v>2188</v>
+        <v>2020</v>
       </c>
       <c r="H1290" t="inlineStr">
         <is>
@@ -72177,12 +72177,12 @@
       </c>
       <c r="J1290" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1290" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1290" t="inlineStr">
@@ -72230,7 +72230,7 @@
       </c>
       <c r="J1291" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1291" t="inlineStr">
@@ -72240,7 +72240,7 @@
       </c>
       <c r="L1291" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72283,7 +72283,7 @@
       </c>
       <c r="J1292" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1292" t="inlineStr">
@@ -72293,7 +72293,7 @@
       </c>
       <c r="L1292" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72322,7 +72322,7 @@
         <v>1745</v>
       </c>
       <c r="G1293" t="n">
-        <v>2268</v>
+        <v>2094</v>
       </c>
       <c r="H1293" t="inlineStr">
         <is>
@@ -72336,12 +72336,12 @@
       </c>
       <c r="J1293" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1293" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1293" t="inlineStr">
@@ -72389,7 +72389,7 @@
       </c>
       <c r="J1294" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1294" t="inlineStr">
@@ -72399,7 +72399,7 @@
       </c>
       <c r="L1294" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72442,7 +72442,7 @@
       </c>
       <c r="J1295" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1295" t="inlineStr">
@@ -72452,7 +72452,7 @@
       </c>
       <c r="L1295" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72481,7 +72481,7 @@
         <v>1475</v>
       </c>
       <c r="G1296" t="n">
-        <v>1918</v>
+        <v>1770</v>
       </c>
       <c r="H1296" t="inlineStr">
         <is>
@@ -72495,12 +72495,12 @@
       </c>
       <c r="J1296" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1296" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1296" t="inlineStr">
@@ -72548,7 +72548,7 @@
       </c>
       <c r="J1297" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1297" t="inlineStr">
@@ -72558,7 +72558,7 @@
       </c>
       <c r="L1297" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72601,7 +72601,7 @@
       </c>
       <c r="J1298" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1298" t="inlineStr">
@@ -72611,7 +72611,7 @@
       </c>
       <c r="L1298" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72640,7 +72640,7 @@
         <v>1542</v>
       </c>
       <c r="G1299" t="n">
-        <v>2005</v>
+        <v>1850</v>
       </c>
       <c r="H1299" t="inlineStr">
         <is>
@@ -72654,12 +72654,12 @@
       </c>
       <c r="J1299" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1299" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1299" t="inlineStr">
@@ -72707,7 +72707,7 @@
       </c>
       <c r="J1300" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1300" t="inlineStr">
@@ -72717,7 +72717,7 @@
       </c>
       <c r="L1300" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72760,7 +72760,7 @@
       </c>
       <c r="J1301" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1301" t="inlineStr">
@@ -72770,7 +72770,7 @@
       </c>
       <c r="L1301" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72799,7 +72799,7 @@
         <v>2673</v>
       </c>
       <c r="G1302" t="n">
-        <v>3100</v>
+        <v>3208</v>
       </c>
       <c r="H1302" t="inlineStr">
         <is>
@@ -72813,12 +72813,12 @@
       </c>
       <c r="J1302" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1302" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1302" t="inlineStr">
@@ -72866,7 +72866,7 @@
       </c>
       <c r="J1303" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1303" t="inlineStr">
@@ -72876,7 +72876,7 @@
       </c>
       <c r="L1303" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72919,7 +72919,7 @@
       </c>
       <c r="J1304" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1304" t="inlineStr">
@@ -72929,7 +72929,7 @@
       </c>
       <c r="L1304" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -72958,7 +72958,7 @@
         <v>1631</v>
       </c>
       <c r="G1305" t="n">
-        <v>2120</v>
+        <v>1957</v>
       </c>
       <c r="H1305" t="inlineStr">
         <is>
@@ -72972,12 +72972,12 @@
       </c>
       <c r="J1305" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1305" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1305" t="inlineStr">
@@ -73025,7 +73025,7 @@
       </c>
       <c r="J1306" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1306" t="inlineStr">
@@ -73035,7 +73035,7 @@
       </c>
       <c r="L1306" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73078,7 +73078,7 @@
       </c>
       <c r="J1307" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1307" t="inlineStr">
@@ -73088,7 +73088,7 @@
       </c>
       <c r="L1307" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73117,7 +73117,7 @@
         <v>1643</v>
       </c>
       <c r="G1308" t="n">
-        <v>2136</v>
+        <v>1972</v>
       </c>
       <c r="H1308" t="inlineStr">
         <is>
@@ -73131,12 +73131,12 @@
       </c>
       <c r="J1308" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1308" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1308" t="inlineStr">
@@ -73184,7 +73184,7 @@
       </c>
       <c r="J1309" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1309" t="inlineStr">
@@ -73194,7 +73194,7 @@
       </c>
       <c r="L1309" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73237,7 +73237,7 @@
       </c>
       <c r="J1310" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1310" t="inlineStr">
@@ -73247,7 +73247,7 @@
       </c>
       <c r="L1310" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73276,7 +73276,7 @@
         <v>1668</v>
       </c>
       <c r="G1311" t="n">
-        <v>2168</v>
+        <v>2002</v>
       </c>
       <c r="H1311" t="inlineStr">
         <is>
@@ -73290,12 +73290,12 @@
       </c>
       <c r="J1311" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1311" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1311" t="inlineStr">
@@ -73343,7 +73343,7 @@
       </c>
       <c r="J1312" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1312" t="inlineStr">
@@ -73353,7 +73353,7 @@
       </c>
       <c r="L1312" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73396,7 +73396,7 @@
       </c>
       <c r="J1313" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1313" t="inlineStr">
@@ -73406,7 +73406,7 @@
       </c>
       <c r="L1313" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73435,7 +73435,7 @@
         <v>1729</v>
       </c>
       <c r="G1314" t="n">
-        <v>2248</v>
+        <v>2075</v>
       </c>
       <c r="H1314" t="inlineStr">
         <is>
@@ -73449,12 +73449,12 @@
       </c>
       <c r="J1314" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1314" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1314" t="inlineStr">
@@ -73502,7 +73502,7 @@
       </c>
       <c r="J1315" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1315" t="inlineStr">
@@ -73512,7 +73512,7 @@
       </c>
       <c r="L1315" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73555,7 +73555,7 @@
       </c>
       <c r="J1316" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1316" t="inlineStr">
@@ -73565,7 +73565,7 @@
       </c>
       <c r="L1316" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73594,7 +73594,7 @@
         <v>3042</v>
       </c>
       <c r="G1317" t="n">
-        <v>3955</v>
+        <v>3650</v>
       </c>
       <c r="H1317" t="inlineStr">
         <is>
@@ -73608,12 +73608,12 @@
       </c>
       <c r="J1317" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1317" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1317" t="inlineStr">
@@ -73661,7 +73661,7 @@
       </c>
       <c r="J1318" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1318" t="inlineStr">
@@ -73671,7 +73671,7 @@
       </c>
       <c r="L1318" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73714,7 +73714,7 @@
       </c>
       <c r="J1319" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1319" t="inlineStr">
@@ -73724,7 +73724,7 @@
       </c>
       <c r="L1319" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73753,7 +73753,7 @@
         <v>1559</v>
       </c>
       <c r="G1320" t="n">
-        <v>2027</v>
+        <v>1871</v>
       </c>
       <c r="H1320" t="inlineStr">
         <is>
@@ -73767,12 +73767,12 @@
       </c>
       <c r="J1320" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1320" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1320" t="inlineStr">
@@ -73820,7 +73820,7 @@
       </c>
       <c r="J1321" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1321" t="inlineStr">
@@ -73830,7 +73830,7 @@
       </c>
       <c r="L1321" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73873,7 +73873,7 @@
       </c>
       <c r="J1322" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1322" t="inlineStr">
@@ -73883,7 +73883,7 @@
       </c>
       <c r="L1322" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -73912,7 +73912,7 @@
         <v>1203</v>
       </c>
       <c r="G1323" t="n">
-        <v>1564</v>
+        <v>1444</v>
       </c>
       <c r="H1323" t="inlineStr">
         <is>
@@ -73926,12 +73926,12 @@
       </c>
       <c r="J1323" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1323" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1323" t="inlineStr">
@@ -73979,7 +73979,7 @@
       </c>
       <c r="J1324" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1324" t="inlineStr">
@@ -73989,7 +73989,7 @@
       </c>
       <c r="L1324" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -74032,7 +74032,7 @@
       </c>
       <c r="J1325" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1325" t="inlineStr">
@@ -74042,7 +74042,7 @@
       </c>
       <c r="L1325" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -74071,7 +74071,7 @@
         <v>1411</v>
       </c>
       <c r="G1326" t="n">
-        <v>1834</v>
+        <v>1693</v>
       </c>
       <c r="H1326" t="inlineStr">
         <is>
@@ -74085,12 +74085,12 @@
       </c>
       <c r="J1326" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1326" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1326" t="inlineStr">
@@ -74138,7 +74138,7 @@
       </c>
       <c r="J1327" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1327" t="inlineStr">
@@ -74148,7 +74148,7 @@
       </c>
       <c r="L1327" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -74191,7 +74191,7 @@
       </c>
       <c r="J1328" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1328" t="inlineStr">
@@ -74201,7 +74201,7 @@
       </c>
       <c r="L1328" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -74230,7 +74230,7 @@
         <v>4675</v>
       </c>
       <c r="G1329" t="n">
-        <v>6078</v>
+        <v>5610</v>
       </c>
       <c r="H1329" t="inlineStr">
         <is>
@@ -74244,12 +74244,12 @@
       </c>
       <c r="J1329" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1329" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1329" t="inlineStr">
@@ -74297,7 +74297,7 @@
       </c>
       <c r="J1330" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1330" t="inlineStr">
@@ -74307,7 +74307,7 @@
       </c>
       <c r="L1330" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -74350,7 +74350,7 @@
       </c>
       <c r="J1331" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1331" t="inlineStr">
@@ -74360,7 +74360,7 @@
       </c>
       <c r="L1331" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -74389,7 +74389,7 @@
         <v>1811</v>
       </c>
       <c r="G1332" t="n">
-        <v>2354</v>
+        <v>2173</v>
       </c>
       <c r="H1332" t="inlineStr">
         <is>
@@ -74403,12 +74403,12 @@
       </c>
       <c r="J1332" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1332" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1332" t="inlineStr">
@@ -74456,7 +74456,7 @@
       </c>
       <c r="J1333" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1333" t="inlineStr">
@@ -74466,7 +74466,7 @@
       </c>
       <c r="L1333" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -74509,7 +74509,7 @@
       </c>
       <c r="J1334" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1334" t="inlineStr">
@@ -74519,7 +74519,7 @@
       </c>
       <c r="L1334" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -74548,7 +74548,7 @@
         <v>5871</v>
       </c>
       <c r="G1335" t="n">
-        <v>6750</v>
+        <v>7045</v>
       </c>
       <c r="H1335" t="inlineStr">
         <is>
@@ -74562,12 +74562,12 @@
       </c>
       <c r="J1335" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Difficulty kept on the common fights of the last floors (R08, R10), measured again on 2026-10-11 with the policy of today, the reference party and the five battery parties (scratch/audit_2026-10-11/e7_stage15_fit.py, rows of eight random battles, 24 rows, floors St15_1120 and St15_1150; mean battles won against vanilla over the twelve cells): with no change the variant is easier (+0.8); HP, ATK and INT x1.30 with x1.95 / x1.69 on three enemies, the rows of 2026-10-09, made it harder for every party but one (-1.1; Mage-Heavy 7.1 to 3.7 on St15_1150) because attack is subtracted from defence and x1.69 ATK was x2 to x3.3 damage, a common enemy above the ATK of the last boss; HP x1.20 alone gives +0.15, the largest gap 1.2 battles, and no hit grows. HP x1.20, ATK and INT of vanilla</t>
         </is>
       </c>
       <c r="K1335" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1335" t="inlineStr">
@@ -74615,7 +74615,7 @@
       </c>
       <c r="J1336" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1336" t="inlineStr">
@@ -74625,7 +74625,7 @@
       </c>
       <c r="L1336" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -74668,7 +74668,7 @@
       </c>
       <c r="J1337" t="inlineStr">
         <is>
-          <t>Difficulty kept on the common fights (R08, R10; the user: harden everything within the windows of vanilla): rows of eight random battles on the floors of C39 and C40 had become far easier on the variant (C39: 4.9 battles won and 8% HP left in vanilla, 6.6 and 50% on the variant; C40: 5.3 and 42%, 7.5 and 92%) through the stronger party. HP, ATK and INT x1.30 for the common enemies of the two floors, x1.95 HP and x1.69 ATK and INT for Macha, Purski and Highway Star, found only on the C40 floor of the two: C39 4.2 and 17%, C40 5.4 and 42% after (24 rows each)</t>
+          <t>Dropped on 2026-10-11: ATK and INT of the common enemies of Stage 15 stay at vanilla. See the hp row of the same enemy: the measure of today is met by HP alone, and a factor on attack multiplied the damage by far more than its figure</t>
         </is>
       </c>
       <c r="K1337" t="inlineStr">
@@ -74678,7 +74678,7 @@
       </c>
       <c r="L1337" t="inlineStr">
         <is>
-          <t>decided</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: B4 alone decided; the drop rows corrected on the reading of the
B4 alone decided; the drop rows corrected on the reading of the slots,
1,363 of 1,363 live rows built

The kept curve is not built (decided 2026-10-11): the register and the
plan carry the figures of B4 alone. EnemyStatusData 0x80 is the count of
equipment slots: the thirteen bosses of P011 - P023 give their piece for
certain and Ryoma's falls at the usual rate, 14 rows dropped. Seven
fixed pieces of common enemies under 2% get the weight that gives 2%
(new field "equipment slot N weight", written, read back and compared
with the simulator). exe_patch leaves a file alone when it already
carries the set.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1457"/>
+  <dimension ref="A1:L1463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75340,7 +75340,7 @@
       </c>
       <c r="J1349" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame boss rarest equipment drop rate gently raised from 1% to 3% to alleviate excessive reload grinding.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1349" t="inlineStr">
@@ -75350,7 +75350,7 @@
       </c>
       <c r="L1349" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75393,7 +75393,7 @@
       </c>
       <c r="J1350" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame boss rarest equipment drop rate gently raised from 1% to 3% to alleviate excessive reload grinding.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1350" t="inlineStr">
@@ -75403,7 +75403,7 @@
       </c>
       <c r="L1350" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75446,7 +75446,7 @@
       </c>
       <c r="J1351" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame superboss rarest equipment drop rate gently raised from 1% to 3%.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1351" t="inlineStr">
@@ -75456,7 +75456,7 @@
       </c>
       <c r="L1351" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75499,7 +75499,7 @@
       </c>
       <c r="J1352" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame superboss rarest equipment drop rate gently raised from 1% to 3%.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1352" t="inlineStr">
@@ -75509,7 +75509,7 @@
       </c>
       <c r="L1352" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75552,7 +75552,7 @@
       </c>
       <c r="J1353" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame superboss rarest equipment drop rate gently raised from 1% to 3%.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1353" t="inlineStr">
@@ -75562,7 +75562,7 @@
       </c>
       <c r="L1353" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75605,7 +75605,7 @@
       </c>
       <c r="J1354" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame superboss rarest equipment drop rate gently raised from 1% to 3%.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1354" t="inlineStr">
@@ -75615,7 +75615,7 @@
       </c>
       <c r="L1354" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75658,7 +75658,7 @@
       </c>
       <c r="J1355" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1355" t="inlineStr">
@@ -75668,7 +75668,7 @@
       </c>
       <c r="L1355" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75711,7 +75711,7 @@
       </c>
       <c r="J1356" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1356" t="inlineStr">
@@ -75721,7 +75721,7 @@
       </c>
       <c r="L1356" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75764,7 +75764,7 @@
       </c>
       <c r="J1357" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1357" t="inlineStr">
@@ -75774,7 +75774,7 @@
       </c>
       <c r="L1357" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75817,7 +75817,7 @@
       </c>
       <c r="J1358" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1358" t="inlineStr">
@@ -75827,7 +75827,7 @@
       </c>
       <c r="L1358" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75870,7 +75870,7 @@
       </c>
       <c r="J1359" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1359" t="inlineStr">
@@ -75880,7 +75880,7 @@
       </c>
       <c r="L1359" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75923,7 +75923,7 @@
       </c>
       <c r="J1360" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1360" t="inlineStr">
@@ -75933,7 +75933,7 @@
       </c>
       <c r="L1360" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -75976,7 +75976,7 @@
       </c>
       <c r="J1361" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Postgame rare equipment drop rate gently raised from 2% to 5%.</t>
+          <t>Dropped on 2026-10-11: the piece of this boss is already certain in vanilla. Its record holds a drop chance of 100 (0x7C), no item, and one slot (0x80 = 1) that names the piece with weight 100 (0x8C); the word the row changed is that count of slots, not a chance (0x558517; scratch/drops_reading.md).</t>
         </is>
       </c>
       <c r="K1361" t="inlineStr">
@@ -75986,7 +75986,7 @@
       </c>
       <c r="L1361" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -76008,14 +76008,14 @@
       </c>
       <c r="D1362" t="inlineStr">
         <is>
-          <t>equipment drop rate</t>
+          <t>equipment slot 1 weight (piece 339)</t>
         </is>
       </c>
       <c r="F1362" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G1362" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H1362" t="inlineStr">
         <is>
@@ -76029,17 +76029,17 @@
       </c>
       <c r="J1362" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Rare equipment drop rate gently raised from 2% to 5%.</t>
+          <t>The fixed pieces of common enemies fall 2 to 4.5% of the time; seven fall under 2%, this one 0.80%: chance of the equipment drop 16 (0x7C) times its weight 5 of 100 (0x558570 - 0x5585a8). Raised to the lowest weight that gives 2%: 2.06%. The weights of the other slots are not touched. Reading: scratch/drops_reading.md, checked on 2026-10-11.</t>
         </is>
       </c>
       <c r="K1362" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="L1362" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>built</t>
         </is>
       </c>
     </row>
@@ -76082,7 +76082,7 @@
       </c>
       <c r="J1363" t="inlineStr">
         <is>
-          <t>Blocked on 2026-10-11: the word the row means is EnemyStatusData 0x80, which is not a chance: it is how many pieces the drop draws (0x558517 allocates that many; 0 to 3 over the 516 enemies), and the chance of the drop is 0x7C, already 100 for these bosses (16 for Garasha and Ryoma). 5 is outside what the game holds. To decide: the count (3 at most), or nothing. Was: Rare equipment drop rate gently raised from 2% to 5%.</t>
+          <t>Dropped on 2026-10-11: the word the row changed is the count of slots. The Sudarshana of Ryoma falls 3.2% of the time (chance 16, weight 20 of 100), which is what a fixed piece of a common enemy falls at across the game (2 to 4.5%).</t>
         </is>
       </c>
       <c r="K1363" t="inlineStr">
@@ -76092,7 +76092,7 @@
       </c>
       <c r="L1363" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>
@@ -81158,6 +81158,324 @@
         </is>
       </c>
       <c r="L1457" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" t="inlineStr">
+        <is>
+          <t>P079</t>
+        </is>
+      </c>
+      <c r="B1458" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1458" t="inlineStr">
+        <is>
+          <t>212 Cat's Eye</t>
+        </is>
+      </c>
+      <c r="D1458" t="inlineStr">
+        <is>
+          <t>equipment slot 1 weight (piece 656)</t>
+        </is>
+      </c>
+      <c r="F1458" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1458" t="n">
+        <v>17</v>
+      </c>
+      <c r="H1458" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1458" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1458" t="inlineStr">
+        <is>
+          <t>The fixed pieces of common enemies fall 2 to 4.5% of the time; seven fall under 2%, this one 0.91%: chance of the equipment drop 13 (0x7C) times its weight 7 of 100 (0x558570 - 0x5585a8). Raised to the lowest weight that gives 2%: 2.01%. The weights of the other slots are not touched. Reading: scratch/drops_reading.md, checked on 2026-10-11.</t>
+        </is>
+      </c>
+      <c r="K1458" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1458" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" t="inlineStr">
+        <is>
+          <t>P080</t>
+        </is>
+      </c>
+      <c r="B1459" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1459" t="inlineStr">
+        <is>
+          <t>732 Knuckle Saint</t>
+        </is>
+      </c>
+      <c r="D1459" t="inlineStr">
+        <is>
+          <t>equipment slot 2 weight (piece 761)</t>
+        </is>
+      </c>
+      <c r="F1459" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1459" t="n">
+        <v>15</v>
+      </c>
+      <c r="H1459" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1459" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1459" t="inlineStr">
+        <is>
+          <t>The fixed pieces of common enemies fall 2 to 4.5% of the time; seven fall under 2%, this one 0.90%: chance of the equipment drop 15 (0x7C) times its weight 6 of 100 (0x558570 - 0x5585a8). Raised to the lowest weight that gives 2%: 2.06%. The weights of the other slots are not touched. Reading: scratch/drops_reading.md, checked on 2026-10-11.</t>
+        </is>
+      </c>
+      <c r="K1459" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1459" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" t="inlineStr">
+        <is>
+          <t>P081</t>
+        </is>
+      </c>
+      <c r="B1460" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1460" t="inlineStr">
+        <is>
+          <t>236 Thor</t>
+        </is>
+      </c>
+      <c r="D1460" t="inlineStr">
+        <is>
+          <t>equipment slot 1 weight (piece 223)</t>
+        </is>
+      </c>
+      <c r="F1460" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1460" t="n">
+        <v>14</v>
+      </c>
+      <c r="H1460" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1460" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1460" t="inlineStr">
+        <is>
+          <t>The fixed pieces of common enemies fall 2 to 4.5% of the time; seven fall under 2%, this one 1.02%: chance of the equipment drop 17 (0x7C) times its weight 6 of 100 (0x558570 - 0x5585a8). Raised to the lowest weight that gives 2%: 2.09%. The weights of the other slots are not touched. Reading: scratch/drops_reading.md, checked on 2026-10-11.</t>
+        </is>
+      </c>
+      <c r="K1460" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1460" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" t="inlineStr">
+        <is>
+          <t>P082</t>
+        </is>
+      </c>
+      <c r="B1461" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1461" t="inlineStr">
+        <is>
+          <t>236 Thor</t>
+        </is>
+      </c>
+      <c r="D1461" t="inlineStr">
+        <is>
+          <t>equipment slot 2 weight (piece 764)</t>
+        </is>
+      </c>
+      <c r="F1461" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1461" t="n">
+        <v>14</v>
+      </c>
+      <c r="H1461" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1461" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1461" t="inlineStr">
+        <is>
+          <t>The fixed pieces of common enemies fall 2 to 4.5% of the time; seven fall under 2%, this one 1.36%: chance of the equipment drop 17 (0x7C) times its weight 8 of 100 (0x558570 - 0x5585a8). Raised to the lowest weight that gives 2%: 2.09%. The weights of the other slots are not touched. Reading: scratch/drops_reading.md, checked on 2026-10-11.</t>
+        </is>
+      </c>
+      <c r="K1461" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1461" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" t="inlineStr">
+        <is>
+          <t>P083</t>
+        </is>
+      </c>
+      <c r="B1462" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1462" t="inlineStr">
+        <is>
+          <t>933 Peach Jam</t>
+        </is>
+      </c>
+      <c r="D1462" t="inlineStr">
+        <is>
+          <t>equipment slot 1 weight (piece 643)</t>
+        </is>
+      </c>
+      <c r="F1462" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1462" t="n">
+        <v>29</v>
+      </c>
+      <c r="H1462" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1462" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1462" t="inlineStr">
+        <is>
+          <t>The fixed pieces of common enemies fall 2 to 4.5% of the time; seven fall under 2%, this one 1.20%: chance of the equipment drop 8 (0x7C) times its weight 15 of 100 (0x558570 - 0x5585a8). Raised to the lowest weight that gives 2%: 2.04%. The weights of the other slots are not touched. Reading: scratch/drops_reading.md, checked on 2026-10-11.</t>
+        </is>
+      </c>
+      <c r="K1462" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1462" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" t="inlineStr">
+        <is>
+          <t>P084</t>
+        </is>
+      </c>
+      <c r="B1463" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1463" t="inlineStr">
+        <is>
+          <t>65 Shanina</t>
+        </is>
+      </c>
+      <c r="D1463" t="inlineStr">
+        <is>
+          <t>equipment slot 2 weight (piece 340)</t>
+        </is>
+      </c>
+      <c r="F1463" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1463" t="n">
+        <v>9</v>
+      </c>
+      <c r="H1463" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1463" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1463" t="inlineStr">
+        <is>
+          <t>The fixed pieces of common enemies fall 2 to 4.5% of the time; seven fall under 2%, this one 1.50%: chance of the equipment drop 25 (0x7C) times its weight 6 of 100 (0x558570 - 0x5585a8). Raised to the lowest weight that gives 2%: 2.18%. The weights of the other slots are not touched. Reading: scratch/drops_reading.md, checked on 2026-10-11.</t>
+        </is>
+      </c>
+      <c r="K1463" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1463" t="inlineStr">
         <is>
           <t>built</t>
         </is>

</xml_diff>

<commit_message>
balance: proposed, not built: the forge rate of the Tantou doubled and
proposed, not built: the forge rate of the Tantou doubled and Danger
Shoot +0.10, measured on classes and curve

Rows W045 and Y001 - Y010 in the state proposed. With them the Kunoichi
(1.31 to 1.10) and the Trickster (1.19 and 1.22 to 1.11 and 1.15) come
into the band and the difficulty curve does not move (37 of 44 within, 7
easier). The Dagger and the Kukri are left alone: at twice their rate
the reference party, which holds a Treasure Hunter, makes 17 bosses
easier than vanilla. BALANCE_PROPOSED=1 lets any tool of the simulator
measure the proposed rows.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1463"/>
+  <dimension ref="A1:L1474"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81481,6 +81481,619 @@
         </is>
       </c>
     </row>
+    <row r="1464">
+      <c r="A1464" t="inlineStr">
+        <is>
+          <t>W045</t>
+        </is>
+      </c>
+      <c r="B1464" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C1464" t="inlineStr">
+        <is>
+          <t>356 Tantou</t>
+        </is>
+      </c>
+      <c r="D1464" t="inlineStr">
+        <is>
+          <t>upgrade rate</t>
+        </is>
+      </c>
+      <c r="F1464" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G1464" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H1464" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="I1464" t="inlineStr">
+        <is>
+          <t>F04, J27</t>
+        </is>
+      </c>
+      <c r="J1464" t="inlineStr">
+        <is>
+          <t>Proposed 2026-10-11 (classes slow at their stage: Assassin, Treasure Hunter, Kunoichi). The light blades gain 1.0 - 1.3 ATK a forge level, the swords, axes and katanas 1.6 - 3.2; damage is attack less defence (FORMULAS 2.4), so at C30 a Kunoichi (ATK 133 against a boss of DEF 162) deals 11 with a plain blow and the Treasure Hunter 4 at C40. Lever L14, as the Whip (W005)</t>
+        </is>
+      </c>
+      <c r="K1464" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1464" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" t="inlineStr">
+        <is>
+          <t>Y001</t>
+        </is>
+      </c>
+      <c r="B1465" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1465" t="inlineStr">
+        <is>
+          <t>Technique 79 Danger Shoot</t>
+        </is>
+      </c>
+      <c r="D1465" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1465" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1465" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G1465" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H1465" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1465" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="J1465" t="inlineStr">
+        <is>
+          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+        </is>
+      </c>
+      <c r="K1465" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1465" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" t="inlineStr">
+        <is>
+          <t>Y002</t>
+        </is>
+      </c>
+      <c r="B1466" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1466" t="inlineStr">
+        <is>
+          <t>Technique 79 Danger Shoot</t>
+        </is>
+      </c>
+      <c r="D1466" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1466" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1466" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G1466" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H1466" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1466" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="J1466" t="inlineStr">
+        <is>
+          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+        </is>
+      </c>
+      <c r="K1466" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1466" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" t="inlineStr">
+        <is>
+          <t>Y003</t>
+        </is>
+      </c>
+      <c r="B1467" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1467" t="inlineStr">
+        <is>
+          <t>Technique 79 Danger Shoot</t>
+        </is>
+      </c>
+      <c r="D1467" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1467" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1467" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G1467" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="H1467" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1467" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="J1467" t="inlineStr">
+        <is>
+          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+        </is>
+      </c>
+      <c r="K1467" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1467" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" t="inlineStr">
+        <is>
+          <t>Y004</t>
+        </is>
+      </c>
+      <c r="B1468" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1468" t="inlineStr">
+        <is>
+          <t>Technique 79 Danger Shoot</t>
+        </is>
+      </c>
+      <c r="D1468" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1468" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1468" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G1468" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="H1468" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1468" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="J1468" t="inlineStr">
+        <is>
+          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+        </is>
+      </c>
+      <c r="K1468" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1468" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" t="inlineStr">
+        <is>
+          <t>Y005</t>
+        </is>
+      </c>
+      <c r="B1469" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1469" t="inlineStr">
+        <is>
+          <t>Technique 79 Danger Shoot</t>
+        </is>
+      </c>
+      <c r="D1469" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1469" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1469" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G1469" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H1469" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1469" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="J1469" t="inlineStr">
+        <is>
+          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+        </is>
+      </c>
+      <c r="K1469" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1469" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" t="inlineStr">
+        <is>
+          <t>Y006</t>
+        </is>
+      </c>
+      <c r="B1470" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1470" t="inlineStr">
+        <is>
+          <t>Technique 79 Danger Shoot</t>
+        </is>
+      </c>
+      <c r="D1470" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1470" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1470" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G1470" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="H1470" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1470" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="J1470" t="inlineStr">
+        <is>
+          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+        </is>
+      </c>
+      <c r="K1470" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1470" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" t="inlineStr">
+        <is>
+          <t>Y007</t>
+        </is>
+      </c>
+      <c r="B1471" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1471" t="inlineStr">
+        <is>
+          <t>Technique 79 Danger Shoot</t>
+        </is>
+      </c>
+      <c r="D1471" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1471" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1471" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G1471" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="H1471" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1471" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="J1471" t="inlineStr">
+        <is>
+          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+        </is>
+      </c>
+      <c r="K1471" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1471" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" t="inlineStr">
+        <is>
+          <t>Y008</t>
+        </is>
+      </c>
+      <c r="B1472" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1472" t="inlineStr">
+        <is>
+          <t>Technique 79 Danger Shoot</t>
+        </is>
+      </c>
+      <c r="D1472" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1472" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1472" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G1472" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H1472" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1472" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="J1472" t="inlineStr">
+        <is>
+          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+        </is>
+      </c>
+      <c r="K1472" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1472" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" t="inlineStr">
+        <is>
+          <t>Y009</t>
+        </is>
+      </c>
+      <c r="B1473" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1473" t="inlineStr">
+        <is>
+          <t>Technique 79 Danger Shoot</t>
+        </is>
+      </c>
+      <c r="D1473" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1473" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1473" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="G1473" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="H1473" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1473" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="J1473" t="inlineStr">
+        <is>
+          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+        </is>
+      </c>
+      <c r="K1473" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1473" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" t="inlineStr">
+        <is>
+          <t>Y010</t>
+        </is>
+      </c>
+      <c r="B1474" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1474" t="inlineStr">
+        <is>
+          <t>Technique 79 Danger Shoot</t>
+        </is>
+      </c>
+      <c r="D1474" t="inlineStr">
+        <is>
+          <t>effect 26 (power)</t>
+        </is>
+      </c>
+      <c r="E1474" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1474" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G1474" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="H1474" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1474" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="J1474" t="inlineStr">
+        <is>
+          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+        </is>
+      </c>
+      <c r="K1474" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1474" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
balance: the Tantou forges at twice its rate and Danger Shoot gains 0.10
the Tantou forges at twice its rate and Danger Shoot gains 0.10, built
and installed; every measure replayed

1,374 of 1,374 live rows built. Battery 65 of 85 in vanilla and 77 of 85
on the variant, curve 37 of 44 within and 0 harder. The class measure
judges a role whose path ends in a support class as a support at every
stage: the healers leave the median of the attackers, and the Scout and
the Spieler show as slow at the base stage (65 of 76 rows). The register
and the plan carry the decisions of 2026-10-11.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -81520,7 +81520,7 @@
       </c>
       <c r="J1464" t="inlineStr">
         <is>
-          <t>Proposed 2026-10-11 (classes slow at their stage: Assassin, Treasure Hunter, Kunoichi). The light blades gain 1.0 - 1.3 ATK a forge level, the swords, axes and katanas 1.6 - 3.2; damage is attack less defence (FORMULAS 2.4), so at C30 a Kunoichi (ATK 133 against a boss of DEF 162) deals 11 with a plain blow and the Treasure Hunter 4 at C40. Lever L14, as the Whip (W005)</t>
+          <t>Decided by the user on 2026-10-11 (classes slow at their stage: Assassin, Treasure Hunter, Kunoichi). The light blades gain 1.0 - 1.3 ATK a forge level, the swords, axes and katanas 1.6 - 3.2; damage is attack less defence (FORMULAS 2.4), so at C30 a Kunoichi (ATK 133 against a boss of DEF 162) deals 11 with a plain blow and the Treasure Hunter 4 at C40. Lever L14, as the Whip (W005). Only the Tantou, the blade of the Kunoichi from level 30: with it at twice its rate she goes from 1.31 to 1.10 of the median attacker at C22, C30, C34, C40 and the difficulty curve does not move (37 of 44 within, 7 easier); the Dagger and the Kukri at twice theirs make 17 bosses easier, the reference party holding a Treasure Hunter</t>
         </is>
       </c>
       <c r="K1464" t="inlineStr">
@@ -81530,7 +81530,7 @@
       </c>
       <c r="L1464" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>built</t>
         </is>
       </c>
     </row>
@@ -81571,12 +81571,12 @@
       </c>
       <c r="I1465" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>T05 (every class at its stage; no row of the register names the Trickster)</t>
         </is>
       </c>
       <c r="J1465" t="inlineStr">
         <is>
-          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+          <t>Decided by the user on 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level. Measured: the Trickster from 1.19 and 1.22 to 1.11 and 1.15 by its two routes; +0.15 gives 1.08 and 1.14 and shortens the fights of the reference party of chapters 15 - 27 by 10 - 15%, so +0.10 is kept</t>
         </is>
       </c>
       <c r="K1465" t="inlineStr">
@@ -81586,7 +81586,7 @@
       </c>
       <c r="L1465" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>built</t>
         </is>
       </c>
     </row>
@@ -81627,12 +81627,12 @@
       </c>
       <c r="I1466" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>T05 (every class at its stage; no row of the register names the Trickster)</t>
         </is>
       </c>
       <c r="J1466" t="inlineStr">
         <is>
-          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+          <t>Decided by the user on 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level. Measured: the Trickster from 1.19 and 1.22 to 1.11 and 1.15 by its two routes; +0.15 gives 1.08 and 1.14 and shortens the fights of the reference party of chapters 15 - 27 by 10 - 15%, so +0.10 is kept</t>
         </is>
       </c>
       <c r="K1466" t="inlineStr">
@@ -81642,7 +81642,7 @@
       </c>
       <c r="L1466" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>built</t>
         </is>
       </c>
     </row>
@@ -81683,12 +81683,12 @@
       </c>
       <c r="I1467" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>T05 (every class at its stage; no row of the register names the Trickster)</t>
         </is>
       </c>
       <c r="J1467" t="inlineStr">
         <is>
-          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+          <t>Decided by the user on 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level. Measured: the Trickster from 1.19 and 1.22 to 1.11 and 1.15 by its two routes; +0.15 gives 1.08 and 1.14 and shortens the fights of the reference party of chapters 15 - 27 by 10 - 15%, so +0.10 is kept</t>
         </is>
       </c>
       <c r="K1467" t="inlineStr">
@@ -81698,7 +81698,7 @@
       </c>
       <c r="L1467" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>built</t>
         </is>
       </c>
     </row>
@@ -81739,12 +81739,12 @@
       </c>
       <c r="I1468" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>T05 (every class at its stage; no row of the register names the Trickster)</t>
         </is>
       </c>
       <c r="J1468" t="inlineStr">
         <is>
-          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+          <t>Decided by the user on 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level. Measured: the Trickster from 1.19 and 1.22 to 1.11 and 1.15 by its two routes; +0.15 gives 1.08 and 1.14 and shortens the fights of the reference party of chapters 15 - 27 by 10 - 15%, so +0.10 is kept</t>
         </is>
       </c>
       <c r="K1468" t="inlineStr">
@@ -81754,7 +81754,7 @@
       </c>
       <c r="L1468" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>built</t>
         </is>
       </c>
     </row>
@@ -81795,12 +81795,12 @@
       </c>
       <c r="I1469" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>T05 (every class at its stage; no row of the register names the Trickster)</t>
         </is>
       </c>
       <c r="J1469" t="inlineStr">
         <is>
-          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+          <t>Decided by the user on 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level. Measured: the Trickster from 1.19 and 1.22 to 1.11 and 1.15 by its two routes; +0.15 gives 1.08 and 1.14 and shortens the fights of the reference party of chapters 15 - 27 by 10 - 15%, so +0.10 is kept</t>
         </is>
       </c>
       <c r="K1469" t="inlineStr">
@@ -81810,7 +81810,7 @@
       </c>
       <c r="L1469" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>built</t>
         </is>
       </c>
     </row>
@@ -81851,12 +81851,12 @@
       </c>
       <c r="I1470" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>T05 (every class at its stage; no row of the register names the Trickster)</t>
         </is>
       </c>
       <c r="J1470" t="inlineStr">
         <is>
-          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+          <t>Decided by the user on 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level. Measured: the Trickster from 1.19 and 1.22 to 1.11 and 1.15 by its two routes; +0.15 gives 1.08 and 1.14 and shortens the fights of the reference party of chapters 15 - 27 by 10 - 15%, so +0.10 is kept</t>
         </is>
       </c>
       <c r="K1470" t="inlineStr">
@@ -81866,7 +81866,7 @@
       </c>
       <c r="L1470" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>built</t>
         </is>
       </c>
     </row>
@@ -81907,12 +81907,12 @@
       </c>
       <c r="I1471" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>T05 (every class at its stage; no row of the register names the Trickster)</t>
         </is>
       </c>
       <c r="J1471" t="inlineStr">
         <is>
-          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+          <t>Decided by the user on 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level. Measured: the Trickster from 1.19 and 1.22 to 1.11 and 1.15 by its two routes; +0.15 gives 1.08 and 1.14 and shortens the fights of the reference party of chapters 15 - 27 by 10 - 15%, so +0.10 is kept</t>
         </is>
       </c>
       <c r="K1471" t="inlineStr">
@@ -81922,7 +81922,7 @@
       </c>
       <c r="L1471" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>built</t>
         </is>
       </c>
     </row>
@@ -81963,12 +81963,12 @@
       </c>
       <c r="I1472" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>T05 (every class at its stage; no row of the register names the Trickster)</t>
         </is>
       </c>
       <c r="J1472" t="inlineStr">
         <is>
-          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+          <t>Decided by the user on 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level. Measured: the Trickster from 1.19 and 1.22 to 1.11 and 1.15 by its two routes; +0.15 gives 1.08 and 1.14 and shortens the fights of the reference party of chapters 15 - 27 by 10 - 15%, so +0.10 is kept</t>
         </is>
       </c>
       <c r="K1472" t="inlineStr">
@@ -81978,7 +81978,7 @@
       </c>
       <c r="L1472" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>built</t>
         </is>
       </c>
     </row>
@@ -82019,12 +82019,12 @@
       </c>
       <c r="I1473" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>T05 (every class at its stage; no row of the register names the Trickster)</t>
         </is>
       </c>
       <c r="J1473" t="inlineStr">
         <is>
-          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+          <t>Decided by the user on 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level. Measured: the Trickster from 1.19 and 1.22 to 1.11 and 1.15 by its two routes; +0.15 gives 1.08 and 1.14 and shortens the fights of the reference party of chapters 15 - 27 by 10 - 15%, so +0.10 is kept</t>
         </is>
       </c>
       <c r="K1473" t="inlineStr">
@@ -82034,7 +82034,7 @@
       </c>
       <c r="L1473" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>built</t>
         </is>
       </c>
     </row>
@@ -82075,12 +82075,12 @@
       </c>
       <c r="I1474" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>T05 (every class at its stage; no row of the register names the Trickster)</t>
         </is>
       </c>
       <c r="J1474" t="inlineStr">
         <is>
-          <t>Proposed 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level</t>
+          <t>Decided by the user on 2026-10-11 (the Trickster is 19 - 22% slower than the median attacker at C10, C13, C18): Danger Shoot dealt about 120 a use where Fireball and Frost Slash dealt 155 - 160; the same amount added at every level. Measured: the Trickster from 1.19 and 1.22 to 1.11 and 1.15 by its two routes; +0.15 gives 1.08 and 1.14 and shortens the fights of the reference party of chapters 15 - 27 by 10 - 15%, so +0.10 is kept</t>
         </is>
       </c>
       <c r="K1474" t="inlineStr">
@@ -82090,7 +82090,7 @@
       </c>
       <c r="L1474" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>built</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: the base stage (Danger Shoot from 20 TP
the base stage (Danger Shoot from 20 TP, the Dagger at 20 ATK) and Item
Steal on the four immune commons

1,380 of 1,380 live rows built and installed. The model stops raising a
skill past what a full TP bar pays, and the doll roles hold Danger Shoot
while they are a Spieler. Classes 74 of 76, battery 64 of 85 in vanilla
and 76 of 85 on the variant, curve 35 of 44 within with 9 easier and 0
harder, anchors 6 of 6.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1474"/>
+  <dimension ref="A1:L1480"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5829,7 +5829,7 @@
         <v>30</v>
       </c>
       <c r="G96" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
@@ -5843,7 +5843,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla</t>
+          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla | Decided 2026-10-11 (the Spieler at the base stage): Danger Shoot is her one attack and its first level cost 27 TP, more than the 20 - 25 TP she has at levels 3 - 5, so she could not use it once (the level a skill is used at is the level it was raised to)</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -5885,7 +5885,7 @@
         <v>33</v>
       </c>
       <c r="G97" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
@@ -5899,7 +5899,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla</t>
+          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla | Decided 2026-10-11 (the Spieler at the base stage): Danger Shoot is her one attack and its first level cost 27 TP, more than the 20 - 25 TP she has at levels 3 - 5, so she could not use it once (the level a skill is used at is the level it was raised to)</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -5941,7 +5941,7 @@
         <v>36</v>
       </c>
       <c r="G98" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
@@ -5955,7 +5955,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla</t>
+          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla | Decided 2026-10-11 (the Spieler at the base stage): Danger Shoot is her one attack and its first level cost 27 TP, more than the 20 - 25 TP she has at levels 3 - 5, so she could not use it once (the level a skill is used at is the level it was raised to)</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -5997,7 +5997,7 @@
         <v>40</v>
       </c>
       <c r="G99" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -6011,7 +6011,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla</t>
+          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla | Decided 2026-10-11 (the Spieler at the base stage): Danger Shoot is her one attack and its first level cost 27 TP, more than the 20 - 25 TP she has at levels 3 - 5, so she could not use it once (the level a skill is used at is the level it was raised to)</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6053,7 +6053,7 @@
         <v>44</v>
       </c>
       <c r="G100" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
@@ -6067,7 +6067,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla</t>
+          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla | Decided 2026-10-11 (the Spieler at the base stage): Danger Shoot is her one attack and its first level cost 27 TP, more than the 20 - 25 TP she has at levels 3 - 5, so she could not use it once (the level a skill is used at is the level it was raised to)</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6109,7 +6109,7 @@
         <v>48</v>
       </c>
       <c r="G101" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla</t>
+          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla | Decided 2026-10-11 (the Spieler at the base stage): Danger Shoot is her one attack and its first level cost 27 TP, more than the 20 - 25 TP she has at levels 3 - 5, so she could not use it once (the level a skill is used at is the level it was raised to)</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6165,7 +6165,7 @@
         <v>52</v>
       </c>
       <c r="G102" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla</t>
+          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla | Decided 2026-10-11 (the Spieler at the base stage): Danger Shoot is her one attack and its first level cost 27 TP, more than the 20 - 25 TP she has at levels 3 - 5, so she could not use it once (the level a skill is used at is the level it was raised to)</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6221,7 +6221,7 @@
         <v>56</v>
       </c>
       <c r="G103" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
@@ -6235,7 +6235,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla</t>
+          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla | Decided 2026-10-11 (the Spieler at the base stage): Danger Shoot is her one attack and its first level cost 27 TP, more than the 20 - 25 TP she has at levels 3 - 5, so she could not use it once (the level a skill is used at is the level it was raised to)</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla</t>
+          <t>A little: power per TP at the top level brought toward 70% of level 1, no cost lowered by more than a quarter (it was 59%); the rise of the cost above level 1 scaled by one factor, never above vanilla | Decided 2026-10-11 (the Spieler at the base stage): Danger Shoot is her one attack and its first level cost 27 TP, more than the 20 - 25 TP she has at levels 3 - 5, so she could not use it once (the level a skill is used at is the level it was raised to)</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -82089,6 +82089,343 @@
         </is>
       </c>
       <c r="L1474" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" t="inlineStr">
+        <is>
+          <t>P085</t>
+        </is>
+      </c>
+      <c r="B1475" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1475" t="inlineStr">
+        <is>
+          <t>17 Odin</t>
+        </is>
+      </c>
+      <c r="D1475" t="inlineStr">
+        <is>
+          <t>steal flag (0x3C bit 15)</t>
+        </is>
+      </c>
+      <c r="F1475" t="inlineStr">
+        <is>
+          <t>0x66ed</t>
+        </is>
+      </c>
+      <c r="G1475" t="inlineStr">
+        <is>
+          <t>0xe6ed</t>
+        </is>
+      </c>
+      <c r="H1475" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I1475" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1475" t="inlineStr">
+        <is>
+          <t>Decided by the user on 2026-10-11: the only four enemies of the random battles Item Steal does not work on (levels 96 - 98, two unique pieces each, 3.9 - 5.4% a kill). With the bit a steal that succeeds draws among their drops as for the other 348 (FORMULAS 12.16)</t>
+        </is>
+      </c>
+      <c r="K1475" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1475" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" t="inlineStr">
+        <is>
+          <t>P086</t>
+        </is>
+      </c>
+      <c r="B1476" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1476" t="inlineStr">
+        <is>
+          <t>40 Myrddin</t>
+        </is>
+      </c>
+      <c r="D1476" t="inlineStr">
+        <is>
+          <t>steal flag (0x3C bit 15)</t>
+        </is>
+      </c>
+      <c r="F1476" t="inlineStr">
+        <is>
+          <t>0x6e75</t>
+        </is>
+      </c>
+      <c r="G1476" t="inlineStr">
+        <is>
+          <t>0xee75</t>
+        </is>
+      </c>
+      <c r="H1476" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I1476" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1476" t="inlineStr">
+        <is>
+          <t>Decided by the user on 2026-10-11: the only four enemies of the random battles Item Steal does not work on (levels 96 - 98, two unique pieces each, 3.9 - 5.4% a kill). With the bit a steal that succeeds draws among their drops as for the other 348 (FORMULAS 12.16)</t>
+        </is>
+      </c>
+      <c r="K1476" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1476" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" t="inlineStr">
+        <is>
+          <t>P087</t>
+        </is>
+      </c>
+      <c r="B1477" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1477" t="inlineStr">
+        <is>
+          <t>144 Asmodeus</t>
+        </is>
+      </c>
+      <c r="D1477" t="inlineStr">
+        <is>
+          <t>steal flag (0x3C bit 15)</t>
+        </is>
+      </c>
+      <c r="F1477" t="inlineStr">
+        <is>
+          <t>0x76fd</t>
+        </is>
+      </c>
+      <c r="G1477" t="inlineStr">
+        <is>
+          <t>0xf6fd</t>
+        </is>
+      </c>
+      <c r="H1477" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I1477" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1477" t="inlineStr">
+        <is>
+          <t>Decided by the user on 2026-10-11: the only four enemies of the random battles Item Steal does not work on (levels 96 - 98, two unique pieces each, 3.9 - 5.4% a kill). With the bit a steal that succeeds draws among their drops as for the other 348 (FORMULAS 12.16)</t>
+        </is>
+      </c>
+      <c r="K1477" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1477" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" t="inlineStr">
+        <is>
+          <t>P088</t>
+        </is>
+      </c>
+      <c r="B1478" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1478" t="inlineStr">
+        <is>
+          <t>444 Carmilla</t>
+        </is>
+      </c>
+      <c r="D1478" t="inlineStr">
+        <is>
+          <t>steal flag (0x3C bit 15)</t>
+        </is>
+      </c>
+      <c r="F1478" t="inlineStr">
+        <is>
+          <t>0x67fd</t>
+        </is>
+      </c>
+      <c r="G1478" t="inlineStr">
+        <is>
+          <t>0xe7fd</t>
+        </is>
+      </c>
+      <c r="H1478" t="inlineStr">
+        <is>
+          <t>L40</t>
+        </is>
+      </c>
+      <c r="I1478" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="J1478" t="inlineStr">
+        <is>
+          <t>Decided by the user on 2026-10-11: the only four enemies of the random battles Item Steal does not work on (levels 96 - 98, two unique pieces each, 3.9 - 5.4% a kill). With the bit a steal that succeeds draws among their drops as for the other 348 (FORMULAS 12.16)</t>
+        </is>
+      </c>
+      <c r="K1478" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1478" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" t="inlineStr">
+        <is>
+          <t>Y011</t>
+        </is>
+      </c>
+      <c r="B1479" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1479" t="inlineStr">
+        <is>
+          <t>Technique 79 Danger Shoot</t>
+        </is>
+      </c>
+      <c r="D1479" t="inlineStr">
+        <is>
+          <t>TP cost</t>
+        </is>
+      </c>
+      <c r="E1479" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1479" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1479" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1479" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1479" t="inlineStr">
+        <is>
+          <t>T05 (every class at its stage)</t>
+        </is>
+      </c>
+      <c r="J1479" t="inlineStr">
+        <is>
+          <t>Decided 2026-10-11 (the Spieler at the base stage): Danger Shoot is her one attack and its first level cost 27 TP, more than the 20 - 25 TP she has at levels 3 - 5, so she could not use it once (the level a skill is used at is the level it was raised to)</t>
+        </is>
+      </c>
+      <c r="K1479" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1479" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" t="inlineStr">
+        <is>
+          <t>W046</t>
+        </is>
+      </c>
+      <c r="B1480" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C1480" t="inlineStr">
+        <is>
+          <t>53 Dagger</t>
+        </is>
+      </c>
+      <c r="D1480" t="inlineStr">
+        <is>
+          <t>ATK (base)</t>
+        </is>
+      </c>
+      <c r="F1480" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1480" t="n">
+        <v>20</v>
+      </c>
+      <c r="H1480" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="I1480" t="inlineStr">
+        <is>
+          <t>T05 (every class at its stage)</t>
+        </is>
+      </c>
+      <c r="J1480" t="inlineStr">
+        <is>
+          <t>Decided 2026-10-11 (the Scout with a dagger at the base stage, 9 - 13% of the damage of the party): the Dagger holds 14 ATK where the Shortsword holds 20 and the Short Bow 27; at levels 5 - 9 the forge adds little</t>
+        </is>
+      </c>
+      <c r="K1480" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1480" t="inlineStr">
         <is>
           <t>built</t>
         </is>

</xml_diff>

<commit_message>
balance: the final boss holds 1.2 times its HP, by exception
the final boss holds 1.2 times its HP, by exception; postgame: three
effects modelled, the Japanese preparation written in

C40 lasts 34.2 against 35.5 in vanilla and is won 95% of the time (1,382
of 1,382 rows built, installed). The simulator acts on effect 86 (twice
the damage on the Magic User line) and 204 (Weird Dance), and declares
200 and 3: 48 of the 55 postgame fights hold nothing it does not act on.
From the Plains of Light on the party holds every elemental resistance
at 100, as the Japanese guide gives for premise, and the weakened Crom
Cruach is fought without its water zone; the guide curve does not move
(51 of 70), so the gap of the postgame lies elsewhere.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1480"/>
+  <dimension ref="A1:L1482"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82431,6 +82431,112 @@
         </is>
       </c>
     </row>
+    <row r="1481">
+      <c r="A1481" t="inlineStr">
+        <is>
+          <t>G116</t>
+        </is>
+      </c>
+      <c r="B1481" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1481" t="inlineStr">
+        <is>
+          <t>958 Demiurge (C40)</t>
+        </is>
+      </c>
+      <c r="D1481" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1481" t="n">
+        <v>24000</v>
+      </c>
+      <c r="G1481" t="n">
+        <v>28800</v>
+      </c>
+      <c r="H1481" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1481" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1481" t="inlineStr">
+        <is>
+          <t>The final boss, an exception decided by the user on 2026-10-11: on the variant the fight lasted 25.1 where vanilla lasts 35.5 and was won 95% of the time against 88%; with the HP of both forms x1.20 it lasts 34.2 and is won 95%. The condition of the gentle fit is set aside for this boss: Anti-Meta-Plus was under the floor of 50% before the change (45%) and goes to 38% (0% in vanilla), Juggernaut-Plus stands at the floor (50%), Mage-Heavy at 72% (40 battles each). x1.30 passes the length of vanilla and takes two more parties under the floor</t>
+        </is>
+      </c>
+      <c r="K1481" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1481" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" t="inlineStr">
+        <is>
+          <t>G117</t>
+        </is>
+      </c>
+      <c r="B1482" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1482" t="inlineStr">
+        <is>
+          <t>961 Atialuco (C40)</t>
+        </is>
+      </c>
+      <c r="D1482" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1482" t="n">
+        <v>21800</v>
+      </c>
+      <c r="G1482" t="n">
+        <v>26160</v>
+      </c>
+      <c r="H1482" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1482" t="inlineStr">
+        <is>
+          <t>R08, R10</t>
+        </is>
+      </c>
+      <c r="J1482" t="inlineStr">
+        <is>
+          <t>The final boss, an exception decided by the user on 2026-10-11: on the variant the fight lasted 25.1 where vanilla lasts 35.5 and was won 95% of the time against 88%; with the HP of both forms x1.20 it lasts 34.2 and is won 95%. The condition of the gentle fit is set aside for this boss: Anti-Meta-Plus was under the floor of 50% before the change (45%) and goes to 38% (0% in vanilla), Juggernaut-Plus stands at the floor (50%), Mage-Heavy at 72% (40 battles each). x1.30 passes the length of vanilla and takes two more parties under the floor</t>
+        </is>
+      </c>
+      <c r="K1482" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1482" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
balance: support Shot fires at 10 - 30% instead of 4 - 12%
support Shot fires at 10 - 30% instead of 4 - 12% (W047 - W051), built
and installed; J02 left for the postgame
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1482"/>
+  <dimension ref="A1:L1487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82537,6 +82537,286 @@
         </is>
       </c>
     </row>
+    <row r="1483">
+      <c r="A1483" t="inlineStr">
+        <is>
+          <t>W047</t>
+        </is>
+      </c>
+      <c r="B1483" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1483" t="inlineStr">
+        <is>
+          <t>Passive 271 Support Shot</t>
+        </is>
+      </c>
+      <c r="D1483" t="inlineStr">
+        <is>
+          <t>effect 260</t>
+        </is>
+      </c>
+      <c r="E1483" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1483" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G1483" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H1483" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1483" t="inlineStr">
+        <is>
+          <t>F52</t>
+        </is>
+      </c>
+      <c r="J1483" t="inlineStr">
+        <is>
+          <t>Decided 2026-10-11 (the user: raise it to a reasonable level): Support Shot fires only after a plain attack of another member, and at 4 - 12% the reference party with and without it was the same inside the noise (C22, C30, C34, C40). At 10 - 30% a Sniper beside members who strike plainly adds a shot to about one of their attacks in three; beside a party that spends TP every turn it stays what it was</t>
+        </is>
+      </c>
+      <c r="K1483" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1483" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" t="inlineStr">
+        <is>
+          <t>W048</t>
+        </is>
+      </c>
+      <c r="B1484" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1484" t="inlineStr">
+        <is>
+          <t>Passive 271 Support Shot</t>
+        </is>
+      </c>
+      <c r="D1484" t="inlineStr">
+        <is>
+          <t>effect 260</t>
+        </is>
+      </c>
+      <c r="E1484" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1484" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G1484" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H1484" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1484" t="inlineStr">
+        <is>
+          <t>F52</t>
+        </is>
+      </c>
+      <c r="J1484" t="inlineStr">
+        <is>
+          <t>Decided 2026-10-11 (the user: raise it to a reasonable level): Support Shot fires only after a plain attack of another member, and at 4 - 12% the reference party with and without it was the same inside the noise (C22, C30, C34, C40). At 10 - 30% a Sniper beside members who strike plainly adds a shot to about one of their attacks in three; beside a party that spends TP every turn it stays what it was</t>
+        </is>
+      </c>
+      <c r="K1484" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1484" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" t="inlineStr">
+        <is>
+          <t>W049</t>
+        </is>
+      </c>
+      <c r="B1485" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1485" t="inlineStr">
+        <is>
+          <t>Passive 271 Support Shot</t>
+        </is>
+      </c>
+      <c r="D1485" t="inlineStr">
+        <is>
+          <t>effect 260</t>
+        </is>
+      </c>
+      <c r="E1485" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1485" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G1485" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H1485" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1485" t="inlineStr">
+        <is>
+          <t>F52</t>
+        </is>
+      </c>
+      <c r="J1485" t="inlineStr">
+        <is>
+          <t>Decided 2026-10-11 (the user: raise it to a reasonable level): Support Shot fires only after a plain attack of another member, and at 4 - 12% the reference party with and without it was the same inside the noise (C22, C30, C34, C40). At 10 - 30% a Sniper beside members who strike plainly adds a shot to about one of their attacks in three; beside a party that spends TP every turn it stays what it was</t>
+        </is>
+      </c>
+      <c r="K1485" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1485" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" t="inlineStr">
+        <is>
+          <t>W050</t>
+        </is>
+      </c>
+      <c r="B1486" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1486" t="inlineStr">
+        <is>
+          <t>Passive 271 Support Shot</t>
+        </is>
+      </c>
+      <c r="D1486" t="inlineStr">
+        <is>
+          <t>effect 260</t>
+        </is>
+      </c>
+      <c r="E1486" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1486" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G1486" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H1486" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1486" t="inlineStr">
+        <is>
+          <t>F52</t>
+        </is>
+      </c>
+      <c r="J1486" t="inlineStr">
+        <is>
+          <t>Decided 2026-10-11 (the user: raise it to a reasonable level): Support Shot fires only after a plain attack of another member, and at 4 - 12% the reference party with and without it was the same inside the noise (C22, C30, C34, C40). At 10 - 30% a Sniper beside members who strike plainly adds a shot to about one of their attacks in three; beside a party that spends TP every turn it stays what it was</t>
+        </is>
+      </c>
+      <c r="K1486" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1486" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" t="inlineStr">
+        <is>
+          <t>W051</t>
+        </is>
+      </c>
+      <c r="B1487" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="C1487" t="inlineStr">
+        <is>
+          <t>Passive 271 Support Shot</t>
+        </is>
+      </c>
+      <c r="D1487" t="inlineStr">
+        <is>
+          <t>effect 260</t>
+        </is>
+      </c>
+      <c r="E1487" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1487" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G1487" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H1487" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="I1487" t="inlineStr">
+        <is>
+          <t>F52</t>
+        </is>
+      </c>
+      <c r="J1487" t="inlineStr">
+        <is>
+          <t>Decided 2026-10-11 (the user: raise it to a reasonable level): Support Shot fires only after a plain attack of another member, and at 4 - 12% the reference party with and without it was the same inside the noise (C22, C30, C34, C40). At 10 - 30% a Sniper beside members who strike plainly adds a shot to about one of their attacks in three; beside a party that spends TP every turn it stays what it was</t>
+        </is>
+      </c>
+      <c r="K1487" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="L1487" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
balance: the damage draw of Roulette Circus back to level x 10
the damage draw of Roulette Circus back to level x 10 (L002 dropped: it
strikes any unit of the battle, the party included)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -26451,7 +26451,7 @@
       </c>
       <c r="J464" t="inlineStr">
         <is>
-          <t>A good draw pays for the TP of the skill. The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
+          <t>Dropped on 2026-10-11 (the user): the outcome strikes one unit of the battle at random, members of the party included (target code 15), so a larger value is a larger risk, not a better draw; it stays at level x 10. Was: A good draw pays for the TP of the skill. The chances of the outcomes (executable, L37) are not touched; the empty outcome, the 666 damage and the money ones stay</t>
         </is>
       </c>
       <c r="K464" t="inlineStr">
@@ -26461,7 +26461,7 @@
       </c>
       <c r="L464" t="inlineStr">
         <is>
-          <t>built</t>
+          <t>dropped</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: RES x0.9 at the six superboss fights that walled magic off
RES x0.9 at the six superboss fights that walled magic off (J02, E213 -
E223) and the EXP enchantment on the Grand Sealbook of Molle (P089);
built and installed, the register closed
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1487"/>
+  <dimension ref="A1:L1499"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82817,6 +82817,646 @@
         </is>
       </c>
     </row>
+    <row r="1488">
+      <c r="A1488" t="inlineStr">
+        <is>
+          <t>E213</t>
+        </is>
+      </c>
+      <c r="B1488" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1488" t="inlineStr">
+        <is>
+          <t>921 Hell's Angel (P28)</t>
+        </is>
+      </c>
+      <c r="D1488" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="F1488" t="n">
+        <v>407</v>
+      </c>
+      <c r="G1488" t="n">
+        <v>366</v>
+      </c>
+      <c r="H1488" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1488" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="J1488" t="inlineStr">
+        <is>
+          <t>Row J02 (decided 2026-10-09: lower a little what walls magic off at the superbosses, keeping their flavour; the user, 2026-10-12: without abuse, the postgame stays hard, the mages keep some of their power). At the six fights where the best option of the mage was under that of the Dark Lord, RES of every enemy times 0.9; the elemental resistances are left alone (lowering them raises the elemental strikes of the Dark Lord as much as the spells: measured, the mage stays at 50 - 84%). The mage beside the Dark Lord there: P28 51%, P29 73%, P30 50%, P33 84%, P50 54%, P51 51% before, P28 59%, P29 95%, P30 80%, P33 104%, P50 70%, P51 57% after</t>
+        </is>
+      </c>
+      <c r="K1488" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1488" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" t="inlineStr">
+        <is>
+          <t>E214</t>
+        </is>
+      </c>
+      <c r="B1489" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1489" t="inlineStr">
+        <is>
+          <t>992 Panagia (P33)</t>
+        </is>
+      </c>
+      <c r="D1489" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="F1489" t="n">
+        <v>556</v>
+      </c>
+      <c r="G1489" t="n">
+        <v>500</v>
+      </c>
+      <c r="H1489" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1489" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="J1489" t="inlineStr">
+        <is>
+          <t>Row J02 (decided 2026-10-09: lower a little what walls magic off at the superbosses, keeping their flavour; the user, 2026-10-12: without abuse, the postgame stays hard, the mages keep some of their power). At the six fights where the best option of the mage was under that of the Dark Lord, RES of every enemy times 0.9; the elemental resistances are left alone (lowering them raises the elemental strikes of the Dark Lord as much as the spells: measured, the mage stays at 50 - 84%). The mage beside the Dark Lord there: P28 51%, P29 73%, P30 50%, P33 84%, P50 54%, P51 51% before, P28 59%, P29 95%, P30 80%, P33 104%, P50 70%, P51 57% after</t>
+        </is>
+      </c>
+      <c r="K1489" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1489" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" t="inlineStr">
+        <is>
+          <t>E215</t>
+        </is>
+      </c>
+      <c r="B1490" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1490" t="inlineStr">
+        <is>
+          <t>972 Tenerezza (P30)</t>
+        </is>
+      </c>
+      <c r="D1490" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="F1490" t="n">
+        <v>548</v>
+      </c>
+      <c r="G1490" t="n">
+        <v>493</v>
+      </c>
+      <c r="H1490" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1490" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="J1490" t="inlineStr">
+        <is>
+          <t>Row J02 (decided 2026-10-09: lower a little what walls magic off at the superbosses, keeping their flavour; the user, 2026-10-12: without abuse, the postgame stays hard, the mages keep some of their power). At the six fights where the best option of the mage was under that of the Dark Lord, RES of every enemy times 0.9; the elemental resistances are left alone (lowering them raises the elemental strikes of the Dark Lord as much as the spells: measured, the mage stays at 50 - 84%). The mage beside the Dark Lord there: P28 51%, P29 73%, P30 50%, P33 84%, P50 54%, P51 51% before, P28 59%, P29 95%, P30 80%, P33 104%, P50 70%, P51 57% after</t>
+        </is>
+      </c>
+      <c r="K1490" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1490" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" t="inlineStr">
+        <is>
+          <t>E216</t>
+        </is>
+      </c>
+      <c r="B1491" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1491" t="inlineStr">
+        <is>
+          <t>975 Lolo (P30)</t>
+        </is>
+      </c>
+      <c r="D1491" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="F1491" t="n">
+        <v>666</v>
+      </c>
+      <c r="G1491" t="n">
+        <v>599</v>
+      </c>
+      <c r="H1491" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1491" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="J1491" t="inlineStr">
+        <is>
+          <t>Row J02 (decided 2026-10-09: lower a little what walls magic off at the superbosses, keeping their flavour; the user, 2026-10-12: without abuse, the postgame stays hard, the mages keep some of their power). At the six fights where the best option of the mage was under that of the Dark Lord, RES of every enemy times 0.9; the elemental resistances are left alone (lowering them raises the elemental strikes of the Dark Lord as much as the spells: measured, the mage stays at 50 - 84%). The mage beside the Dark Lord there: P28 51%, P29 73%, P30 50%, P33 84%, P50 54%, P51 51% before, P28 59%, P29 95%, P30 80%, P33 104%, P50 70%, P51 57% after</t>
+        </is>
+      </c>
+      <c r="K1491" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1491" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" t="inlineStr">
+        <is>
+          <t>E217</t>
+        </is>
+      </c>
+      <c r="B1492" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1492" t="inlineStr">
+        <is>
+          <t>993 Panagia (P33)</t>
+        </is>
+      </c>
+      <c r="D1492" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="F1492" t="n">
+        <v>532</v>
+      </c>
+      <c r="G1492" t="n">
+        <v>478</v>
+      </c>
+      <c r="H1492" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1492" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="J1492" t="inlineStr">
+        <is>
+          <t>Row J02 (decided 2026-10-09: lower a little what walls magic off at the superbosses, keeping their flavour; the user, 2026-10-12: without abuse, the postgame stays hard, the mages keep some of their power). At the six fights where the best option of the mage was under that of the Dark Lord, RES of every enemy times 0.9; the elemental resistances are left alone (lowering them raises the elemental strikes of the Dark Lord as much as the spells: measured, the mage stays at 50 - 84%). The mage beside the Dark Lord there: P28 51%, P29 73%, P30 50%, P33 84%, P50 54%, P51 51% before, P28 59%, P29 95%, P30 80%, P33 104%, P50 70%, P51 57% after</t>
+        </is>
+      </c>
+      <c r="K1492" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1492" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" t="inlineStr">
+        <is>
+          <t>E218</t>
+        </is>
+      </c>
+      <c r="B1493" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1493" t="inlineStr">
+        <is>
+          <t>996 Radiant Being (P33)</t>
+        </is>
+      </c>
+      <c r="D1493" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="F1493" t="n">
+        <v>431</v>
+      </c>
+      <c r="G1493" t="n">
+        <v>387</v>
+      </c>
+      <c r="H1493" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1493" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="J1493" t="inlineStr">
+        <is>
+          <t>Row J02 (decided 2026-10-09: lower a little what walls magic off at the superbosses, keeping their flavour; the user, 2026-10-12: without abuse, the postgame stays hard, the mages keep some of their power). At the six fights where the best option of the mage was under that of the Dark Lord, RES of every enemy times 0.9; the elemental resistances are left alone (lowering them raises the elemental strikes of the Dark Lord as much as the spells: measured, the mage stays at 50 - 84%). The mage beside the Dark Lord there: P28 51%, P29 73%, P30 50%, P33 84%, P50 54%, P51 51% before, P28 59%, P29 95%, P30 80%, P33 104%, P50 70%, P51 57% after</t>
+        </is>
+      </c>
+      <c r="K1493" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1493" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" t="inlineStr">
+        <is>
+          <t>E219</t>
+        </is>
+      </c>
+      <c r="B1494" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1494" t="inlineStr">
+        <is>
+          <t>973 Tenerezza (P50)</t>
+        </is>
+      </c>
+      <c r="D1494" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="F1494" t="n">
+        <v>1648</v>
+      </c>
+      <c r="G1494" t="n">
+        <v>1483</v>
+      </c>
+      <c r="H1494" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1494" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="J1494" t="inlineStr">
+        <is>
+          <t>Row J02 (decided 2026-10-09: lower a little what walls magic off at the superbosses, keeping their flavour; the user, 2026-10-12: without abuse, the postgame stays hard, the mages keep some of their power). At the six fights where the best option of the mage was under that of the Dark Lord, RES of every enemy times 0.9; the elemental resistances are left alone (lowering them raises the elemental strikes of the Dark Lord as much as the spells: measured, the mage stays at 50 - 84%). The mage beside the Dark Lord there: P28 51%, P29 73%, P30 50%, P33 84%, P50 54%, P51 51% before, P28 59%, P29 95%, P30 80%, P33 104%, P50 70%, P51 57% after</t>
+        </is>
+      </c>
+      <c r="K1494" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1494" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" t="inlineStr">
+        <is>
+          <t>E220</t>
+        </is>
+      </c>
+      <c r="B1495" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1495" t="inlineStr">
+        <is>
+          <t>976 Lolo (P50)</t>
+        </is>
+      </c>
+      <c r="D1495" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="F1495" t="n">
+        <v>745</v>
+      </c>
+      <c r="G1495" t="n">
+        <v>670</v>
+      </c>
+      <c r="H1495" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1495" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="J1495" t="inlineStr">
+        <is>
+          <t>Row J02 (decided 2026-10-09: lower a little what walls magic off at the superbosses, keeping their flavour; the user, 2026-10-12: without abuse, the postgame stays hard, the mages keep some of their power). At the six fights where the best option of the mage was under that of the Dark Lord, RES of every enemy times 0.9; the elemental resistances are left alone (lowering them raises the elemental strikes of the Dark Lord as much as the spells: measured, the mage stays at 50 - 84%). The mage beside the Dark Lord there: P28 51%, P29 73%, P30 50%, P33 84%, P50 54%, P51 51% before, P28 59%, P29 95%, P30 80%, P33 104%, P50 70%, P51 57% after</t>
+        </is>
+      </c>
+      <c r="K1495" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1495" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" t="inlineStr">
+        <is>
+          <t>E221</t>
+        </is>
+      </c>
+      <c r="B1496" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1496" t="inlineStr">
+        <is>
+          <t>985 Samson (P51)</t>
+        </is>
+      </c>
+      <c r="D1496" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="F1496" t="n">
+        <v>972</v>
+      </c>
+      <c r="G1496" t="n">
+        <v>874</v>
+      </c>
+      <c r="H1496" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1496" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="J1496" t="inlineStr">
+        <is>
+          <t>Row J02 (decided 2026-10-09: lower a little what walls magic off at the superbosses, keeping their flavour; the user, 2026-10-12: without abuse, the postgame stays hard, the mages keep some of their power). At the six fights where the best option of the mage was under that of the Dark Lord, RES of every enemy times 0.9; the elemental resistances are left alone (lowering them raises the elemental strikes of the Dark Lord as much as the spells: measured, the mage stays at 50 - 84%). The mage beside the Dark Lord there: P28 51%, P29 73%, P30 50%, P33 84%, P50 54%, P51 51% before, P28 59%, P29 95%, P30 80%, P33 104%, P50 70%, P51 57% after</t>
+        </is>
+      </c>
+      <c r="K1496" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1496" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" t="inlineStr">
+        <is>
+          <t>E222</t>
+        </is>
+      </c>
+      <c r="B1497" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1497" t="inlineStr">
+        <is>
+          <t>979 Magna Meretrix (P51)</t>
+        </is>
+      </c>
+      <c r="D1497" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="F1497" t="n">
+        <v>1298</v>
+      </c>
+      <c r="G1497" t="n">
+        <v>1168</v>
+      </c>
+      <c r="H1497" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1497" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="J1497" t="inlineStr">
+        <is>
+          <t>Row J02 (decided 2026-10-09: lower a little what walls magic off at the superbosses, keeping their flavour; the user, 2026-10-12: without abuse, the postgame stays hard, the mages keep some of their power). At the six fights where the best option of the mage was under that of the Dark Lord, RES of every enemy times 0.9; the elemental resistances are left alone (lowering them raises the elemental strikes of the Dark Lord as much as the spells: measured, the mage stays at 50 - 84%). The mage beside the Dark Lord there: P28 51%, P29 73%, P30 50%, P33 84%, P50 54%, P51 51% before, P28 59%, P29 95%, P30 80%, P33 104%, P50 70%, P51 57% after</t>
+        </is>
+      </c>
+      <c r="K1497" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1497" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" t="inlineStr">
+        <is>
+          <t>E223</t>
+        </is>
+      </c>
+      <c r="B1498" t="inlineStr">
+        <is>
+          <t>enemies</t>
+        </is>
+      </c>
+      <c r="C1498" t="inlineStr">
+        <is>
+          <t>982 Adon (P51)</t>
+        </is>
+      </c>
+      <c r="D1498" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="F1498" t="n">
+        <v>844</v>
+      </c>
+      <c r="G1498" t="n">
+        <v>759</v>
+      </c>
+      <c r="H1498" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="I1498" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="J1498" t="inlineStr">
+        <is>
+          <t>Row J02 (decided 2026-10-09: lower a little what walls magic off at the superbosses, keeping their flavour; the user, 2026-10-12: without abuse, the postgame stays hard, the mages keep some of their power). At the six fights where the best option of the mage was under that of the Dark Lord, RES of every enemy times 0.9; the elemental resistances are left alone (lowering them raises the elemental strikes of the Dark Lord as much as the spells: measured, the mage stays at 50 - 84%). The mage beside the Dark Lord there: P28 51%, P29 73%, P30 50%, P33 84%, P50 54%, P51 51% before, P28 59%, P29 95%, P30 80%, P33 104%, P50 70%, P51 57% after</t>
+        </is>
+      </c>
+      <c r="K1498" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1498" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" t="inlineStr">
+        <is>
+          <t>P089</t>
+        </is>
+      </c>
+      <c r="B1499" t="inlineStr">
+        <is>
+          <t>sealbooks</t>
+        </is>
+      </c>
+      <c r="C1499" t="inlineStr">
+        <is>
+          <t>Grand Sealbook [Molle] (0829)</t>
+        </is>
+      </c>
+      <c r="D1499" t="inlineStr">
+        <is>
+          <t>secondary enchantment</t>
+        </is>
+      </c>
+      <c r="F1499" t="inlineStr">
+        <is>
+          <t>ench_cnt=1 (262 only)</t>
+        </is>
+      </c>
+      <c r="G1499" t="inlineStr">
+        <is>
+          <t>ench_cnt=2 (262 Escape probability UP, 270 Gain more EXP from higher-level enemies)</t>
+        </is>
+      </c>
+      <c r="H1499" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1499" t="inlineStr">
+        <is>
+          <t>U01</t>
+        </is>
+      </c>
+      <c r="J1499" t="inlineStr">
+        <is>
+          <t>The user, 2026-10-12: the piece that raises the EXP factors of B4 comes late (the Grand Sealbook of Dragon Papi, level 44); he wants the same effect around level 20 - 30, on one unique thing that is neither farmed nor stolen, without filling the game with such pieces. Molle is a boss of the story at level 23 and its grand sealbook, made once from it, held only "Escape probability UP". The book of Dragon Papi keeps its own</t>
+        </is>
+      </c>
+      <c r="K1499" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1499" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
balance: the EXP enchantment on the Bathroom Slippers
the EXP enchantment on the Bathroom Slippers, the reward of quest rank 3
(P090); the Grand Sealbook of Molle back to vanilla (P089 dropped)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1499"/>
+  <dimension ref="A1:L1500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83443,7 +83443,7 @@
       </c>
       <c r="J1499" t="inlineStr">
         <is>
-          <t>The user, 2026-10-12: the piece that raises the EXP factors of B4 comes late (the Grand Sealbook of Dragon Papi, level 44); he wants the same effect around level 20 - 30, on one unique thing that is neither farmed nor stolen, without filling the game with such pieces. Molle is a boss of the story at level 23 and its grand sealbook, made once from it, held only "Escape probability UP". The book of Dragon Papi keeps its own</t>
+          <t>Dropped on 2026-10-12 (the user): the effect goes on an accessory, not on a sealbook; the book of Molle is as in vanilla. Was: The user, 2026-10-12: the piece that raises the EXP factors of B4 comes late (the Grand Sealbook of Dragon Papi, level 44); he wants the same effect around level 20 - 30, on one unique thing that is neither farmed nor stolen, without filling the game with such pieces. Molle is a boss of the story at level 23 and its grand sealbook, made once from it, held only "Escape probability UP". The book of Dragon Papi keeps its own</t>
         </is>
       </c>
       <c r="K1499" t="inlineStr">
@@ -83452,6 +83452,59 @@
         </is>
       </c>
       <c r="L1499" t="inlineStr">
+        <is>
+          <t>dropped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" t="inlineStr">
+        <is>
+          <t>P090</t>
+        </is>
+      </c>
+      <c r="B1500" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C1500" t="inlineStr">
+        <is>
+          <t>732 Bathroom Slippers</t>
+        </is>
+      </c>
+      <c r="D1500" t="inlineStr">
+        <is>
+          <t>Enchant 2 (0x64)</t>
+        </is>
+      </c>
+      <c r="F1500" t="n">
+        <v>33</v>
+      </c>
+      <c r="G1500" t="n">
+        <v>270</v>
+      </c>
+      <c r="H1500" t="inlineStr">
+        <is>
+          <t>L15</t>
+        </is>
+      </c>
+      <c r="I1500" t="inlineStr">
+        <is>
+          <t>U01</t>
+        </is>
+      </c>
+      <c r="J1500" t="inlineStr">
+        <is>
+          <t>The user, 2026-10-12: the piece that raises the EXP factors of B4 comes late (the Grand Sealbook of Dragon Papi, level 44); he wants the same effect earlier on one unique accessory that is neither farmed nor stolen, without filling the game with such pieces. The Bathroom Slippers are the reward of quest rank 3, given once, wearable by every class; they keep "Nullify poison" and give up "Physical defense UP" (enchantment 33), the count of innate enchantments staying as it is (lever L15)</t>
+        </is>
+      </c>
+      <c r="K1500" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1500" t="inlineStr">
         <is>
           <t>built</t>
         </is>

</xml_diff>

<commit_message>
balance: fascinating Waltz and Dumbing Mazurka times 1.5 again
fascinating Waltz and Dumbing Mazurka times 1.5 again (the Etoile as the
one support), built and installed; six support skills tried with other
values, none built
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -39827,7 +39827,7 @@
         <v>-0.04</v>
       </c>
       <c r="G702" t="n">
-        <v>-0.06</v>
+        <v>-0.09</v>
       </c>
       <c r="H702" t="inlineStr">
         <is>
@@ -39841,7 +39841,7 @@
       </c>
       <c r="J702" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K702" t="inlineStr">
@@ -39883,7 +39883,7 @@
         <v>-0.06</v>
       </c>
       <c r="G703" t="n">
-        <v>-0.09</v>
+        <v>-0.14</v>
       </c>
       <c r="H703" t="inlineStr">
         <is>
@@ -39897,7 +39897,7 @@
       </c>
       <c r="J703" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K703" t="inlineStr">
@@ -39939,7 +39939,7 @@
         <v>-0.08</v>
       </c>
       <c r="G704" t="n">
-        <v>-0.12</v>
+        <v>-0.18</v>
       </c>
       <c r="H704" t="inlineStr">
         <is>
@@ -39953,7 +39953,7 @@
       </c>
       <c r="J704" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K704" t="inlineStr">
@@ -39995,7 +39995,7 @@
         <v>-0.1</v>
       </c>
       <c r="G705" t="n">
-        <v>-0.15</v>
+        <v>-0.22</v>
       </c>
       <c r="H705" t="inlineStr">
         <is>
@@ -40009,7 +40009,7 @@
       </c>
       <c r="J705" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K705" t="inlineStr">
@@ -40051,7 +40051,7 @@
         <v>-0.11</v>
       </c>
       <c r="G706" t="n">
-        <v>-0.17</v>
+        <v>-0.26</v>
       </c>
       <c r="H706" t="inlineStr">
         <is>
@@ -40065,7 +40065,7 @@
       </c>
       <c r="J706" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K706" t="inlineStr">
@@ -40107,7 +40107,7 @@
         <v>-0.12</v>
       </c>
       <c r="G707" t="n">
-        <v>-0.18</v>
+        <v>-0.27</v>
       </c>
       <c r="H707" t="inlineStr">
         <is>
@@ -40121,7 +40121,7 @@
       </c>
       <c r="J707" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K707" t="inlineStr">
@@ -40163,7 +40163,7 @@
         <v>-0.13</v>
       </c>
       <c r="G708" t="n">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="H708" t="inlineStr">
         <is>
@@ -40177,7 +40177,7 @@
       </c>
       <c r="J708" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K708" t="inlineStr">
@@ -40219,7 +40219,7 @@
         <v>-0.14</v>
       </c>
       <c r="G709" t="n">
-        <v>-0.21</v>
+        <v>-0.32</v>
       </c>
       <c r="H709" t="inlineStr">
         <is>
@@ -40233,7 +40233,7 @@
       </c>
       <c r="J709" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K709" t="inlineStr">
@@ -40275,7 +40275,7 @@
         <v>-0.15</v>
       </c>
       <c r="G710" t="n">
-        <v>-0.23</v>
+        <v>-0.35</v>
       </c>
       <c r="H710" t="inlineStr">
         <is>
@@ -40289,7 +40289,7 @@
       </c>
       <c r="J710" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K710" t="inlineStr">
@@ -40331,7 +40331,7 @@
         <v>-0.16</v>
       </c>
       <c r="G711" t="n">
-        <v>-0.24</v>
+        <v>-0.36</v>
       </c>
       <c r="H711" t="inlineStr">
         <is>
@@ -40345,7 +40345,7 @@
       </c>
       <c r="J711" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K711" t="inlineStr">
@@ -42067,7 +42067,7 @@
         <v>-0.05</v>
       </c>
       <c r="G742" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.11</v>
       </c>
       <c r="H742" t="inlineStr">
         <is>
@@ -42081,7 +42081,7 @@
       </c>
       <c r="J742" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K742" t="inlineStr">
@@ -42123,7 +42123,7 @@
         <v>-0.06</v>
       </c>
       <c r="G743" t="n">
-        <v>-0.09</v>
+        <v>-0.14</v>
       </c>
       <c r="H743" t="inlineStr">
         <is>
@@ -42137,7 +42137,7 @@
       </c>
       <c r="J743" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K743" t="inlineStr">
@@ -42179,7 +42179,7 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="G744" t="n">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="H744" t="inlineStr">
         <is>
@@ -42193,7 +42193,7 @@
       </c>
       <c r="J744" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K744" t="inlineStr">
@@ -42235,7 +42235,7 @@
         <v>-0.08</v>
       </c>
       <c r="G745" t="n">
-        <v>-0.12</v>
+        <v>-0.18</v>
       </c>
       <c r="H745" t="inlineStr">
         <is>
@@ -42249,7 +42249,7 @@
       </c>
       <c r="J745" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K745" t="inlineStr">
@@ -42291,7 +42291,7 @@
         <v>-0.09</v>
       </c>
       <c r="G746" t="n">
-        <v>-0.14</v>
+        <v>-0.21</v>
       </c>
       <c r="H746" t="inlineStr">
         <is>
@@ -42305,7 +42305,7 @@
       </c>
       <c r="J746" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K746" t="inlineStr">
@@ -42347,7 +42347,7 @@
         <v>-0.1</v>
       </c>
       <c r="G747" t="n">
-        <v>-0.15</v>
+        <v>-0.22</v>
       </c>
       <c r="H747" t="inlineStr">
         <is>
@@ -42361,7 +42361,7 @@
       </c>
       <c r="J747" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K747" t="inlineStr">
@@ -42403,7 +42403,7 @@
         <v>-0.11</v>
       </c>
       <c r="G748" t="n">
-        <v>-0.17</v>
+        <v>-0.26</v>
       </c>
       <c r="H748" t="inlineStr">
         <is>
@@ -42417,7 +42417,7 @@
       </c>
       <c r="J748" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K748" t="inlineStr">
@@ -42459,7 +42459,7 @@
         <v>-0.12</v>
       </c>
       <c r="G749" t="n">
-        <v>-0.18</v>
+        <v>-0.27</v>
       </c>
       <c r="H749" t="inlineStr">
         <is>
@@ -42473,7 +42473,7 @@
       </c>
       <c r="J749" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K749" t="inlineStr">
@@ -42515,7 +42515,7 @@
         <v>-0.13</v>
       </c>
       <c r="G750" t="n">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="H750" t="inlineStr">
         <is>
@@ -42529,7 +42529,7 @@
       </c>
       <c r="J750" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K750" t="inlineStr">
@@ -42571,7 +42571,7 @@
         <v>-0.14</v>
       </c>
       <c r="G751" t="n">
-        <v>-0.21</v>
+        <v>-0.32</v>
       </c>
       <c r="H751" t="inlineStr">
         <is>
@@ -42585,7 +42585,7 @@
       </c>
       <c r="J751" t="inlineStr">
         <is>
-          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length</t>
+          <t>Debuffs x1.5, so that a debuff pays back the turn it costs within its length | 2026-10-12 (the user: raise the Etoile more, without making her a Diva): times 1.5 again. As the one support of the Meta party she won 50% / 88% / 67% at C30 / C34 / C38 and wins 68% / 98% / 82% with it; C36 (10%) and the last boss (0%) stay out of her reach, they ask for a heal she does not have, nor with Primevil. Beside a Diva the party gains at most 14 points (C38), nothing elsewhere: scratch/audit_2026-10-11/etoile_trial.py</t>
         </is>
       </c>
       <c r="K751" t="inlineStr">

</xml_diff>

<commit_message>
balance: the three TP fruits give a fifth more TP (Y012 - Y014)
the three TP fruits give a fifth more TP (Y012 - Y014); the build
writes, reads back and words the values of items
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/balance_changes.xlsx
+++ b/mod_project/data_tables/balance_changes.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1500"/>
+  <dimension ref="A1:L1503"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83510,6 +83510,165 @@
         </is>
       </c>
     </row>
+    <row r="1501">
+      <c r="A1501" t="inlineStr">
+        <is>
+          <t>Y012</t>
+        </is>
+      </c>
+      <c r="B1501" t="inlineStr">
+        <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="C1501" t="inlineStr">
+        <is>
+          <t>19 Magical Fruit</t>
+        </is>
+      </c>
+      <c r="D1501" t="inlineStr">
+        <is>
+          <t>effect 1 value (TP to one member)</t>
+        </is>
+      </c>
+      <c r="F1501" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1501" t="n">
+        <v>30</v>
+      </c>
+      <c r="H1501" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1501" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="J1501" t="inlineStr">
+        <is>
+          <t>The user, 2026-10-12 (row F01: no party without the Maid line wins from C30 on): a fifth more TP from the fruit, not a new cut of TP costs, which would move every party. Measured before it: the Meta party with a Bishop for its Diva wins 2% at C30 and C34 with 8 fruit of 50 TP, 50% with 24, 100% with TP at will; C36 and the last boss do not turn on TP. The Maid keeps her part; without her the fights are won with effort and a bag of fruit</t>
+        </is>
+      </c>
+      <c r="K1501" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1501" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" t="inlineStr">
+        <is>
+          <t>Y013</t>
+        </is>
+      </c>
+      <c r="B1502" t="inlineStr">
+        <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="C1502" t="inlineStr">
+        <is>
+          <t>20 Fairy Apple</t>
+        </is>
+      </c>
+      <c r="D1502" t="inlineStr">
+        <is>
+          <t>effect 1 value (TP to one member)</t>
+        </is>
+      </c>
+      <c r="F1502" t="n">
+        <v>50</v>
+      </c>
+      <c r="G1502" t="n">
+        <v>60</v>
+      </c>
+      <c r="H1502" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1502" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="J1502" t="inlineStr">
+        <is>
+          <t>The user, 2026-10-12 (row F01: no party without the Maid line wins from C30 on): a fifth more TP from the fruit, not a new cut of TP costs, which would move every party. Measured before it: the Meta party with a Bishop for its Diva wins 2% at C30 and C34 with 8 fruit of 50 TP, 50% with 24, 100% with TP at will; C36 and the last boss do not turn on TP. The Maid keeps her part; without her the fights are won with effort and a bag of fruit</t>
+        </is>
+      </c>
+      <c r="K1502" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1502" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" t="inlineStr">
+        <is>
+          <t>Y014</t>
+        </is>
+      </c>
+      <c r="B1503" t="inlineStr">
+        <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="C1503" t="inlineStr">
+        <is>
+          <t>21 Golden Apple</t>
+        </is>
+      </c>
+      <c r="D1503" t="inlineStr">
+        <is>
+          <t>effect 1 value (TP to one member)</t>
+        </is>
+      </c>
+      <c r="F1503" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1503" t="n">
+        <v>120</v>
+      </c>
+      <c r="H1503" t="inlineStr">
+        <is>
+          <t>L19</t>
+        </is>
+      </c>
+      <c r="I1503" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="J1503" t="inlineStr">
+        <is>
+          <t>The user, 2026-10-12 (row F01: no party without the Maid line wins from C30 on): a fifth more TP from the fruit, not a new cut of TP costs, which would move every party. Measured before it: the Meta party with a Bishop for its Diva wins 2% at C30 and C34 with 8 fruit of 50 TP, 50% with 24, 100% with TP at will; C36 and the last boss do not turn on TP. The Maid keeps her part; without her the fights are won with effort and a bag of fruit</t>
+        </is>
+      </c>
+      <c r="K1503" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L1503" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>